<commit_message>
Inseln nach Aufgabenfeldern, Themen für alle Fächer
- Graph: Fächer als farbige Inseln je Aufgabenfeld (data/aufgabenfelder.csv), Themen in der Mitte, Linien nur bei Auswahl
- Themen in data/themen.csv: 20 Themen, 138 Verknüpfungen über alle 17 Fächer (Vorschlag, Stichworte aus Kap. 6 mit Seite)
- faecher.csv mit Aufgabenfeld; Themenliste aus kerncurricula.py entfernt
- Excel: Anknüpfungspunkte aus themen.csv

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/Kerncurricula_Hessen_Sek1.xlsx
+++ b/output/Kerncurricula_Hessen_Sek1.xlsx
@@ -22,7 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Schwerpunkte'!$A$1:$H$499</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Kompetenzbereiche'!$A$1:$E$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Querbezüge belegt'!$A$1:$D$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Anknüpfungspunkte'!$A$1:$F$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Anknüpfungspunkte'!$A$1:$F$139</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'BNE Belege'!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'SDG-Vorschläge'!$A$1:$F$65</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Hinweise und Lücken'!$A$1:$B$15</definedName>
@@ -93,12 +93,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DBF5ED"/>
+        <fgColor rgb="00E4F7EA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D7F3F7"/>
+        <fgColor rgb="00E2F7F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D8F4EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAEFE4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7EADE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCF4EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4ECE2"/>
       </patternFill>
     </fill>
     <fill>
@@ -108,72 +133,47 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F7F1E7"/>
+        <fgColor rgb="00DFF8EF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FBE8EA"/>
+        <fgColor rgb="00EDF3FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8ECE2"/>
+        <fgColor rgb="00EFE8FC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4F6E1"/>
+        <fgColor rgb="00F5EFFD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE7E0"/>
+        <fgColor rgb="00EAE3F8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0ECFF"/>
+        <fgColor rgb="00FCE7ED"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEFE7"/>
+        <fgColor rgb="00FDEEF2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4F7"/>
+        <fgColor rgb="00F8E2E8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F3E8FD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EBF9DE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EDF3F7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F7F3ED"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F3EFFA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E7E8FF"/>
+        <fgColor rgb="00E9FBF5"/>
       </patternFill>
     </fill>
   </fills>
@@ -26211,7 +26211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -26245,7 +26245,7 @@
       </c>
       <c r="E1" s="25" t="inlineStr">
         <is>
-          <t>Stufe laut KC</t>
+          <t>Stufe laut KC bzw. Seite (Kap. 6)</t>
         </is>
       </c>
       <c r="F1" s="25" t="inlineStr">
@@ -26449,27 +26449,27 @@
     <row r="8">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>Klima und Wetter</t>
-        </is>
-      </c>
-      <c r="B8" s="29" t="inlineStr">
-        <is>
-          <t>Physik</t>
+          <t>Energie</t>
+        </is>
+      </c>
+      <c r="B8" s="33" t="inlineStr">
+        <is>
+          <t>Arbeitslehre</t>
         </is>
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t>Wettererscheinungen und Klima</t>
+          <t>Technische Systeme und Prozesse</t>
         </is>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>Einfluss des Menschen auf das Klima und Folgen</t>
+          <t>Folgen von Techniknutzung im Zielkonflikt Technik, Ökonomie, Ökologie</t>
         </is>
       </c>
       <c r="E8" s="26" t="inlineStr">
         <is>
-          <t>zusätzlich bis Ende 9/10</t>
+          <t>S. 20</t>
         </is>
       </c>
       <c r="F8" s="26" t="inlineStr">
@@ -26481,27 +26481,27 @@
     <row r="9">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>Klima und Wetter</t>
-        </is>
-      </c>
-      <c r="B9" s="30" t="inlineStr">
-        <is>
-          <t>Erdkunde</t>
+          <t>Energie</t>
+        </is>
+      </c>
+      <c r="B9" s="32" t="inlineStr">
+        <is>
+          <t>Geschichte</t>
         </is>
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>Natur/Umwelt</t>
+          <t>Epochenbezug Neuzeit</t>
         </is>
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>Geofaktor Klima</t>
+          <t>Industrielle Revolutionen</t>
         </is>
       </c>
       <c r="E9" s="26" t="inlineStr">
         <is>
-          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
+          <t>S. 22</t>
         </is>
       </c>
       <c r="F9" s="26" t="inlineStr">
@@ -26516,19 +26516,19 @@
           <t>Klima und Wetter</t>
         </is>
       </c>
-      <c r="B10" s="27" t="inlineStr">
-        <is>
-          <t>Biologie</t>
+      <c r="B10" s="29" t="inlineStr">
+        <is>
+          <t>Physik</t>
         </is>
       </c>
       <c r="C10" s="26" t="inlineStr">
         <is>
-          <t>Stoffwechsel und Regelmechanismen</t>
+          <t>Wettererscheinungen und Klima</t>
         </is>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>Stoffkreisläufe (z. B. Kohlenstoffkreislauf)</t>
+          <t>Einfluss des Menschen auf das Klima und Folgen</t>
         </is>
       </c>
       <c r="E10" s="26" t="inlineStr">
@@ -26548,19 +26548,19 @@
           <t>Klima und Wetter</t>
         </is>
       </c>
-      <c r="B11" s="31" t="inlineStr">
-        <is>
-          <t>Politik und Wirtschaft</t>
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>Erdkunde</t>
         </is>
       </c>
       <c r="C11" s="26" t="inlineStr">
         <is>
-          <t>Gesellschaft und Natur</t>
+          <t>Natur/Umwelt</t>
         </is>
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>Nachhaltige Entwicklung, Generationenverantwortung</t>
+          <t>Geofaktor Klima</t>
         </is>
       </c>
       <c r="E11" s="26" t="inlineStr">
@@ -26577,22 +26577,22 @@
     <row r="12">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>Wasser, Luft, Boden, Stoffkreisläufe</t>
-        </is>
-      </c>
-      <c r="B12" s="28" t="inlineStr">
-        <is>
-          <t>Chemie</t>
+          <t>Klima und Wetter</t>
+        </is>
+      </c>
+      <c r="B12" s="27" t="inlineStr">
+        <is>
+          <t>Biologie</t>
         </is>
       </c>
       <c r="C12" s="26" t="inlineStr">
         <is>
-          <t>Schatzkiste der Natur – Chemie in Alltag und Technik</t>
+          <t>Stoffwechsel und Regelmechanismen</t>
         </is>
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
-          <t>Luft, Wasser, Boden; Stoffkreisläufe in Natur und Technik</t>
+          <t>Stoffkreisläufe (z. B. Kohlenstoffkreislauf)</t>
         </is>
       </c>
       <c r="E12" s="26" t="inlineStr">
@@ -26609,27 +26609,27 @@
     <row r="13">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>Wasser, Luft, Boden, Stoffkreisläufe</t>
-        </is>
-      </c>
-      <c r="B13" s="28" t="inlineStr">
-        <is>
-          <t>Chemie</t>
+          <t>Klima und Wetter</t>
+        </is>
+      </c>
+      <c r="B13" s="31" t="inlineStr">
+        <is>
+          <t>Politik und Wirtschaft</t>
         </is>
       </c>
       <c r="C13" s="26" t="inlineStr">
         <is>
-          <t>Welt der Stoffe – Identifikation und Ordnung von Stoffen</t>
+          <t>Gesellschaft und Natur</t>
         </is>
       </c>
       <c r="D13" s="26" t="inlineStr">
         <is>
-          <t>Alltags-, Lebens- und Umweltrelevanz von Luft und Wasser</t>
+          <t>Nachhaltige Entwicklung, Generationenverantwortung</t>
         </is>
       </c>
       <c r="E13" s="26" t="inlineStr">
         <is>
-          <t>zusätzlich bis Ende 9/10</t>
+          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
         </is>
       </c>
       <c r="F13" s="26" t="inlineStr">
@@ -26641,27 +26641,27 @@
     <row r="14">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>Wasser, Luft, Boden, Stoffkreisläufe</t>
-        </is>
-      </c>
-      <c r="B14" s="29" t="inlineStr">
-        <is>
-          <t>Physik</t>
+          <t>Klima und Wetter</t>
+        </is>
+      </c>
+      <c r="B14" s="35" t="inlineStr">
+        <is>
+          <t>Mathematik</t>
         </is>
       </c>
       <c r="C14" s="26" t="inlineStr">
         <is>
-          <t>Wettererscheinungen und Klima</t>
+          <t>Statistische Erhebungen und ihre Auswertung</t>
         </is>
       </c>
       <c r="D14" s="26" t="inlineStr">
         <is>
-          <t>Anomalie des Wassers</t>
+          <t>Erhebung und Auswertung von Daten</t>
         </is>
       </c>
       <c r="E14" s="26" t="inlineStr">
         <is>
-          <t>nach ca. Hälfte des Stundenkontingents</t>
+          <t>S. 21</t>
         </is>
       </c>
       <c r="F14" s="26" t="inlineStr">
@@ -26673,27 +26673,27 @@
     <row r="15">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>Wasser, Luft, Boden, Stoffkreisläufe</t>
-        </is>
-      </c>
-      <c r="B15" s="27" t="inlineStr">
-        <is>
-          <t>Biologie</t>
+          <t>Klima und Wetter</t>
+        </is>
+      </c>
+      <c r="B15" s="40" t="inlineStr">
+        <is>
+          <t>Ethik</t>
         </is>
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
-          <t>Stoffwechsel und Regelmechanismen</t>
+          <t>Mensch, Natur und Technik</t>
         </is>
       </c>
       <c r="D15" s="26" t="inlineStr">
         <is>
-          <t>Stoffkreisläufe (z. B. Kohlenstoffkreislauf)</t>
+          <t>Verantwortung im Umgang mit der Natur</t>
         </is>
       </c>
       <c r="E15" s="26" t="inlineStr">
         <is>
-          <t>zusätzlich bis Ende 9/10</t>
+          <t>S. 19</t>
         </is>
       </c>
       <c r="F15" s="26" t="inlineStr">
@@ -26708,24 +26708,24 @@
           <t>Wasser, Luft, Boden, Stoffkreisläufe</t>
         </is>
       </c>
-      <c r="B16" s="30" t="inlineStr">
-        <is>
-          <t>Erdkunde</t>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>Chemie</t>
         </is>
       </c>
       <c r="C16" s="26" t="inlineStr">
         <is>
-          <t>Natur/Umwelt</t>
+          <t>Schatzkiste der Natur – Chemie in Alltag und Technik</t>
         </is>
       </c>
       <c r="D16" s="26" t="inlineStr">
         <is>
-          <t>Geofaktor Boden</t>
+          <t>Luft, Wasser, Boden; Stoffkreisläufe in Natur und Technik</t>
         </is>
       </c>
       <c r="E16" s="26" t="inlineStr">
         <is>
-          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
+          <t>zusätzlich bis Ende 9/10</t>
         </is>
       </c>
       <c r="F16" s="26" t="inlineStr">
@@ -26737,22 +26737,22 @@
     <row r="17">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>Ökosysteme und Eingriffe des Menschen</t>
-        </is>
-      </c>
-      <c r="B17" s="27" t="inlineStr">
-        <is>
-          <t>Biologie</t>
+          <t>Wasser, Luft, Boden, Stoffkreisläufe</t>
+        </is>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>Chemie</t>
         </is>
       </c>
       <c r="C17" s="26" t="inlineStr">
         <is>
-          <t>Wechselwirkungen in Ökosystemen</t>
+          <t>Welt der Stoffe – Identifikation und Ordnung von Stoffen</t>
         </is>
       </c>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t>Gefährdung von Ökosystemen durch Eingriffe des Menschen</t>
+          <t>Alltags-, Lebens- und Umweltrelevanz von Luft und Wasser</t>
         </is>
       </c>
       <c r="E17" s="26" t="inlineStr">
@@ -26769,27 +26769,27 @@
     <row r="18">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>Ökosysteme und Eingriffe des Menschen</t>
-        </is>
-      </c>
-      <c r="B18" s="27" t="inlineStr">
-        <is>
-          <t>Biologie</t>
+          <t>Wasser, Luft, Boden, Stoffkreisläufe</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="inlineStr">
+        <is>
+          <t>Physik</t>
         </is>
       </c>
       <c r="C18" s="26" t="inlineStr">
         <is>
-          <t>Stoffwechsel und Regelmechanismen</t>
+          <t>Wettererscheinungen und Klima</t>
         </is>
       </c>
       <c r="D18" s="26" t="inlineStr">
         <is>
-          <t>Auswirkungen von Eingriffen des Menschen in ökologische Beziehungen</t>
+          <t>Anomalie des Wassers</t>
         </is>
       </c>
       <c r="E18" s="26" t="inlineStr">
         <is>
-          <t>bis Ende 5/6</t>
+          <t>nach ca. Hälfte des Stundenkontingents</t>
         </is>
       </c>
       <c r="F18" s="26" t="inlineStr">
@@ -26801,27 +26801,27 @@
     <row r="19">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>Ökosysteme und Eingriffe des Menschen</t>
-        </is>
-      </c>
-      <c r="B19" s="30" t="inlineStr">
-        <is>
-          <t>Erdkunde</t>
+          <t>Wasser, Luft, Boden, Stoffkreisläufe</t>
+        </is>
+      </c>
+      <c r="B19" s="27" t="inlineStr">
+        <is>
+          <t>Biologie</t>
         </is>
       </c>
       <c r="C19" s="26" t="inlineStr">
         <is>
-          <t>Umwelt-Gesellschaft-Beziehungen und globale Probleme</t>
+          <t>Stoffwechsel und Regelmechanismen</t>
         </is>
       </c>
       <c r="D19" s="26" t="inlineStr">
         <is>
-          <t>Umweltgefährdung</t>
+          <t>Stoffkreisläufe (z. B. Kohlenstoffkreislauf)</t>
         </is>
       </c>
       <c r="E19" s="26" t="inlineStr">
         <is>
-          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
+          <t>zusätzlich bis Ende 9/10</t>
         </is>
       </c>
       <c r="F19" s="26" t="inlineStr">
@@ -26833,7 +26833,7 @@
     <row r="20">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>Ökosysteme und Eingriffe des Menschen</t>
+          <t>Wasser, Luft, Boden, Stoffkreisläufe</t>
         </is>
       </c>
       <c r="B20" s="30" t="inlineStr">
@@ -26843,12 +26843,12 @@
       </c>
       <c r="C20" s="26" t="inlineStr">
         <is>
-          <t>Geographie auf regionaler Ebene</t>
+          <t>Natur/Umwelt</t>
         </is>
       </c>
       <c r="D20" s="26" t="inlineStr">
         <is>
-          <t>Folgen von Eingriffen des Menschen in die Umwelt</t>
+          <t>Geofaktor Boden</t>
         </is>
       </c>
       <c r="E20" s="26" t="inlineStr">
@@ -26868,24 +26868,24 @@
           <t>Ökosysteme und Eingriffe des Menschen</t>
         </is>
       </c>
-      <c r="B21" s="29" t="inlineStr">
-        <is>
-          <t>Physik</t>
+      <c r="B21" s="27" t="inlineStr">
+        <is>
+          <t>Biologie</t>
         </is>
       </c>
       <c r="C21" s="26" t="inlineStr">
         <is>
-          <t>Physik in der Verantwortung</t>
+          <t>Wechselwirkungen in Ökosystemen</t>
         </is>
       </c>
       <c r="D21" s="26" t="inlineStr">
         <is>
-          <t>Verantwortung gegenüber der Umwelt</t>
+          <t>Gefährdung von Ökosystemen durch Eingriffe des Menschen</t>
         </is>
       </c>
       <c r="E21" s="26" t="inlineStr">
         <is>
-          <t>nach ca. Hälfte des Stundenkontingents</t>
+          <t>zusätzlich bis Ende 9/10</t>
         </is>
       </c>
       <c r="F21" s="26" t="inlineStr">
@@ -26900,24 +26900,24 @@
           <t>Ökosysteme und Eingriffe des Menschen</t>
         </is>
       </c>
-      <c r="B22" s="31" t="inlineStr">
-        <is>
-          <t>Politik und Wirtschaft</t>
+      <c r="B22" s="27" t="inlineStr">
+        <is>
+          <t>Biologie</t>
         </is>
       </c>
       <c r="C22" s="26" t="inlineStr">
         <is>
-          <t>Gesellschaft und Natur</t>
+          <t>Stoffwechsel und Regelmechanismen</t>
         </is>
       </c>
       <c r="D22" s="26" t="inlineStr">
         <is>
-          <t>Nachhaltige Entwicklung</t>
+          <t>Auswirkungen von Eingriffen des Menschen in ökologische Beziehungen</t>
         </is>
       </c>
       <c r="E22" s="26" t="inlineStr">
         <is>
-          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
+          <t>bis Ende 5/6</t>
         </is>
       </c>
       <c r="F22" s="26" t="inlineStr">
@@ -26929,27 +26929,27 @@
     <row r="23">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>Sinne und Wahrnehmung</t>
-        </is>
-      </c>
-      <c r="B23" s="27" t="inlineStr">
-        <is>
-          <t>Biologie</t>
+          <t>Ökosysteme und Eingriffe des Menschen</t>
+        </is>
+      </c>
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t>Erdkunde</t>
         </is>
       </c>
       <c r="C23" s="26" t="inlineStr">
         <is>
-          <t>Informationsfluss im Organismus und zwischen Organismen</t>
+          <t>Umwelt-Gesellschaft-Beziehungen und globale Probleme</t>
         </is>
       </c>
       <c r="D23" s="26" t="inlineStr">
         <is>
-          <t>Sinnesorgane (Auge oder Ohr), Gesundheitsschutz</t>
+          <t>Umweltgefährdung</t>
         </is>
       </c>
       <c r="E23" s="26" t="inlineStr">
         <is>
-          <t>zusätzlich bis Ende 9/10</t>
+          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
         </is>
       </c>
       <c r="F23" s="26" t="inlineStr">
@@ -26961,27 +26961,27 @@
     <row r="24">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>Sinne und Wahrnehmung</t>
-        </is>
-      </c>
-      <c r="B24" s="29" t="inlineStr">
-        <is>
-          <t>Physik</t>
+          <t>Ökosysteme und Eingriffe des Menschen</t>
+        </is>
+      </c>
+      <c r="B24" s="30" t="inlineStr">
+        <is>
+          <t>Erdkunde</t>
         </is>
       </c>
       <c r="C24" s="26" t="inlineStr">
         <is>
-          <t>Erweiterung der Sinne</t>
+          <t>Geographie auf regionaler Ebene</t>
         </is>
       </c>
       <c r="D24" s="26" t="inlineStr">
         <is>
-          <t>Wahrnehmung der Umgebung mit den Sinnesorganen</t>
+          <t>Folgen von Eingriffen des Menschen in die Umwelt</t>
         </is>
       </c>
       <c r="E24" s="26" t="inlineStr">
         <is>
-          <t>nach ca. Hälfte des Stundenkontingents</t>
+          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
         </is>
       </c>
       <c r="F24" s="26" t="inlineStr">
@@ -26993,7 +26993,7 @@
     <row r="25">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>Sinne und Wahrnehmung</t>
+          <t>Ökosysteme und Eingriffe des Menschen</t>
         </is>
       </c>
       <c r="B25" s="29" t="inlineStr">
@@ -27003,17 +27003,17 @@
       </c>
       <c r="C25" s="26" t="inlineStr">
         <is>
-          <t>Erweiterung der Sinne</t>
+          <t>Physik in der Verantwortung</t>
         </is>
       </c>
       <c r="D25" s="26" t="inlineStr">
         <is>
-          <t>Auswirkungen von Lärm auf die Gesundheit</t>
+          <t>Verantwortung gegenüber der Umwelt</t>
         </is>
       </c>
       <c r="E25" s="26" t="inlineStr">
         <is>
-          <t>zusätzlich bis Ende 9/10</t>
+          <t>nach ca. Hälfte des Stundenkontingents</t>
         </is>
       </c>
       <c r="F25" s="26" t="inlineStr">
@@ -27025,27 +27025,27 @@
     <row r="26">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>Mobilität und Verkehr</t>
-        </is>
-      </c>
-      <c r="B26" s="29" t="inlineStr">
-        <is>
-          <t>Physik</t>
+          <t>Ökosysteme und Eingriffe des Menschen</t>
+        </is>
+      </c>
+      <c r="B26" s="31" t="inlineStr">
+        <is>
+          <t>Politik und Wirtschaft</t>
         </is>
       </c>
       <c r="C26" s="26" t="inlineStr">
         <is>
-          <t>Fortbewegung und Mobilität</t>
+          <t>Gesellschaft und Natur</t>
         </is>
       </c>
       <c r="D26" s="26" t="inlineStr">
         <is>
-          <t>Weg, Zeit, Geschwindigkeit; Trägheit und Risiken im Straßenverkehr</t>
+          <t>Nachhaltige Entwicklung</t>
         </is>
       </c>
       <c r="E26" s="26" t="inlineStr">
         <is>
-          <t>nach ca. Hälfte des Stundenkontingents / zusätzlich bis Ende 9/10</t>
+          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
         </is>
       </c>
       <c r="F26" s="26" t="inlineStr">
@@ -27057,27 +27057,27 @@
     <row r="27">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>Mobilität und Verkehr</t>
-        </is>
-      </c>
-      <c r="B27" s="28" t="inlineStr">
-        <is>
-          <t>Chemie</t>
+          <t>Ökosysteme und Eingriffe des Menschen</t>
+        </is>
+      </c>
+      <c r="B27" s="40" t="inlineStr">
+        <is>
+          <t>Ethik</t>
         </is>
       </c>
       <c r="C27" s="26" t="inlineStr">
         <is>
-          <t>Magie des Kohlenstoffs – Organische Verbindungen</t>
+          <t>Mensch, Natur und Technik</t>
         </is>
       </c>
       <c r="D27" s="26" t="inlineStr">
         <is>
-          <t>Kohlenwasserstoffverbindungen u. a. aus Energiewirtschaft und Verkehr (Kap. 6, S. 27)</t>
+          <t>Verfügungsanspruch des Menschen über die Natur</t>
         </is>
       </c>
       <c r="E27" s="26" t="inlineStr">
         <is>
-          <t>Inhaltsfeldbeschreibung</t>
+          <t>S. 19</t>
         </is>
       </c>
       <c r="F27" s="26" t="inlineStr">
@@ -27089,27 +27089,27 @@
     <row r="28">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>Mobilität und Verkehr</t>
-        </is>
-      </c>
-      <c r="B28" s="31" t="inlineStr">
-        <is>
-          <t>Politik und Wirtschaft</t>
+          <t>Ökosysteme und Eingriffe des Menschen</t>
+        </is>
+      </c>
+      <c r="B28" s="41" t="inlineStr">
+        <is>
+          <t>Evangelische Religion</t>
         </is>
       </c>
       <c r="C28" s="26" t="inlineStr">
         <is>
-          <t>Wirtschaft</t>
+          <t>Mensch und Welt</t>
         </is>
       </c>
       <c r="D28" s="26" t="inlineStr">
         <is>
-          <t>Analysekompetenz: externe Effekte bei verkehrspolitischen Fragen (Kap. 4, S. 16)</t>
+          <t>Die Welt als Schöpfung</t>
         </is>
       </c>
       <c r="E28" s="26" t="inlineStr">
         <is>
-          <t>Kompetenzbeschreibung</t>
+          <t>S. 19</t>
         </is>
       </c>
       <c r="F28" s="26" t="inlineStr">
@@ -27121,27 +27121,27 @@
     <row r="29">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>Mobilität und Verkehr</t>
-        </is>
-      </c>
-      <c r="B29" s="30" t="inlineStr">
-        <is>
-          <t>Erdkunde</t>
+          <t>Ökosysteme und Eingriffe des Menschen</t>
+        </is>
+      </c>
+      <c r="B29" s="42" t="inlineStr">
+        <is>
+          <t>Katholische Religion</t>
         </is>
       </c>
       <c r="C29" s="26" t="inlineStr">
         <is>
-          <t>Mensch/Gesellschaft</t>
+          <t>Mensch und Welt</t>
         </is>
       </c>
       <c r="D29" s="26" t="inlineStr">
         <is>
-          <t>Humangeographisches Teilsystem Verkehr (Kap. 5, S. 19)</t>
+          <t>Schöpfungsauftrag, die Welt zu gestalten und zu bewahren</t>
         </is>
       </c>
       <c r="E29" s="26" t="inlineStr">
         <is>
-          <t>Konzeptbeschreibung</t>
+          <t>S. 17</t>
         </is>
       </c>
       <c r="F29" s="26" t="inlineStr">
@@ -27153,27 +27153,27 @@
     <row r="30">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>Ernährung, Gesundheit, Konsum</t>
-        </is>
-      </c>
-      <c r="B30" s="27" t="inlineStr">
-        <is>
-          <t>Biologie</t>
+          <t>Ökosysteme und Eingriffe des Menschen</t>
+        </is>
+      </c>
+      <c r="B30" s="37" t="inlineStr">
+        <is>
+          <t>Kunst</t>
         </is>
       </c>
       <c r="C30" s="26" t="inlineStr">
         <is>
-          <t>Stoffwechsel und Regelmechanismen</t>
+          <t>Wahrnehmung der Umwelt</t>
         </is>
       </c>
       <c r="D30" s="26" t="inlineStr">
         <is>
-          <t>Aspekte zur ausgewogenen Ernährung</t>
+          <t>Haltung zur Umwelt</t>
         </is>
       </c>
       <c r="E30" s="26" t="inlineStr">
         <is>
-          <t>bis Ende 5/6</t>
+          <t>S. 21</t>
         </is>
       </c>
       <c r="F30" s="26" t="inlineStr">
@@ -27185,7 +27185,7 @@
     <row r="31">
       <c r="A31" s="26" t="inlineStr">
         <is>
-          <t>Ernährung, Gesundheit, Konsum</t>
+          <t>Sinne und Wahrnehmung</t>
         </is>
       </c>
       <c r="B31" s="27" t="inlineStr">
@@ -27195,17 +27195,17 @@
       </c>
       <c r="C31" s="26" t="inlineStr">
         <is>
-          <t>Stoffwechsel und Regelmechanismen</t>
+          <t>Informationsfluss im Organismus und zwischen Organismen</t>
         </is>
       </c>
       <c r="D31" s="26" t="inlineStr">
         <is>
-          <t>Bewertung des Konsumverhaltens im Hinblick auf Haltung und Nutzung von Lebewesen</t>
+          <t>Sinnesorgane (Auge oder Ohr), Gesundheitsschutz</t>
         </is>
       </c>
       <c r="E31" s="26" t="inlineStr">
         <is>
-          <t>bis Ende 5/6</t>
+          <t>zusätzlich bis Ende 9/10</t>
         </is>
       </c>
       <c r="F31" s="26" t="inlineStr">
@@ -27217,27 +27217,27 @@
     <row r="32">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>Ernährung, Gesundheit, Konsum</t>
-        </is>
-      </c>
-      <c r="B32" s="28" t="inlineStr">
-        <is>
-          <t>Chemie</t>
+          <t>Sinne und Wahrnehmung</t>
+        </is>
+      </c>
+      <c r="B32" s="29" t="inlineStr">
+        <is>
+          <t>Physik</t>
         </is>
       </c>
       <c r="C32" s="26" t="inlineStr">
         <is>
-          <t>Magie des Kohlenstoffs – Organische Verbindungen</t>
+          <t>Erweiterung der Sinne</t>
         </is>
       </c>
       <c r="D32" s="26" t="inlineStr">
         <is>
-          <t>Organische Stoffe aus Ernährung und Hygiene (Kap. 6, S. 27)</t>
+          <t>Wahrnehmung der Umgebung mit den Sinnesorganen</t>
         </is>
       </c>
       <c r="E32" s="26" t="inlineStr">
         <is>
-          <t>Inhaltsfeldbeschreibung</t>
+          <t>nach ca. Hälfte des Stundenkontingents</t>
         </is>
       </c>
       <c r="F32" s="26" t="inlineStr">
@@ -27249,27 +27249,27 @@
     <row r="33">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>Ernährung, Gesundheit, Konsum</t>
-        </is>
-      </c>
-      <c r="B33" s="31" t="inlineStr">
-        <is>
-          <t>Politik und Wirtschaft</t>
+          <t>Sinne und Wahrnehmung</t>
+        </is>
+      </c>
+      <c r="B33" s="29" t="inlineStr">
+        <is>
+          <t>Physik</t>
         </is>
       </c>
       <c r="C33" s="26" t="inlineStr">
         <is>
-          <t>Wirtschaft</t>
+          <t>Erweiterung der Sinne</t>
         </is>
       </c>
       <c r="D33" s="26" t="inlineStr">
         <is>
-          <t>Rolle als Verbraucherinnen und Verbraucher</t>
+          <t>Auswirkungen von Lärm auf die Gesundheit</t>
         </is>
       </c>
       <c r="E33" s="26" t="inlineStr">
         <is>
-          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
+          <t>zusätzlich bis Ende 9/10</t>
         </is>
       </c>
       <c r="F33" s="26" t="inlineStr">
@@ -27281,27 +27281,27 @@
     <row r="34">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>Teilchen und Aufbau der Materie</t>
-        </is>
-      </c>
-      <c r="B34" s="28" t="inlineStr">
-        <is>
-          <t>Chemie</t>
+          <t>Sinne und Wahrnehmung</t>
+        </is>
+      </c>
+      <c r="B34" s="38" t="inlineStr">
+        <is>
+          <t>Musik</t>
         </is>
       </c>
       <c r="C34" s="26" t="inlineStr">
         <is>
-          <t>Blick hinter die Kulissen – Aufbau von Stoffen und chemische Bindung</t>
+          <t>Hörkultur</t>
         </is>
       </c>
       <c r="D34" s="26" t="inlineStr">
         <is>
-          <t>Teilchenmodell zur Deutung von Phänomenen</t>
+          <t>Spektrum an Hörleistungen</t>
         </is>
       </c>
       <c r="E34" s="26" t="inlineStr">
         <is>
-          <t>1. Lernjahr</t>
+          <t>S. 17</t>
         </is>
       </c>
       <c r="F34" s="26" t="inlineStr">
@@ -27313,27 +27313,27 @@
     <row r="35">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>Teilchen und Aufbau der Materie</t>
-        </is>
-      </c>
-      <c r="B35" s="29" t="inlineStr">
-        <is>
-          <t>Physik</t>
+          <t>Sinne und Wahrnehmung</t>
+        </is>
+      </c>
+      <c r="B35" s="38" t="inlineStr">
+        <is>
+          <t>Musik</t>
         </is>
       </c>
       <c r="C35" s="26" t="inlineStr">
         <is>
-          <t>Wettererscheinungen und Klima</t>
+          <t>Klang</t>
         </is>
       </c>
       <c r="D35" s="26" t="inlineStr">
         <is>
-          <t>Modelle des Aufbaus der Materie; Aggregatzustände</t>
+          <t>Klang</t>
         </is>
       </c>
       <c r="E35" s="26" t="inlineStr">
         <is>
-          <t>nach ca. Hälfte des Stundenkontingents</t>
+          <t>S. 17</t>
         </is>
       </c>
       <c r="F35" s="26" t="inlineStr">
@@ -27345,27 +27345,27 @@
     <row r="36">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>Teilchen und Aufbau der Materie</t>
-        </is>
-      </c>
-      <c r="B36" s="28" t="inlineStr">
-        <is>
-          <t>Chemie</t>
+          <t>Sinne und Wahrnehmung</t>
+        </is>
+      </c>
+      <c r="B36" s="37" t="inlineStr">
+        <is>
+          <t>Kunst</t>
         </is>
       </c>
       <c r="C36" s="26" t="inlineStr">
         <is>
-          <t>Verwandlungen – Chemische Reaktion</t>
+          <t>Wahrnehmung der Umwelt</t>
         </is>
       </c>
       <c r="D36" s="26" t="inlineStr">
         <is>
-          <t>Aggregatzustand und Aggregatzustandsänderungen</t>
+          <t>Wahrnehmung der Umwelt</t>
         </is>
       </c>
       <c r="E36" s="26" t="inlineStr">
         <is>
-          <t>1. Lernjahr</t>
+          <t>S. 21</t>
         </is>
       </c>
       <c r="F36" s="26" t="inlineStr">
@@ -27377,27 +27377,27 @@
     <row r="37">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>Teilchen und Aufbau der Materie</t>
-        </is>
-      </c>
-      <c r="B37" s="29" t="inlineStr">
-        <is>
-          <t>Physik</t>
+          <t>Sinne und Wahrnehmung</t>
+        </is>
+      </c>
+      <c r="B37" s="39" t="inlineStr">
+        <is>
+          <t>Sport</t>
         </is>
       </c>
       <c r="C37" s="26" t="inlineStr">
         <is>
-          <t>Physik in der Verantwortung</t>
+          <t>Bewegung gymnastisch, rhythmisch und tänzerisch gestalten</t>
         </is>
       </c>
       <c r="D37" s="26" t="inlineStr">
         <is>
-          <t>Radioaktive Zerfallsprozesse</t>
+          <t>Leitidee Körperwahrnehmung</t>
         </is>
       </c>
       <c r="E37" s="26" t="inlineStr">
         <is>
-          <t>zusätzlich bis Ende 9/10</t>
+          <t>S. 21</t>
         </is>
       </c>
       <c r="F37" s="26" t="inlineStr">
@@ -27409,27 +27409,27 @@
     <row r="38">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>Ressourcen und Recycling</t>
-        </is>
-      </c>
-      <c r="B38" s="28" t="inlineStr">
-        <is>
-          <t>Chemie</t>
+          <t>Mobilität und Verkehr</t>
+        </is>
+      </c>
+      <c r="B38" s="29" t="inlineStr">
+        <is>
+          <t>Physik</t>
         </is>
       </c>
       <c r="C38" s="26" t="inlineStr">
         <is>
-          <t>Magie des Kohlenstoffs – Organische Verbindungen</t>
+          <t>Fortbewegung und Mobilität</t>
         </is>
       </c>
       <c r="D38" s="26" t="inlineStr">
         <is>
-          <t>Gewinnung, Verwendung und Recycling organischer Stoffe</t>
+          <t>Weg, Zeit, Geschwindigkeit; Trägheit und Risiken im Straßenverkehr</t>
         </is>
       </c>
       <c r="E38" s="26" t="inlineStr">
         <is>
-          <t>zusätzlich bis Ende 9/10</t>
+          <t>nach ca. Hälfte des Stundenkontingents / zusätzlich bis Ende 9/10</t>
         </is>
       </c>
       <c r="F38" s="26" t="inlineStr">
@@ -27441,27 +27441,27 @@
     <row r="39">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>Ressourcen und Recycling</t>
-        </is>
-      </c>
-      <c r="B39" s="29" t="inlineStr">
-        <is>
-          <t>Physik</t>
+          <t>Mobilität und Verkehr</t>
+        </is>
+      </c>
+      <c r="B39" s="28" t="inlineStr">
+        <is>
+          <t>Chemie</t>
         </is>
       </c>
       <c r="C39" s="26" t="inlineStr">
         <is>
-          <t>Zukunftssichere Energieversorgung</t>
+          <t>Magie des Kohlenstoffs – Organische Verbindungen</t>
         </is>
       </c>
       <c r="D39" s="26" t="inlineStr">
         <is>
-          <t>Regenerative und erschöpfbare Energien</t>
+          <t>Kohlenwasserstoffverbindungen u. a. aus Energiewirtschaft und Verkehr (Kap. 6, S. 27)</t>
         </is>
       </c>
       <c r="E39" s="26" t="inlineStr">
         <is>
-          <t>nach ca. Hälfte des Stundenkontingents</t>
+          <t>Inhaltsfeldbeschreibung</t>
         </is>
       </c>
       <c r="F39" s="26" t="inlineStr">
@@ -27473,27 +27473,27 @@
     <row r="40">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>Ressourcen und Recycling</t>
-        </is>
-      </c>
-      <c r="B40" s="30" t="inlineStr">
-        <is>
-          <t>Erdkunde</t>
+          <t>Mobilität und Verkehr</t>
+        </is>
+      </c>
+      <c r="B40" s="31" t="inlineStr">
+        <is>
+          <t>Politik und Wirtschaft</t>
         </is>
       </c>
       <c r="C40" s="26" t="inlineStr">
         <is>
-          <t>Umwelt-Gesellschaft-Beziehungen und globale Probleme</t>
+          <t>Wirtschaft</t>
         </is>
       </c>
       <c r="D40" s="26" t="inlineStr">
         <is>
-          <t>Ressourcensicherung</t>
+          <t>Analysekompetenz: externe Effekte bei verkehrspolitischen Fragen (Kap. 4, S. 16)</t>
         </is>
       </c>
       <c r="E40" s="26" t="inlineStr">
         <is>
-          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
+          <t>Kompetenzbeschreibung</t>
         </is>
       </c>
       <c r="F40" s="26" t="inlineStr">
@@ -27505,27 +27505,27 @@
     <row r="41">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>Ressourcen und Recycling</t>
-        </is>
-      </c>
-      <c r="B41" s="31" t="inlineStr">
-        <is>
-          <t>Politik und Wirtschaft</t>
+          <t>Mobilität und Verkehr</t>
+        </is>
+      </c>
+      <c r="B41" s="30" t="inlineStr">
+        <is>
+          <t>Erdkunde</t>
         </is>
       </c>
       <c r="C41" s="26" t="inlineStr">
         <is>
-          <t>Gesellschaft und Natur</t>
+          <t>Mensch/Gesellschaft</t>
         </is>
       </c>
       <c r="D41" s="26" t="inlineStr">
         <is>
-          <t>Spannungsfeld zwischen Ökonomie und Ökologie</t>
+          <t>Humangeographisches Teilsystem Verkehr (Kap. 5, S. 19)</t>
         </is>
       </c>
       <c r="E41" s="26" t="inlineStr">
         <is>
-          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
+          <t>Konzeptbeschreibung</t>
         </is>
       </c>
       <c r="F41" s="26" t="inlineStr">
@@ -27537,27 +27537,27 @@
     <row r="42">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>Migration und Globalisierung</t>
-        </is>
-      </c>
-      <c r="B42" s="30" t="inlineStr">
-        <is>
-          <t>Erdkunde</t>
+          <t>Mobilität und Verkehr</t>
+        </is>
+      </c>
+      <c r="B42" s="39" t="inlineStr">
+        <is>
+          <t>Sport</t>
         </is>
       </c>
       <c r="C42" s="26" t="inlineStr">
         <is>
-          <t>Mensch/Gesellschaft</t>
+          <t>Fahren, Rollen, Gleiten</t>
         </is>
       </c>
       <c r="D42" s="26" t="inlineStr">
         <is>
-          <t>Migration, Globalisierung, Metropolisierung</t>
+          <t>Leitidee „Wagnis“: Geschwindigkeit, labiles Gleichgewicht</t>
         </is>
       </c>
       <c r="E42" s="26" t="inlineStr">
         <is>
-          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
+          <t>S. 23</t>
         </is>
       </c>
       <c r="F42" s="26" t="inlineStr">
@@ -27569,27 +27569,27 @@
     <row r="43">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>Migration und Globalisierung</t>
-        </is>
-      </c>
-      <c r="B43" s="30" t="inlineStr">
-        <is>
-          <t>Erdkunde</t>
+          <t>Ernährung, Gesundheit, Konsum</t>
+        </is>
+      </c>
+      <c r="B43" s="27" t="inlineStr">
+        <is>
+          <t>Biologie</t>
         </is>
       </c>
       <c r="C43" s="26" t="inlineStr">
         <is>
-          <t>Umwelt-Gesellschaft-Beziehungen und globale Probleme</t>
+          <t>Stoffwechsel und Regelmechanismen</t>
         </is>
       </c>
       <c r="D43" s="26" t="inlineStr">
         <is>
-          <t>Migration, Standortverlagerungen, wirtschaftliche Globalisierung</t>
+          <t>Aspekte zur ausgewogenen Ernährung</t>
         </is>
       </c>
       <c r="E43" s="26" t="inlineStr">
         <is>
-          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
+          <t>bis Ende 5/6</t>
         </is>
       </c>
       <c r="F43" s="26" t="inlineStr">
@@ -27601,27 +27601,27 @@
     <row r="44">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>Migration und Globalisierung</t>
-        </is>
-      </c>
-      <c r="B44" s="31" t="inlineStr">
-        <is>
-          <t>Politik und Wirtschaft</t>
+          <t>Ernährung, Gesundheit, Konsum</t>
+        </is>
+      </c>
+      <c r="B44" s="27" t="inlineStr">
+        <is>
+          <t>Biologie</t>
         </is>
       </c>
       <c r="C44" s="26" t="inlineStr">
         <is>
-          <t>Internationale Beziehungen und Globalisierung</t>
+          <t>Stoffwechsel und Regelmechanismen</t>
         </is>
       </c>
       <c r="D44" s="26" t="inlineStr">
         <is>
-          <t>Globalisierung; Migration und Integration</t>
+          <t>Bewertung des Konsumverhaltens im Hinblick auf Haltung und Nutzung von Lebewesen</t>
         </is>
       </c>
       <c r="E44" s="26" t="inlineStr">
         <is>
-          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
+          <t>bis Ende 5/6</t>
         </is>
       </c>
       <c r="F44" s="26" t="inlineStr">
@@ -27633,27 +27633,27 @@
     <row r="45">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>Technik, Forschung und Verantwortung</t>
-        </is>
-      </c>
-      <c r="B45" s="29" t="inlineStr">
-        <is>
-          <t>Physik</t>
+          <t>Ernährung, Gesundheit, Konsum</t>
+        </is>
+      </c>
+      <c r="B45" s="28" t="inlineStr">
+        <is>
+          <t>Chemie</t>
         </is>
       </c>
       <c r="C45" s="26" t="inlineStr">
         <is>
-          <t>Physik in der Verantwortung</t>
+          <t>Magie des Kohlenstoffs – Organische Verbindungen</t>
         </is>
       </c>
       <c r="D45" s="26" t="inlineStr">
         <is>
-          <t>Konsequenzen der Nutzung physikalischer Forschungsergebnisse</t>
+          <t>Organische Stoffe aus Ernährung und Hygiene (Kap. 6, S. 27)</t>
         </is>
       </c>
       <c r="E45" s="26" t="inlineStr">
         <is>
-          <t>zusätzlich bis Ende 9/10</t>
+          <t>Inhaltsfeldbeschreibung</t>
         </is>
       </c>
       <c r="F45" s="26" t="inlineStr">
@@ -27665,27 +27665,27 @@
     <row r="46">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>Technik, Forschung und Verantwortung</t>
-        </is>
-      </c>
-      <c r="B46" s="27" t="inlineStr">
-        <is>
-          <t>Biologie</t>
+          <t>Ernährung, Gesundheit, Konsum</t>
+        </is>
+      </c>
+      <c r="B46" s="31" t="inlineStr">
+        <is>
+          <t>Politik und Wirtschaft</t>
         </is>
       </c>
       <c r="C46" s="26" t="inlineStr">
         <is>
-          <t>Vielfalt, Veränderung und Abstammung von Lebewesen</t>
+          <t>Wirtschaft</t>
         </is>
       </c>
       <c r="D46" s="26" t="inlineStr">
         <is>
-          <t>Bewertung der Eingriffe des Menschen in das Erbgut</t>
+          <t>Rolle als Verbraucherinnen und Verbraucher</t>
         </is>
       </c>
       <c r="E46" s="26" t="inlineStr">
         <is>
-          <t>zusätzlich bis Ende 9/10</t>
+          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
         </is>
       </c>
       <c r="F46" s="26" t="inlineStr">
@@ -27697,27 +27697,27 @@
     <row r="47">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>Technik, Forschung und Verantwortung</t>
-        </is>
-      </c>
-      <c r="B47" s="27" t="inlineStr">
-        <is>
-          <t>Biologie</t>
+          <t>Ernährung, Gesundheit, Konsum</t>
+        </is>
+      </c>
+      <c r="B47" s="33" t="inlineStr">
+        <is>
+          <t>Arbeitslehre</t>
         </is>
       </c>
       <c r="C47" s="26" t="inlineStr">
         <is>
-          <t>Fortpflanzung und Entwicklung</t>
+          <t>Erhalt der psychischen und physischen Gesundheit</t>
         </is>
       </c>
       <c r="D47" s="26" t="inlineStr">
         <is>
-          <t>Bewertung gentechnischer Veränderungen von Pflanzen und Tieren</t>
+          <t>Gesundheitsförderliche Ernährung und Lebensstil</t>
         </is>
       </c>
       <c r="E47" s="26" t="inlineStr">
         <is>
-          <t>zusätzlich bis Ende 9/10</t>
+          <t>S. 21</t>
         </is>
       </c>
       <c r="F47" s="26" t="inlineStr">
@@ -27729,37 +27729,2949 @@
     <row r="48">
       <c r="A48" s="26" t="inlineStr">
         <is>
+          <t>Ernährung, Gesundheit, Konsum</t>
+        </is>
+      </c>
+      <c r="B48" s="33" t="inlineStr">
+        <is>
+          <t>Arbeitslehre</t>
+        </is>
+      </c>
+      <c r="C48" s="26" t="inlineStr">
+        <is>
+          <t>Ökonomisch geprägte Situationen und Strukturen des Zusammenlebens</t>
+        </is>
+      </c>
+      <c r="D48" s="26" t="inlineStr">
+        <is>
+          <t>Konsum, Marketingstrategien und Marktmechanismen</t>
+        </is>
+      </c>
+      <c r="E48" s="26" t="inlineStr">
+        <is>
+          <t>S. 21</t>
+        </is>
+      </c>
+      <c r="F48" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="26" t="inlineStr">
+        <is>
+          <t>Ernährung, Gesundheit, Konsum</t>
+        </is>
+      </c>
+      <c r="B49" s="39" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="C49" s="26" t="inlineStr">
+        <is>
+          <t>Den Körper trainieren, die Fitness verbessern</t>
+        </is>
+      </c>
+      <c r="D49" s="26" t="inlineStr">
+        <is>
+          <t>Fitness verbessern</t>
+        </is>
+      </c>
+      <c r="E49" s="26" t="inlineStr">
+        <is>
+          <t>S. 24</t>
+        </is>
+      </c>
+      <c r="F49" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="26" t="inlineStr">
+        <is>
+          <t>Ernährung, Gesundheit, Konsum</t>
+        </is>
+      </c>
+      <c r="B50" s="32" t="inlineStr">
+        <is>
+          <t>Geschichte</t>
+        </is>
+      </c>
+      <c r="C50" s="26" t="inlineStr">
+        <is>
+          <t>Alltagskulturen</t>
+        </is>
+      </c>
+      <c r="D50" s="26" t="inlineStr">
+        <is>
+          <t>Wohnen, Ernährung, Kleidung im Wandel</t>
+        </is>
+      </c>
+      <c r="E50" s="26" t="inlineStr">
+        <is>
+          <t>S. 22</t>
+        </is>
+      </c>
+      <c r="F50" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="26" t="inlineStr">
+        <is>
+          <t>Ernährung, Gesundheit, Konsum</t>
+        </is>
+      </c>
+      <c r="B51" s="35" t="inlineStr">
+        <is>
+          <t>Mathematik</t>
+        </is>
+      </c>
+      <c r="C51" s="26" t="inlineStr">
+        <is>
+          <t>Operationen und ihre Eigenschaften</t>
+        </is>
+      </c>
+      <c r="D51" s="26" t="inlineStr">
+        <is>
+          <t>Prozent- und Zinsrechnung für lebensnahe Fragestellungen</t>
+        </is>
+      </c>
+      <c r="E51" s="26" t="inlineStr">
+        <is>
+          <t>S. 19</t>
+        </is>
+      </c>
+      <c r="F51" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="26" t="inlineStr">
+        <is>
+          <t>Teilchen und Aufbau der Materie</t>
+        </is>
+      </c>
+      <c r="B52" s="28" t="inlineStr">
+        <is>
+          <t>Chemie</t>
+        </is>
+      </c>
+      <c r="C52" s="26" t="inlineStr">
+        <is>
+          <t>Blick hinter die Kulissen – Aufbau von Stoffen und chemische Bindung</t>
+        </is>
+      </c>
+      <c r="D52" s="26" t="inlineStr">
+        <is>
+          <t>Teilchenmodell zur Deutung von Phänomenen</t>
+        </is>
+      </c>
+      <c r="E52" s="26" t="inlineStr">
+        <is>
+          <t>1. Lernjahr</t>
+        </is>
+      </c>
+      <c r="F52" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="26" t="inlineStr">
+        <is>
+          <t>Teilchen und Aufbau der Materie</t>
+        </is>
+      </c>
+      <c r="B53" s="29" t="inlineStr">
+        <is>
+          <t>Physik</t>
+        </is>
+      </c>
+      <c r="C53" s="26" t="inlineStr">
+        <is>
+          <t>Wettererscheinungen und Klima</t>
+        </is>
+      </c>
+      <c r="D53" s="26" t="inlineStr">
+        <is>
+          <t>Modelle des Aufbaus der Materie; Aggregatzustände</t>
+        </is>
+      </c>
+      <c r="E53" s="26" t="inlineStr">
+        <is>
+          <t>nach ca. Hälfte des Stundenkontingents</t>
+        </is>
+      </c>
+      <c r="F53" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="26" t="inlineStr">
+        <is>
+          <t>Teilchen und Aufbau der Materie</t>
+        </is>
+      </c>
+      <c r="B54" s="28" t="inlineStr">
+        <is>
+          <t>Chemie</t>
+        </is>
+      </c>
+      <c r="C54" s="26" t="inlineStr">
+        <is>
+          <t>Verwandlungen – Chemische Reaktion</t>
+        </is>
+      </c>
+      <c r="D54" s="26" t="inlineStr">
+        <is>
+          <t>Aggregatzustand und Aggregatzustandsänderungen</t>
+        </is>
+      </c>
+      <c r="E54" s="26" t="inlineStr">
+        <is>
+          <t>1. Lernjahr</t>
+        </is>
+      </c>
+      <c r="F54" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="26" t="inlineStr">
+        <is>
+          <t>Teilchen und Aufbau der Materie</t>
+        </is>
+      </c>
+      <c r="B55" s="29" t="inlineStr">
+        <is>
+          <t>Physik</t>
+        </is>
+      </c>
+      <c r="C55" s="26" t="inlineStr">
+        <is>
+          <t>Physik in der Verantwortung</t>
+        </is>
+      </c>
+      <c r="D55" s="26" t="inlineStr">
+        <is>
+          <t>Radioaktive Zerfallsprozesse</t>
+        </is>
+      </c>
+      <c r="E55" s="26" t="inlineStr">
+        <is>
+          <t>zusätzlich bis Ende 9/10</t>
+        </is>
+      </c>
+      <c r="F55" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="26" t="inlineStr">
+        <is>
+          <t>Ressourcen und Recycling</t>
+        </is>
+      </c>
+      <c r="B56" s="28" t="inlineStr">
+        <is>
+          <t>Chemie</t>
+        </is>
+      </c>
+      <c r="C56" s="26" t="inlineStr">
+        <is>
+          <t>Magie des Kohlenstoffs – Organische Verbindungen</t>
+        </is>
+      </c>
+      <c r="D56" s="26" t="inlineStr">
+        <is>
+          <t>Gewinnung, Verwendung und Recycling organischer Stoffe</t>
+        </is>
+      </c>
+      <c r="E56" s="26" t="inlineStr">
+        <is>
+          <t>zusätzlich bis Ende 9/10</t>
+        </is>
+      </c>
+      <c r="F56" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="26" t="inlineStr">
+        <is>
+          <t>Ressourcen und Recycling</t>
+        </is>
+      </c>
+      <c r="B57" s="29" t="inlineStr">
+        <is>
+          <t>Physik</t>
+        </is>
+      </c>
+      <c r="C57" s="26" t="inlineStr">
+        <is>
+          <t>Zukunftssichere Energieversorgung</t>
+        </is>
+      </c>
+      <c r="D57" s="26" t="inlineStr">
+        <is>
+          <t>Regenerative und erschöpfbare Energien</t>
+        </is>
+      </c>
+      <c r="E57" s="26" t="inlineStr">
+        <is>
+          <t>nach ca. Hälfte des Stundenkontingents</t>
+        </is>
+      </c>
+      <c r="F57" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="26" t="inlineStr">
+        <is>
+          <t>Ressourcen und Recycling</t>
+        </is>
+      </c>
+      <c r="B58" s="30" t="inlineStr">
+        <is>
+          <t>Erdkunde</t>
+        </is>
+      </c>
+      <c r="C58" s="26" t="inlineStr">
+        <is>
+          <t>Umwelt-Gesellschaft-Beziehungen und globale Probleme</t>
+        </is>
+      </c>
+      <c r="D58" s="26" t="inlineStr">
+        <is>
+          <t>Ressourcensicherung</t>
+        </is>
+      </c>
+      <c r="E58" s="26" t="inlineStr">
+        <is>
+          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
+        </is>
+      </c>
+      <c r="F58" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="26" t="inlineStr">
+        <is>
+          <t>Ressourcen und Recycling</t>
+        </is>
+      </c>
+      <c r="B59" s="31" t="inlineStr">
+        <is>
+          <t>Politik und Wirtschaft</t>
+        </is>
+      </c>
+      <c r="C59" s="26" t="inlineStr">
+        <is>
+          <t>Gesellschaft und Natur</t>
+        </is>
+      </c>
+      <c r="D59" s="26" t="inlineStr">
+        <is>
+          <t>Spannungsfeld zwischen Ökonomie und Ökologie</t>
+        </is>
+      </c>
+      <c r="E59" s="26" t="inlineStr">
+        <is>
+          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
+        </is>
+      </c>
+      <c r="F59" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="26" t="inlineStr">
+        <is>
+          <t>Ressourcen und Recycling</t>
+        </is>
+      </c>
+      <c r="B60" s="33" t="inlineStr">
+        <is>
+          <t>Arbeitslehre</t>
+        </is>
+      </c>
+      <c r="C60" s="26" t="inlineStr">
+        <is>
+          <t>Organisation von Arbeit</t>
+        </is>
+      </c>
+      <c r="D60" s="26" t="inlineStr">
+        <is>
+          <t>Umweltschutz und Nachhaltigkeit</t>
+        </is>
+      </c>
+      <c r="E60" s="26" t="inlineStr">
+        <is>
+          <t>S. 21</t>
+        </is>
+      </c>
+      <c r="F60" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="26" t="inlineStr">
+        <is>
+          <t>Ressourcen und Recycling</t>
+        </is>
+      </c>
+      <c r="B61" s="32" t="inlineStr">
+        <is>
+          <t>Geschichte</t>
+        </is>
+      </c>
+      <c r="C61" s="26" t="inlineStr">
+        <is>
+          <t>Bewältigung und Nutzung von Räumen</t>
+        </is>
+      </c>
+      <c r="D61" s="26" t="inlineStr">
+        <is>
+          <t>Agrarische und industrielle Nutzung von Natur</t>
+        </is>
+      </c>
+      <c r="E61" s="26" t="inlineStr">
+        <is>
+          <t>S. 24</t>
+        </is>
+      </c>
+      <c r="F61" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="26" t="inlineStr">
+        <is>
+          <t>Migration und Globalisierung</t>
+        </is>
+      </c>
+      <c r="B62" s="30" t="inlineStr">
+        <is>
+          <t>Erdkunde</t>
+        </is>
+      </c>
+      <c r="C62" s="26" t="inlineStr">
+        <is>
+          <t>Mensch/Gesellschaft</t>
+        </is>
+      </c>
+      <c r="D62" s="26" t="inlineStr">
+        <is>
+          <t>Migration, Globalisierung, Metropolisierung</t>
+        </is>
+      </c>
+      <c r="E62" s="26" t="inlineStr">
+        <is>
+          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
+        </is>
+      </c>
+      <c r="F62" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="26" t="inlineStr">
+        <is>
+          <t>Migration und Globalisierung</t>
+        </is>
+      </c>
+      <c r="B63" s="30" t="inlineStr">
+        <is>
+          <t>Erdkunde</t>
+        </is>
+      </c>
+      <c r="C63" s="26" t="inlineStr">
+        <is>
+          <t>Umwelt-Gesellschaft-Beziehungen und globale Probleme</t>
+        </is>
+      </c>
+      <c r="D63" s="26" t="inlineStr">
+        <is>
+          <t>Migration, Standortverlagerungen, wirtschaftliche Globalisierung</t>
+        </is>
+      </c>
+      <c r="E63" s="26" t="inlineStr">
+        <is>
+          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
+        </is>
+      </c>
+      <c r="F63" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="26" t="inlineStr">
+        <is>
+          <t>Migration und Globalisierung</t>
+        </is>
+      </c>
+      <c r="B64" s="31" t="inlineStr">
+        <is>
+          <t>Politik und Wirtschaft</t>
+        </is>
+      </c>
+      <c r="C64" s="26" t="inlineStr">
+        <is>
+          <t>Internationale Beziehungen und Globalisierung</t>
+        </is>
+      </c>
+      <c r="D64" s="26" t="inlineStr">
+        <is>
+          <t>Globalisierung; Migration und Integration</t>
+        </is>
+      </c>
+      <c r="E64" s="26" t="inlineStr">
+        <is>
+          <t>keine Stufung im KC (gilt bis Ende 9/10)</t>
+        </is>
+      </c>
+      <c r="F64" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="26" t="inlineStr">
+        <is>
+          <t>Migration und Globalisierung</t>
+        </is>
+      </c>
+      <c r="B65" s="32" t="inlineStr">
+        <is>
+          <t>Geschichte</t>
+        </is>
+      </c>
+      <c r="C65" s="26" t="inlineStr">
+        <is>
+          <t>Eigenes und Fremdes</t>
+        </is>
+      </c>
+      <c r="D65" s="26" t="inlineStr">
+        <is>
+          <t>Zugehörigkeit durch Religion, Nation, Kultur, Ethnie</t>
+        </is>
+      </c>
+      <c r="E65" s="26" t="inlineStr">
+        <is>
+          <t>S. 23</t>
+        </is>
+      </c>
+      <c r="F65" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="26" t="inlineStr">
+        <is>
+          <t>Migration und Globalisierung</t>
+        </is>
+      </c>
+      <c r="B66" s="32" t="inlineStr">
+        <is>
+          <t>Geschichte</t>
+        </is>
+      </c>
+      <c r="C66" s="26" t="inlineStr">
+        <is>
+          <t>Epochenbezug Neuzeit</t>
+        </is>
+      </c>
+      <c r="D66" s="26" t="inlineStr">
+        <is>
+          <t>Kolonialismus, Imperialismus</t>
+        </is>
+      </c>
+      <c r="E66" s="26" t="inlineStr">
+        <is>
+          <t>S. 22</t>
+        </is>
+      </c>
+      <c r="F66" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="26" t="inlineStr">
+        <is>
+          <t>Migration und Globalisierung</t>
+        </is>
+      </c>
+      <c r="B67" s="36" t="inlineStr">
+        <is>
+          <t>Moderne Fremdsprachen</t>
+        </is>
+      </c>
+      <c r="C67" s="26" t="inlineStr">
+        <is>
+          <t>Kulturelle Lebenswelten „Ich und die Welt“</t>
+        </is>
+      </c>
+      <c r="D67" s="26" t="inlineStr">
+        <is>
+          <t>Kulturelle Aspekte des jeweiligen Sprachraums</t>
+        </is>
+      </c>
+      <c r="E67" s="26" t="inlineStr">
+        <is>
+          <t>S. 29</t>
+        </is>
+      </c>
+      <c r="F67" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="26" t="inlineStr">
+        <is>
+          <t>Migration und Globalisierung</t>
+        </is>
+      </c>
+      <c r="B68" s="40" t="inlineStr">
+        <is>
+          <t>Ethik</t>
+        </is>
+      </c>
+      <c r="C68" s="26" t="inlineStr">
+        <is>
+          <t>Religionen, Weltbilder und Kulturen</t>
+        </is>
+      </c>
+      <c r="D68" s="26" t="inlineStr">
+        <is>
+          <t>Weltbilder und Kulturen</t>
+        </is>
+      </c>
+      <c r="E68" s="26" t="inlineStr">
+        <is>
+          <t>S. 19</t>
+        </is>
+      </c>
+      <c r="F68" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="26" t="inlineStr">
+        <is>
+          <t>Migration und Globalisierung</t>
+        </is>
+      </c>
+      <c r="B69" s="33" t="inlineStr">
+        <is>
+          <t>Arbeitslehre</t>
+        </is>
+      </c>
+      <c r="C69" s="26" t="inlineStr">
+        <is>
+          <t>Berufswegeplanung</t>
+        </is>
+      </c>
+      <c r="D69" s="26" t="inlineStr">
+        <is>
+          <t>Wandel von Arbeit und Beruf, regional bis international</t>
+        </is>
+      </c>
+      <c r="E69" s="26" t="inlineStr">
+        <is>
+          <t>S. 20</t>
+        </is>
+      </c>
+      <c r="F69" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="26" t="inlineStr">
+        <is>
           <t>Technik, Forschung und Verantwortung</t>
         </is>
       </c>
-      <c r="B48" s="28" t="inlineStr">
+      <c r="B70" s="29" t="inlineStr">
+        <is>
+          <t>Physik</t>
+        </is>
+      </c>
+      <c r="C70" s="26" t="inlineStr">
+        <is>
+          <t>Physik in der Verantwortung</t>
+        </is>
+      </c>
+      <c r="D70" s="26" t="inlineStr">
+        <is>
+          <t>Konsequenzen der Nutzung physikalischer Forschungsergebnisse</t>
+        </is>
+      </c>
+      <c r="E70" s="26" t="inlineStr">
+        <is>
+          <t>zusätzlich bis Ende 9/10</t>
+        </is>
+      </c>
+      <c r="F70" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="26" t="inlineStr">
+        <is>
+          <t>Technik, Forschung und Verantwortung</t>
+        </is>
+      </c>
+      <c r="B71" s="27" t="inlineStr">
+        <is>
+          <t>Biologie</t>
+        </is>
+      </c>
+      <c r="C71" s="26" t="inlineStr">
+        <is>
+          <t>Vielfalt, Veränderung und Abstammung von Lebewesen</t>
+        </is>
+      </c>
+      <c r="D71" s="26" t="inlineStr">
+        <is>
+          <t>Bewertung der Eingriffe des Menschen in das Erbgut</t>
+        </is>
+      </c>
+      <c r="E71" s="26" t="inlineStr">
+        <is>
+          <t>zusätzlich bis Ende 9/10</t>
+        </is>
+      </c>
+      <c r="F71" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="26" t="inlineStr">
+        <is>
+          <t>Technik, Forschung und Verantwortung</t>
+        </is>
+      </c>
+      <c r="B72" s="27" t="inlineStr">
+        <is>
+          <t>Biologie</t>
+        </is>
+      </c>
+      <c r="C72" s="26" t="inlineStr">
+        <is>
+          <t>Fortpflanzung und Entwicklung</t>
+        </is>
+      </c>
+      <c r="D72" s="26" t="inlineStr">
+        <is>
+          <t>Bewertung gentechnischer Veränderungen von Pflanzen und Tieren</t>
+        </is>
+      </c>
+      <c r="E72" s="26" t="inlineStr">
+        <is>
+          <t>zusätzlich bis Ende 9/10</t>
+        </is>
+      </c>
+      <c r="F72" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="26" t="inlineStr">
+        <is>
+          <t>Technik, Forschung und Verantwortung</t>
+        </is>
+      </c>
+      <c r="B73" s="28" t="inlineStr">
         <is>
           <t>Chemie</t>
         </is>
       </c>
-      <c r="C48" s="26" t="inlineStr">
+      <c r="C73" s="26" t="inlineStr">
         <is>
           <t>Verwandlungen – Chemische Reaktion</t>
         </is>
       </c>
-      <c r="D48" s="26" t="inlineStr">
+      <c r="D73" s="26" t="inlineStr">
         <is>
           <t>Chancen und Grenzen bei der Herstellung von Stoffen (Bewertung, Kap. 6, S. 24)</t>
         </is>
       </c>
-      <c r="E48" s="26" t="inlineStr">
+      <c r="E73" s="26" t="inlineStr">
         <is>
           <t>Inhaltsfeldbeschreibung</t>
         </is>
       </c>
-      <c r="F48" s="26" t="inlineStr">
+      <c r="F73" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" s="26" t="inlineStr">
+        <is>
+          <t>Technik, Forschung und Verantwortung</t>
+        </is>
+      </c>
+      <c r="B74" s="40" t="inlineStr">
+        <is>
+          <t>Ethik</t>
+        </is>
+      </c>
+      <c r="C74" s="26" t="inlineStr">
+        <is>
+          <t>Mensch, Natur und Technik</t>
+        </is>
+      </c>
+      <c r="D74" s="26" t="inlineStr">
+        <is>
+          <t>Verantwortung im Umgang mit Technik, angewandte Ethik</t>
+        </is>
+      </c>
+      <c r="E74" s="26" t="inlineStr">
+        <is>
+          <t>S. 19</t>
+        </is>
+      </c>
+      <c r="F74" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="26" t="inlineStr">
+        <is>
+          <t>Technik, Forschung und Verantwortung</t>
+        </is>
+      </c>
+      <c r="B75" s="33" t="inlineStr">
+        <is>
+          <t>Arbeitslehre</t>
+        </is>
+      </c>
+      <c r="C75" s="26" t="inlineStr">
+        <is>
+          <t>Technische Systeme und Prozesse</t>
+        </is>
+      </c>
+      <c r="D75" s="26" t="inlineStr">
+        <is>
+          <t>Reflektierte Anwendung von Technik</t>
+        </is>
+      </c>
+      <c r="E75" s="26" t="inlineStr">
+        <is>
+          <t>S. 20</t>
+        </is>
+      </c>
+      <c r="F75" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="26" t="inlineStr">
+        <is>
+          <t>Technik, Forschung und Verantwortung</t>
+        </is>
+      </c>
+      <c r="B76" s="43" t="inlineStr">
+        <is>
+          <t>Informatik</t>
+        </is>
+      </c>
+      <c r="C76" s="26" t="inlineStr">
+        <is>
+          <t>Kryptologie</t>
+        </is>
+      </c>
+      <c r="D76" s="26" t="inlineStr">
+        <is>
+          <t>Verschlüsselung von Daten</t>
+        </is>
+      </c>
+      <c r="E76" s="26" t="inlineStr">
+        <is>
+          <t>S. 21</t>
+        </is>
+      </c>
+      <c r="F76" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="26" t="inlineStr">
+        <is>
+          <t>Technik, Forschung und Verantwortung</t>
+        </is>
+      </c>
+      <c r="B77" s="42" t="inlineStr">
+        <is>
+          <t>Katholische Religion</t>
+        </is>
+      </c>
+      <c r="C77" s="26" t="inlineStr">
+        <is>
+          <t>Mensch und Welt</t>
+        </is>
+      </c>
+      <c r="D77" s="26" t="inlineStr">
+        <is>
+          <t>Schöpfungsglaube und naturwissenschaftliche Theorien</t>
+        </is>
+      </c>
+      <c r="E77" s="26" t="inlineStr">
+        <is>
+          <t>S. 17</t>
+        </is>
+      </c>
+      <c r="F77" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="26" t="inlineStr">
+        <is>
+          <t>Identität und Erwachsenwerden</t>
+        </is>
+      </c>
+      <c r="B78" s="40" t="inlineStr">
+        <is>
+          <t>Ethik</t>
+        </is>
+      </c>
+      <c r="C78" s="26" t="inlineStr">
+        <is>
+          <t>Selbst und Welt</t>
+        </is>
+      </c>
+      <c r="D78" s="26" t="inlineStr">
+        <is>
+          <t>Der Mensch als fühlendes, denkendes und handelndes Wesen</t>
+        </is>
+      </c>
+      <c r="E78" s="26" t="inlineStr">
+        <is>
+          <t>S. 18</t>
+        </is>
+      </c>
+      <c r="F78" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="26" t="inlineStr">
+        <is>
+          <t>Identität und Erwachsenwerden</t>
+        </is>
+      </c>
+      <c r="B79" s="41" t="inlineStr">
+        <is>
+          <t>Evangelische Religion</t>
+        </is>
+      </c>
+      <c r="C79" s="26" t="inlineStr">
+        <is>
+          <t>Mensch und Welt</t>
+        </is>
+      </c>
+      <c r="D79" s="26" t="inlineStr">
+        <is>
+          <t>Fragen nach Identität und Sinn des eigenen Lebens</t>
+        </is>
+      </c>
+      <c r="E79" s="26" t="inlineStr">
+        <is>
+          <t>S. 19</t>
+        </is>
+      </c>
+      <c r="F79" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="26" t="inlineStr">
+        <is>
+          <t>Identität und Erwachsenwerden</t>
+        </is>
+      </c>
+      <c r="B80" s="37" t="inlineStr">
+        <is>
+          <t>Kunst</t>
+        </is>
+      </c>
+      <c r="C80" s="26" t="inlineStr">
+        <is>
+          <t>Standpunkte zu Konfliktfeldern des Erwachsenwerdens</t>
+        </is>
+      </c>
+      <c r="D80" s="26" t="inlineStr">
+        <is>
+          <t>Konfliktfelder des Erwachsenwerdens</t>
+        </is>
+      </c>
+      <c r="E80" s="26" t="inlineStr">
+        <is>
+          <t>S. 21</t>
+        </is>
+      </c>
+      <c r="F80" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="26" t="inlineStr">
+        <is>
+          <t>Identität und Erwachsenwerden</t>
+        </is>
+      </c>
+      <c r="B81" s="27" t="inlineStr">
+        <is>
+          <t>Biologie</t>
+        </is>
+      </c>
+      <c r="C81" s="26" t="inlineStr">
+        <is>
+          <t>Sexualität des Menschen</t>
+        </is>
+      </c>
+      <c r="D81" s="26" t="inlineStr">
+        <is>
+          <t>Veränderungen während der Pubertät</t>
+        </is>
+      </c>
+      <c r="E81" s="26" t="inlineStr">
+        <is>
+          <t>S. 46</t>
+        </is>
+      </c>
+      <c r="F81" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="26" t="inlineStr">
+        <is>
+          <t>Identität und Erwachsenwerden</t>
+        </is>
+      </c>
+      <c r="B82" s="33" t="inlineStr">
+        <is>
+          <t>Arbeitslehre</t>
+        </is>
+      </c>
+      <c r="C82" s="26" t="inlineStr">
+        <is>
+          <t>Berufswegeplanung</t>
+        </is>
+      </c>
+      <c r="D82" s="26" t="inlineStr">
+        <is>
+          <t>Identität und berufliches Selbstkonzept</t>
+        </is>
+      </c>
+      <c r="E82" s="26" t="inlineStr">
+        <is>
+          <t>S. 20</t>
+        </is>
+      </c>
+      <c r="F82" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="26" t="inlineStr">
+        <is>
+          <t>Identität und Erwachsenwerden</t>
+        </is>
+      </c>
+      <c r="B83" s="36" t="inlineStr">
+        <is>
+          <t>Moderne Fremdsprachen</t>
+        </is>
+      </c>
+      <c r="C83" s="26" t="inlineStr">
+        <is>
+          <t>Persönliche Lebenswelten „Ich und die Anderen“</t>
+        </is>
+      </c>
+      <c r="D83" s="26" t="inlineStr">
+        <is>
+          <t>„Ich und die Anderen“</t>
+        </is>
+      </c>
+      <c r="E83" s="26" t="inlineStr">
+        <is>
+          <t>S. 29</t>
+        </is>
+      </c>
+      <c r="F83" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="26" t="inlineStr">
+        <is>
+          <t>Identität und Erwachsenwerden</t>
+        </is>
+      </c>
+      <c r="B84" s="32" t="inlineStr">
+        <is>
+          <t>Geschichte</t>
+        </is>
+      </c>
+      <c r="C84" s="26" t="inlineStr">
+        <is>
+          <t>Eigenes und Fremdes</t>
+        </is>
+      </c>
+      <c r="D84" s="26" t="inlineStr">
+        <is>
+          <t>Identität und Wahrnehmung des eigenen Ichs</t>
+        </is>
+      </c>
+      <c r="E84" s="26" t="inlineStr">
+        <is>
+          <t>S. 23</t>
+        </is>
+      </c>
+      <c r="F84" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="26" t="inlineStr">
+        <is>
+          <t>Kommunikation und Medien</t>
+        </is>
+      </c>
+      <c r="B85" s="34" t="inlineStr">
+        <is>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="C85" s="26" t="inlineStr">
+        <is>
+          <t>Text-/Medienformen</t>
+        </is>
+      </c>
+      <c r="D85" s="26" t="inlineStr">
+        <is>
+          <t>Text- und Medienformen</t>
+        </is>
+      </c>
+      <c r="E85" s="26" t="inlineStr">
+        <is>
+          <t>S. 24</t>
+        </is>
+      </c>
+      <c r="F85" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="26" t="inlineStr">
+        <is>
+          <t>Kommunikation und Medien</t>
+        </is>
+      </c>
+      <c r="B86" s="34" t="inlineStr">
+        <is>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="C86" s="26" t="inlineStr">
+        <is>
+          <t>Rede- und Gesprächsformen</t>
+        </is>
+      </c>
+      <c r="D86" s="26" t="inlineStr">
+        <is>
+          <t>Informierende und argumentierende Gespräche</t>
+        </is>
+      </c>
+      <c r="E86" s="26" t="inlineStr">
+        <is>
+          <t>S. 22</t>
+        </is>
+      </c>
+      <c r="F86" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="26" t="inlineStr">
+        <is>
+          <t>Kommunikation und Medien</t>
+        </is>
+      </c>
+      <c r="B87" s="37" t="inlineStr">
+        <is>
+          <t>Kunst</t>
+        </is>
+      </c>
+      <c r="C87" s="26" t="inlineStr">
+        <is>
+          <t>Medien, Techniken und Verfahren der Bildgestaltung</t>
+        </is>
+      </c>
+      <c r="D87" s="26" t="inlineStr">
+        <is>
+          <t>Digitale Gestaltung, Fotografie</t>
+        </is>
+      </c>
+      <c r="E87" s="26" t="inlineStr">
+        <is>
+          <t>S. 20</t>
+        </is>
+      </c>
+      <c r="F87" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="26" t="inlineStr">
+        <is>
+          <t>Kommunikation und Medien</t>
+        </is>
+      </c>
+      <c r="B88" s="38" t="inlineStr">
+        <is>
+          <t>Musik</t>
+        </is>
+      </c>
+      <c r="C88" s="26" t="inlineStr">
+        <is>
+          <t>Bewegung und Gestaltungsmedien</t>
+        </is>
+      </c>
+      <c r="D88" s="26" t="inlineStr">
+        <is>
+          <t>Analoge und digitale Medien</t>
+        </is>
+      </c>
+      <c r="E88" s="26" t="inlineStr">
+        <is>
+          <t>S. 18</t>
+        </is>
+      </c>
+      <c r="F88" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="26" t="inlineStr">
+        <is>
+          <t>Kommunikation und Medien</t>
+        </is>
+      </c>
+      <c r="B89" s="43" t="inlineStr">
+        <is>
+          <t>Informatik</t>
+        </is>
+      </c>
+      <c r="C89" s="26" t="inlineStr">
+        <is>
+          <t>Internet und HTML</t>
+        </is>
+      </c>
+      <c r="D89" s="26" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="E89" s="26" t="inlineStr">
+        <is>
+          <t>S. 17</t>
+        </is>
+      </c>
+      <c r="F89" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="26" t="inlineStr">
+        <is>
+          <t>Kommunikation und Medien</t>
+        </is>
+      </c>
+      <c r="B90" s="33" t="inlineStr">
+        <is>
+          <t>Arbeitslehre</t>
+        </is>
+      </c>
+      <c r="C90" s="26" t="inlineStr">
+        <is>
+          <t>Technische Systeme und Prozesse</t>
+        </is>
+      </c>
+      <c r="D90" s="26" t="inlineStr">
+        <is>
+          <t>Informations- und Kommunikationstechnik</t>
+        </is>
+      </c>
+      <c r="E90" s="26" t="inlineStr">
+        <is>
+          <t>S. 20</t>
+        </is>
+      </c>
+      <c r="F90" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="26" t="inlineStr">
+        <is>
+          <t>Kommunikation und Medien</t>
+        </is>
+      </c>
+      <c r="B91" s="31" t="inlineStr">
+        <is>
+          <t>Politik und Wirtschaft</t>
+        </is>
+      </c>
+      <c r="C91" s="26" t="inlineStr">
+        <is>
+          <t>Demokratie</t>
+        </is>
+      </c>
+      <c r="D91" s="26" t="inlineStr">
+        <is>
+          <t>Rolle der Medien in der Demokratie</t>
+        </is>
+      </c>
+      <c r="E91" s="26" t="inlineStr">
+        <is>
+          <t>S. 25</t>
+        </is>
+      </c>
+      <c r="F91" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="26" t="inlineStr">
+        <is>
+          <t>Demokratie, Recht und Gerechtigkeit</t>
+        </is>
+      </c>
+      <c r="B92" s="31" t="inlineStr">
+        <is>
+          <t>Politik und Wirtschaft</t>
+        </is>
+      </c>
+      <c r="C92" s="26" t="inlineStr">
+        <is>
+          <t>Demokratie</t>
+        </is>
+      </c>
+      <c r="D92" s="26" t="inlineStr">
+        <is>
+          <t>Demokratie</t>
+        </is>
+      </c>
+      <c r="E92" s="26" t="inlineStr">
+        <is>
+          <t>S. 25</t>
+        </is>
+      </c>
+      <c r="F92" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="26" t="inlineStr">
+        <is>
+          <t>Demokratie, Recht und Gerechtigkeit</t>
+        </is>
+      </c>
+      <c r="B93" s="31" t="inlineStr">
+        <is>
+          <t>Politik und Wirtschaft</t>
+        </is>
+      </c>
+      <c r="C93" s="26" t="inlineStr">
+        <is>
+          <t>Recht und Rechtsprechung</t>
+        </is>
+      </c>
+      <c r="D93" s="26" t="inlineStr">
+        <is>
+          <t>Recht und Rechtsprechung</t>
+        </is>
+      </c>
+      <c r="E93" s="26" t="inlineStr">
+        <is>
+          <t>S. 26</t>
+        </is>
+      </c>
+      <c r="F93" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="26" t="inlineStr">
+        <is>
+          <t>Demokratie, Recht und Gerechtigkeit</t>
+        </is>
+      </c>
+      <c r="B94" s="32" t="inlineStr">
+        <is>
+          <t>Geschichte</t>
+        </is>
+      </c>
+      <c r="C94" s="26" t="inlineStr">
+        <is>
+          <t>Herrschaft</t>
+        </is>
+      </c>
+      <c r="D94" s="26" t="inlineStr">
+        <is>
+          <t>Freiheitsrechte (Menschenrechte), rechtsstaatliche und demokratische Ordnungen</t>
+        </is>
+      </c>
+      <c r="E94" s="26" t="inlineStr">
+        <is>
+          <t>S. 23</t>
+        </is>
+      </c>
+      <c r="F94" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="26" t="inlineStr">
+        <is>
+          <t>Demokratie, Recht und Gerechtigkeit</t>
+        </is>
+      </c>
+      <c r="B95" s="32" t="inlineStr">
+        <is>
+          <t>Geschichte</t>
+        </is>
+      </c>
+      <c r="C95" s="26" t="inlineStr">
+        <is>
+          <t>Epochenbezug Antike</t>
+        </is>
+      </c>
+      <c r="D95" s="26" t="inlineStr">
+        <is>
+          <t>Freiheit und Mitbestimmung in der griechischen Polis</t>
+        </is>
+      </c>
+      <c r="E95" s="26" t="inlineStr">
+        <is>
+          <t>S. 21</t>
+        </is>
+      </c>
+      <c r="F95" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="26" t="inlineStr">
+        <is>
+          <t>Demokratie, Recht und Gerechtigkeit</t>
+        </is>
+      </c>
+      <c r="B96" s="40" t="inlineStr">
+        <is>
+          <t>Ethik</t>
+        </is>
+      </c>
+      <c r="C96" s="26" t="inlineStr">
+        <is>
+          <t>Recht und Gerechtigkeit</t>
+        </is>
+      </c>
+      <c r="D96" s="26" t="inlineStr">
+        <is>
+          <t>Arten der Gerechtigkeit, Menschenrechte</t>
+        </is>
+      </c>
+      <c r="E96" s="26" t="inlineStr">
+        <is>
+          <t>S. 18</t>
+        </is>
+      </c>
+      <c r="F96" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="26" t="inlineStr">
+        <is>
+          <t>Demokratie, Recht und Gerechtigkeit</t>
+        </is>
+      </c>
+      <c r="B97" s="40" t="inlineStr">
+        <is>
+          <t>Ethik</t>
+        </is>
+      </c>
+      <c r="C97" s="26" t="inlineStr">
+        <is>
+          <t>Freiheit und Würde</t>
+        </is>
+      </c>
+      <c r="D97" s="26" t="inlineStr">
+        <is>
+          <t>Würde aller Menschen</t>
+        </is>
+      </c>
+      <c r="E97" s="26" t="inlineStr">
+        <is>
+          <t>S. 19</t>
+        </is>
+      </c>
+      <c r="F97" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="26" t="inlineStr">
+        <is>
+          <t>Demokratie, Recht und Gerechtigkeit</t>
+        </is>
+      </c>
+      <c r="B98" s="34" t="inlineStr">
+        <is>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="C98" s="26" t="inlineStr">
+        <is>
+          <t>Rede- und Gesprächskonventionen</t>
+        </is>
+      </c>
+      <c r="D98" s="26" t="inlineStr">
+        <is>
+          <t>Gesprächskonventionen als Voraussetzung von Demokratie</t>
+        </is>
+      </c>
+      <c r="E98" s="26" t="inlineStr">
+        <is>
+          <t>S. 23</t>
+        </is>
+      </c>
+      <c r="F98" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="26" t="inlineStr">
+        <is>
+          <t>Demokratie, Recht und Gerechtigkeit</t>
+        </is>
+      </c>
+      <c r="B99" s="39" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="C99" s="26" t="inlineStr">
+        <is>
+          <t>Spielen</t>
+        </is>
+      </c>
+      <c r="D99" s="26" t="inlineStr">
+        <is>
+          <t>Regeln aushandeln, einhalten und verändern</t>
+        </is>
+      </c>
+      <c r="E99" s="26" t="inlineStr">
+        <is>
+          <t>S. 20</t>
+        </is>
+      </c>
+      <c r="F99" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="26" t="inlineStr">
+        <is>
+          <t>Demokratie, Recht und Gerechtigkeit</t>
+        </is>
+      </c>
+      <c r="B100" s="42" t="inlineStr">
+        <is>
+          <t>Katholische Religion</t>
+        </is>
+      </c>
+      <c r="C100" s="26" t="inlineStr">
+        <is>
+          <t>Bibel und Tradition</t>
+        </is>
+      </c>
+      <c r="D100" s="26" t="inlineStr">
+        <is>
+          <t>Frieden, Gerechtigkeit und Bewahrung der Schöpfung</t>
+        </is>
+      </c>
+      <c r="E100" s="26" t="inlineStr">
+        <is>
+          <t>S. 18</t>
+        </is>
+      </c>
+      <c r="F100" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="26" t="inlineStr">
+        <is>
+          <t>Glaube, Religionen und Weltdeutung</t>
+        </is>
+      </c>
+      <c r="B101" s="41" t="inlineStr">
+        <is>
+          <t>Evangelische Religion</t>
+        </is>
+      </c>
+      <c r="C101" s="26" t="inlineStr">
+        <is>
+          <t>Religionen</t>
+        </is>
+      </c>
+      <c r="D101" s="26" t="inlineStr">
+        <is>
+          <t>Interreligiöser Dialog, besonders Judentum und Christentum</t>
+        </is>
+      </c>
+      <c r="E101" s="26" t="inlineStr">
+        <is>
+          <t>S. 21</t>
+        </is>
+      </c>
+      <c r="F101" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="26" t="inlineStr">
+        <is>
+          <t>Glaube, Religionen und Weltdeutung</t>
+        </is>
+      </c>
+      <c r="B102" s="42" t="inlineStr">
+        <is>
+          <t>Katholische Religion</t>
+        </is>
+      </c>
+      <c r="C102" s="26" t="inlineStr">
+        <is>
+          <t>Religionen</t>
+        </is>
+      </c>
+      <c r="D102" s="26" t="inlineStr">
+        <is>
+          <t>Religionen</t>
+        </is>
+      </c>
+      <c r="E102" s="26" t="inlineStr">
+        <is>
+          <t>S. 19</t>
+        </is>
+      </c>
+      <c r="F102" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="26" t="inlineStr">
+        <is>
+          <t>Glaube, Religionen und Weltdeutung</t>
+        </is>
+      </c>
+      <c r="B103" s="41" t="inlineStr">
+        <is>
+          <t>Evangelische Religion</t>
+        </is>
+      </c>
+      <c r="C103" s="26" t="inlineStr">
+        <is>
+          <t>Gott</t>
+        </is>
+      </c>
+      <c r="D103" s="26" t="inlineStr">
+        <is>
+          <t>Gott</t>
+        </is>
+      </c>
+      <c r="E103" s="26" t="inlineStr">
+        <is>
+          <t>S. 19</t>
+        </is>
+      </c>
+      <c r="F103" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="26" t="inlineStr">
+        <is>
+          <t>Glaube, Religionen und Weltdeutung</t>
+        </is>
+      </c>
+      <c r="B104" s="42" t="inlineStr">
+        <is>
+          <t>Katholische Religion</t>
+        </is>
+      </c>
+      <c r="C104" s="26" t="inlineStr">
+        <is>
+          <t>Gott</t>
+        </is>
+      </c>
+      <c r="D104" s="26" t="inlineStr">
+        <is>
+          <t>Gott</t>
+        </is>
+      </c>
+      <c r="E104" s="26" t="inlineStr">
+        <is>
+          <t>S. 17</t>
+        </is>
+      </c>
+      <c r="F104" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="26" t="inlineStr">
+        <is>
+          <t>Glaube, Religionen und Weltdeutung</t>
+        </is>
+      </c>
+      <c r="B105" s="40" t="inlineStr">
+        <is>
+          <t>Ethik</t>
+        </is>
+      </c>
+      <c r="C105" s="26" t="inlineStr">
+        <is>
+          <t>Religionen, Weltbilder und Kulturen</t>
+        </is>
+      </c>
+      <c r="D105" s="26" t="inlineStr">
+        <is>
+          <t>Religionen und Weltbilder</t>
+        </is>
+      </c>
+      <c r="E105" s="26" t="inlineStr">
+        <is>
+          <t>S. 19</t>
+        </is>
+      </c>
+      <c r="F105" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="26" t="inlineStr">
+        <is>
+          <t>Glaube, Religionen und Weltdeutung</t>
+        </is>
+      </c>
+      <c r="B106" s="32" t="inlineStr">
+        <is>
+          <t>Geschichte</t>
+        </is>
+      </c>
+      <c r="C106" s="26" t="inlineStr">
+        <is>
+          <t>Epochenbezug Mittelalter</t>
+        </is>
+      </c>
+      <c r="D106" s="26" t="inlineStr">
+        <is>
+          <t>Einflüsse von Religionen auf Weltdeutungen</t>
+        </is>
+      </c>
+      <c r="E106" s="26" t="inlineStr">
+        <is>
+          <t>S. 21</t>
+        </is>
+      </c>
+      <c r="F106" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="26" t="inlineStr">
+        <is>
+          <t>Glaube, Religionen und Weltdeutung</t>
+        </is>
+      </c>
+      <c r="B107" s="32" t="inlineStr">
+        <is>
+          <t>Geschichte</t>
+        </is>
+      </c>
+      <c r="C107" s="26" t="inlineStr">
+        <is>
+          <t>Alltagskulturen</t>
+        </is>
+      </c>
+      <c r="D107" s="26" t="inlineStr">
+        <is>
+          <t>Glauben und Religion im Alltag</t>
+        </is>
+      </c>
+      <c r="E107" s="26" t="inlineStr">
+        <is>
+          <t>S. 22</t>
+        </is>
+      </c>
+      <c r="F107" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="26" t="inlineStr">
+        <is>
+          <t>Arbeit, Beruf und Zukunft</t>
+        </is>
+      </c>
+      <c r="B108" s="33" t="inlineStr">
+        <is>
+          <t>Arbeitslehre</t>
+        </is>
+      </c>
+      <c r="C108" s="26" t="inlineStr">
+        <is>
+          <t>Berufswegeplanung</t>
+        </is>
+      </c>
+      <c r="D108" s="26" t="inlineStr">
+        <is>
+          <t>Berufswahl als Prozess</t>
+        </is>
+      </c>
+      <c r="E108" s="26" t="inlineStr">
+        <is>
+          <t>S. 20</t>
+        </is>
+      </c>
+      <c r="F108" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="26" t="inlineStr">
+        <is>
+          <t>Arbeit, Beruf und Zukunft</t>
+        </is>
+      </c>
+      <c r="B109" s="33" t="inlineStr">
+        <is>
+          <t>Arbeitslehre</t>
+        </is>
+      </c>
+      <c r="C109" s="26" t="inlineStr">
+        <is>
+          <t>Zukunft der Arbeit</t>
+        </is>
+      </c>
+      <c r="D109" s="26" t="inlineStr">
+        <is>
+          <t>Szenarien zukünftiger Arbeit</t>
+        </is>
+      </c>
+      <c r="E109" s="26" t="inlineStr">
+        <is>
+          <t>S. 21</t>
+        </is>
+      </c>
+      <c r="F109" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="26" t="inlineStr">
+        <is>
+          <t>Arbeit, Beruf und Zukunft</t>
+        </is>
+      </c>
+      <c r="B110" s="33" t="inlineStr">
+        <is>
+          <t>Arbeitslehre</t>
+        </is>
+      </c>
+      <c r="C110" s="26" t="inlineStr">
+        <is>
+          <t>Organisation von Arbeit</t>
+        </is>
+      </c>
+      <c r="D110" s="26" t="inlineStr">
+        <is>
+          <t>Menschengerechte Arbeitsbedingungen</t>
+        </is>
+      </c>
+      <c r="E110" s="26" t="inlineStr">
+        <is>
+          <t>S. 21</t>
+        </is>
+      </c>
+      <c r="F110" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="26" t="inlineStr">
+        <is>
+          <t>Arbeit, Beruf und Zukunft</t>
+        </is>
+      </c>
+      <c r="B111" s="31" t="inlineStr">
+        <is>
+          <t>Politik und Wirtschaft</t>
+        </is>
+      </c>
+      <c r="C111" s="26" t="inlineStr">
+        <is>
+          <t>Wirtschaft</t>
+        </is>
+      </c>
+      <c r="D111" s="26" t="inlineStr">
+        <is>
+          <t>Wirtschaft</t>
+        </is>
+      </c>
+      <c r="E111" s="26" t="inlineStr">
+        <is>
+          <t>S. 25 f.</t>
+        </is>
+      </c>
+      <c r="F111" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="26" t="inlineStr">
+        <is>
+          <t>Arbeit, Beruf und Zukunft</t>
+        </is>
+      </c>
+      <c r="B112" s="32" t="inlineStr">
+        <is>
+          <t>Geschichte</t>
+        </is>
+      </c>
+      <c r="C112" s="26" t="inlineStr">
+        <is>
+          <t>Wirtschaft</t>
+        </is>
+      </c>
+      <c r="D112" s="26" t="inlineStr">
+        <is>
+          <t>Bedeutung von Arbeit für die Lebensgrundlagen</t>
+        </is>
+      </c>
+      <c r="E112" s="26" t="inlineStr">
+        <is>
+          <t>S. 23</t>
+        </is>
+      </c>
+      <c r="F112" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="26" t="inlineStr">
+        <is>
+          <t>Arbeit, Beruf und Zukunft</t>
+        </is>
+      </c>
+      <c r="B113" s="42" t="inlineStr">
+        <is>
+          <t>Katholische Religion</t>
+        </is>
+      </c>
+      <c r="C113" s="26" t="inlineStr">
+        <is>
+          <t>Mensch und Welt</t>
+        </is>
+      </c>
+      <c r="D113" s="26" t="inlineStr">
+        <is>
+          <t>Durch Arbeit Anteil am Schöpfungsauftrag</t>
+        </is>
+      </c>
+      <c r="E113" s="26" t="inlineStr">
+        <is>
+          <t>S. 17</t>
+        </is>
+      </c>
+      <c r="F113" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="26" t="inlineStr">
+        <is>
+          <t>Arbeit, Beruf und Zukunft</t>
+        </is>
+      </c>
+      <c r="B114" s="34" t="inlineStr">
+        <is>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="C114" s="26" t="inlineStr">
+        <is>
+          <t>Rede- und Gesprächsformen</t>
+        </is>
+      </c>
+      <c r="D114" s="26" t="inlineStr">
+        <is>
+          <t>Vorstellen und Bewerben</t>
+        </is>
+      </c>
+      <c r="E114" s="26" t="inlineStr">
+        <is>
+          <t>S. 22</t>
+        </is>
+      </c>
+      <c r="F114" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="26" t="inlineStr">
+        <is>
+          <t>Kultur und künstlerischer Ausdruck</t>
+        </is>
+      </c>
+      <c r="B115" s="37" t="inlineStr">
+        <is>
+          <t>Kunst</t>
+        </is>
+      </c>
+      <c r="C115" s="26" t="inlineStr">
+        <is>
+          <t>Ausdrucksmöglichkeiten der Kunst in kulturellen und gesellschaftlichen Kontexten / Bildbetrachtung</t>
+        </is>
+      </c>
+      <c r="D115" s="26" t="inlineStr">
+        <is>
+          <t>Kunst in kulturellen Kontexten</t>
+        </is>
+      </c>
+      <c r="E115" s="26" t="inlineStr">
+        <is>
+          <t>S. 20</t>
+        </is>
+      </c>
+      <c r="F115" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="26" t="inlineStr">
+        <is>
+          <t>Kultur und künstlerischer Ausdruck</t>
+        </is>
+      </c>
+      <c r="B116" s="38" t="inlineStr">
+        <is>
+          <t>Musik</t>
+        </is>
+      </c>
+      <c r="C116" s="26" t="inlineStr">
+        <is>
+          <t>Kontext</t>
+        </is>
+      </c>
+      <c r="D116" s="26" t="inlineStr">
+        <is>
+          <t>Geschichtliche, personale und ethnische Kontexte von Musik</t>
+        </is>
+      </c>
+      <c r="E116" s="26" t="inlineStr">
+        <is>
+          <t>S. 18</t>
+        </is>
+      </c>
+      <c r="F116" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="26" t="inlineStr">
+        <is>
+          <t>Kultur und künstlerischer Ausdruck</t>
+        </is>
+      </c>
+      <c r="B117" s="38" t="inlineStr">
+        <is>
+          <t>Musik</t>
+        </is>
+      </c>
+      <c r="C117" s="26" t="inlineStr">
+        <is>
+          <t>Gebrauchspraxis</t>
+        </is>
+      </c>
+      <c r="D117" s="26" t="inlineStr">
+        <is>
+          <t>Identitätsstiftendes Moment musikalischer Gebrauchspraxis</t>
+        </is>
+      </c>
+      <c r="E117" s="26" t="inlineStr">
+        <is>
+          <t>S. 18</t>
+        </is>
+      </c>
+      <c r="F117" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="26" t="inlineStr">
+        <is>
+          <t>Kultur und künstlerischer Ausdruck</t>
+        </is>
+      </c>
+      <c r="B118" s="39" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="C118" s="26" t="inlineStr">
+        <is>
+          <t>Bewegung gymnastisch, rhythmisch und tänzerisch gestalten</t>
+        </is>
+      </c>
+      <c r="D118" s="26" t="inlineStr">
+        <is>
+          <t>Bewegen mit und zur Musik</t>
+        </is>
+      </c>
+      <c r="E118" s="26" t="inlineStr">
+        <is>
+          <t>S. 22</t>
+        </is>
+      </c>
+      <c r="F118" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="26" t="inlineStr">
+        <is>
+          <t>Kultur und künstlerischer Ausdruck</t>
+        </is>
+      </c>
+      <c r="B119" s="34" t="inlineStr">
+        <is>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="C119" s="26" t="inlineStr">
+        <is>
+          <t>Lesarten und Rezeptionskonventionen</t>
+        </is>
+      </c>
+      <c r="D119" s="26" t="inlineStr">
+        <is>
+          <t>Lesarten und Rezeptionskonventionen</t>
+        </is>
+      </c>
+      <c r="E119" s="26" t="inlineStr">
+        <is>
+          <t>S. 25</t>
+        </is>
+      </c>
+      <c r="F119" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="26" t="inlineStr">
+        <is>
+          <t>Kultur und künstlerischer Ausdruck</t>
+        </is>
+      </c>
+      <c r="B120" s="32" t="inlineStr">
+        <is>
+          <t>Geschichte</t>
+        </is>
+      </c>
+      <c r="C120" s="26" t="inlineStr">
+        <is>
+          <t>Alltagskulturen</t>
+        </is>
+      </c>
+      <c r="D120" s="26" t="inlineStr">
+        <is>
+          <t>Rituale und Symbole</t>
+        </is>
+      </c>
+      <c r="E120" s="26" t="inlineStr">
+        <is>
+          <t>S. 22</t>
+        </is>
+      </c>
+      <c r="F120" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="26" t="inlineStr">
+        <is>
+          <t>Kultur und künstlerischer Ausdruck</t>
+        </is>
+      </c>
+      <c r="B121" s="36" t="inlineStr">
+        <is>
+          <t>Moderne Fremdsprachen</t>
+        </is>
+      </c>
+      <c r="C121" s="26" t="inlineStr">
+        <is>
+          <t>Kulturelle Lebenswelten „Ich und die Welt“</t>
+        </is>
+      </c>
+      <c r="D121" s="26" t="inlineStr">
+        <is>
+          <t>Kultur des Sprachraums</t>
+        </is>
+      </c>
+      <c r="E121" s="26" t="inlineStr">
+        <is>
+          <t>S. 29</t>
+        </is>
+      </c>
+      <c r="F121" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="26" t="inlineStr">
+        <is>
+          <t>Daten, Messen und Modelle</t>
+        </is>
+      </c>
+      <c r="B122" s="35" t="inlineStr">
+        <is>
+          <t>Mathematik</t>
+        </is>
+      </c>
+      <c r="C122" s="26" t="inlineStr">
+        <is>
+          <t>Statistische Erhebungen und ihre Auswertung</t>
+        </is>
+      </c>
+      <c r="D122" s="26" t="inlineStr">
+        <is>
+          <t>Statistische Erhebungen</t>
+        </is>
+      </c>
+      <c r="E122" s="26" t="inlineStr">
+        <is>
+          <t>S. 21</t>
+        </is>
+      </c>
+      <c r="F122" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="26" t="inlineStr">
+        <is>
+          <t>Daten, Messen und Modelle</t>
+        </is>
+      </c>
+      <c r="B123" s="35" t="inlineStr">
+        <is>
+          <t>Mathematik</t>
+        </is>
+      </c>
+      <c r="C123" s="26" t="inlineStr">
+        <is>
+          <t>Umgang mit dem Zufall</t>
+        </is>
+      </c>
+      <c r="D123" s="26" t="inlineStr">
+        <is>
+          <t>Zufall</t>
+        </is>
+      </c>
+      <c r="E123" s="26" t="inlineStr">
+        <is>
+          <t>S. 21</t>
+        </is>
+      </c>
+      <c r="F123" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="26" t="inlineStr">
+        <is>
+          <t>Daten, Messen und Modelle</t>
+        </is>
+      </c>
+      <c r="B124" s="35" t="inlineStr">
+        <is>
+          <t>Mathematik</t>
+        </is>
+      </c>
+      <c r="C124" s="26" t="inlineStr">
+        <is>
+          <t>Messvorgänge</t>
+        </is>
+      </c>
+      <c r="D124" s="26" t="inlineStr">
+        <is>
+          <t>Messvorgänge</t>
+        </is>
+      </c>
+      <c r="E124" s="26" t="inlineStr">
+        <is>
+          <t>S. 20</t>
+        </is>
+      </c>
+      <c r="F124" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="26" t="inlineStr">
+        <is>
+          <t>Daten, Messen und Modelle</t>
+        </is>
+      </c>
+      <c r="B125" s="43" t="inlineStr">
+        <is>
+          <t>Informatik</t>
+        </is>
+      </c>
+      <c r="C125" s="26" t="inlineStr">
+        <is>
+          <t>Grundlagen Datenbanken</t>
+        </is>
+      </c>
+      <c r="D125" s="26" t="inlineStr">
+        <is>
+          <t>Datenbanken</t>
+        </is>
+      </c>
+      <c r="E125" s="26" t="inlineStr">
+        <is>
+          <t>S. 20</t>
+        </is>
+      </c>
+      <c r="F125" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="26" t="inlineStr">
+        <is>
+          <t>Daten, Messen und Modelle</t>
+        </is>
+      </c>
+      <c r="B126" s="29" t="inlineStr">
+        <is>
+          <t>Physik</t>
+        </is>
+      </c>
+      <c r="C126" s="26" t="inlineStr">
+        <is>
+          <t>Haus der Naturwissenschaften</t>
+        </is>
+      </c>
+      <c r="D126" s="26" t="inlineStr">
+        <is>
+          <t>Physikalische Größen und ihre Messung</t>
+        </is>
+      </c>
+      <c r="E126" s="26" t="inlineStr">
+        <is>
+          <t>S. 29</t>
+        </is>
+      </c>
+      <c r="F126" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="26" t="inlineStr">
+        <is>
+          <t>Daten, Messen und Modelle</t>
+        </is>
+      </c>
+      <c r="B127" s="28" t="inlineStr">
+        <is>
+          <t>Chemie</t>
+        </is>
+      </c>
+      <c r="C127" s="26" t="inlineStr">
+        <is>
+          <t>Welt der Stoffe – Identifikation und Ordnung von Stoffen</t>
+        </is>
+      </c>
+      <c r="D127" s="26" t="inlineStr">
+        <is>
+          <t>Mess- und Nachweisverfahren</t>
+        </is>
+      </c>
+      <c r="E127" s="26" t="inlineStr">
+        <is>
+          <t>S. 29</t>
+        </is>
+      </c>
+      <c r="F127" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="26" t="inlineStr">
+        <is>
+          <t>Raum und Orientierung</t>
+        </is>
+      </c>
+      <c r="B128" s="30" t="inlineStr">
+        <is>
+          <t>Erdkunde</t>
+        </is>
+      </c>
+      <c r="C128" s="26" t="inlineStr">
+        <is>
+          <t>Räumliches Orientierungswissen</t>
+        </is>
+      </c>
+      <c r="D128" s="26" t="inlineStr">
+        <is>
+          <t>Orientierungsraster, Karten, Atlas</t>
+        </is>
+      </c>
+      <c r="E128" s="26" t="inlineStr">
+        <is>
+          <t>S. 26</t>
+        </is>
+      </c>
+      <c r="F128" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="26" t="inlineStr">
+        <is>
+          <t>Raum und Orientierung</t>
+        </is>
+      </c>
+      <c r="B129" s="30" t="inlineStr">
+        <is>
+          <t>Erdkunde</t>
+        </is>
+      </c>
+      <c r="C129" s="26" t="inlineStr">
+        <is>
+          <t>Erde als Planet</t>
+        </is>
+      </c>
+      <c r="D129" s="26" t="inlineStr">
+        <is>
+          <t>Erde als Planet</t>
+        </is>
+      </c>
+      <c r="E129" s="26" t="inlineStr">
+        <is>
+          <t>S. 26</t>
+        </is>
+      </c>
+      <c r="F129" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="26" t="inlineStr">
+        <is>
+          <t>Raum und Orientierung</t>
+        </is>
+      </c>
+      <c r="B130" s="35" t="inlineStr">
+        <is>
+          <t>Mathematik</t>
+        </is>
+      </c>
+      <c r="C130" s="26" t="inlineStr">
+        <is>
+          <t>Ebene Figuren</t>
+        </is>
+      </c>
+      <c r="D130" s="26" t="inlineStr">
+        <is>
+          <t>Kartesisches Koordinatensystem</t>
+        </is>
+      </c>
+      <c r="E130" s="26" t="inlineStr">
+        <is>
+          <t>S. 19</t>
+        </is>
+      </c>
+      <c r="F130" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="26" t="inlineStr">
+        <is>
+          <t>Raum und Orientierung</t>
+        </is>
+      </c>
+      <c r="B131" s="35" t="inlineStr">
+        <is>
+          <t>Mathematik</t>
+        </is>
+      </c>
+      <c r="C131" s="26" t="inlineStr">
+        <is>
+          <t>Körper</t>
+        </is>
+      </c>
+      <c r="D131" s="26" t="inlineStr">
+        <is>
+          <t>Körper aus Technik und Lebensumwelt</t>
+        </is>
+      </c>
+      <c r="E131" s="26" t="inlineStr">
+        <is>
+          <t>S. 19</t>
+        </is>
+      </c>
+      <c r="F131" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="26" t="inlineStr">
+        <is>
+          <t>Raum und Orientierung</t>
+        </is>
+      </c>
+      <c r="B132" s="32" t="inlineStr">
+        <is>
+          <t>Geschichte</t>
+        </is>
+      </c>
+      <c r="C132" s="26" t="inlineStr">
+        <is>
+          <t>Bewältigung und Nutzung von Räumen</t>
+        </is>
+      </c>
+      <c r="D132" s="26" t="inlineStr">
+        <is>
+          <t>Mensch-Raum-Beziehung</t>
+        </is>
+      </c>
+      <c r="E132" s="26" t="inlineStr">
+        <is>
+          <t>S. 24</t>
+        </is>
+      </c>
+      <c r="F132" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="26" t="inlineStr">
+        <is>
+          <t>Raum und Orientierung</t>
+        </is>
+      </c>
+      <c r="B133" s="29" t="inlineStr">
+        <is>
+          <t>Physik</t>
+        </is>
+      </c>
+      <c r="C133" s="26" t="inlineStr">
+        <is>
+          <t>Erweiterung der Sinne</t>
+        </is>
+      </c>
+      <c r="D133" s="26" t="inlineStr">
+        <is>
+          <t>Astronomische Phänomene: Sonne, Erde, Mond</t>
+        </is>
+      </c>
+      <c r="E133" s="26" t="inlineStr">
+        <is>
+          <t>S. 30</t>
+        </is>
+      </c>
+      <c r="F133" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="26" t="inlineStr">
+        <is>
+          <t>Körper und Bewegung</t>
+        </is>
+      </c>
+      <c r="B134" s="39" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="C134" s="26" t="inlineStr">
+        <is>
+          <t>Den Körper trainieren, die Fitness verbessern</t>
+        </is>
+      </c>
+      <c r="D134" s="26" t="inlineStr">
+        <is>
+          <t>Den Körper trainieren</t>
+        </is>
+      </c>
+      <c r="E134" s="26" t="inlineStr">
+        <is>
+          <t>S. 24</t>
+        </is>
+      </c>
+      <c r="F134" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="26" t="inlineStr">
+        <is>
+          <t>Körper und Bewegung</t>
+        </is>
+      </c>
+      <c r="B135" s="39" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="C135" s="26" t="inlineStr">
+        <is>
+          <t>Bewegen an und mit Geräten</t>
+        </is>
+      </c>
+      <c r="D135" s="26" t="inlineStr">
+        <is>
+          <t>Sichern und Helfen</t>
+        </is>
+      </c>
+      <c r="E135" s="26" t="inlineStr">
+        <is>
+          <t>S. 21</t>
+        </is>
+      </c>
+      <c r="F135" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="26" t="inlineStr">
+        <is>
+          <t>Körper und Bewegung</t>
+        </is>
+      </c>
+      <c r="B136" s="27" t="inlineStr">
+        <is>
+          <t>Biologie</t>
+        </is>
+      </c>
+      <c r="C136" s="26" t="inlineStr">
+        <is>
+          <t>Biologische Strukturen und ihre Funktion</t>
+        </is>
+      </c>
+      <c r="D136" s="26" t="inlineStr">
+        <is>
+          <t>Gegenspielerprinzip am Beispiel der Skelettmuskulatur</t>
+        </is>
+      </c>
+      <c r="E136" s="26" t="inlineStr">
+        <is>
+          <t>S. 41</t>
+        </is>
+      </c>
+      <c r="F136" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="26" t="inlineStr">
+        <is>
+          <t>Körper und Bewegung</t>
+        </is>
+      </c>
+      <c r="B137" s="27" t="inlineStr">
+        <is>
+          <t>Biologie</t>
+        </is>
+      </c>
+      <c r="C137" s="26" t="inlineStr">
+        <is>
+          <t>Vielfalt, Veränderung und Abstammung von Lebewesen</t>
+        </is>
+      </c>
+      <c r="D137" s="26" t="inlineStr">
+        <is>
+          <t>Muskelaufbau durch Krafttraining</t>
+        </is>
+      </c>
+      <c r="E137" s="26" t="inlineStr">
+        <is>
+          <t>S. 47</t>
+        </is>
+      </c>
+      <c r="F137" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="26" t="inlineStr">
+        <is>
+          <t>Körper und Bewegung</t>
+        </is>
+      </c>
+      <c r="B138" s="29" t="inlineStr">
+        <is>
+          <t>Physik</t>
+        </is>
+      </c>
+      <c r="C138" s="26" t="inlineStr">
+        <is>
+          <t>Fortbewegung und Mobilität</t>
+        </is>
+      </c>
+      <c r="D138" s="26" t="inlineStr">
+        <is>
+          <t>Wirkungen von Kräften</t>
+        </is>
+      </c>
+      <c r="E138" s="26" t="inlineStr">
+        <is>
+          <t>S. 34</t>
+        </is>
+      </c>
+      <c r="F138" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="26" t="inlineStr">
+        <is>
+          <t>Körper und Bewegung</t>
+        </is>
+      </c>
+      <c r="B139" s="38" t="inlineStr">
+        <is>
+          <t>Musik</t>
+        </is>
+      </c>
+      <c r="C139" s="26" t="inlineStr">
+        <is>
+          <t>Bewegung und Gestaltungsmedien</t>
+        </is>
+      </c>
+      <c r="D139" s="26" t="inlineStr">
+        <is>
+          <t>Bewegung zur Musik</t>
+        </is>
+      </c>
+      <c r="E139" s="26" t="inlineStr">
+        <is>
+          <t>S. 18</t>
+        </is>
+      </c>
+      <c r="F139" s="26" t="inlineStr">
+        <is>
+          <t>Vorschlag, fachlich zu prüfen</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F48"/>
+  <autoFilter ref="A1:F139"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
SDG-Unterziele und SDG-Verbindungen bei Themen und Fächern
- bne_unterziele.csv: 63 schulrelevante Unterziele im amtlichen deutschen Wortlaut (Destatis, sdg-indikatoren.de)
- bne_sdg.csv mit amtlichem Zieltext, bne_vorschlaege.csv mit Unterziel je Zuordnung
- Seite: Themen und Fächer zeigen die Ziele ihrer Inhaltsfelder (Liste und Linien), SDG-Ansicht mit Zieltext und aufklappbaren Unterzielen, Unterziel 4.7 beim BNE-Knoten
- Klick auf ein Ziel schaltet die BNE-Ebene ein (vorher toter Klick)
- Excel-Blatt SDG-Unterziele, Prüfliste mit Unterziel

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/Kerncurricula_Hessen_Sek1.xlsx
+++ b/output/Kerncurricula_Hessen_Sek1.xlsx
@@ -15,7 +15,8 @@
     <sheet name="Anknüpfungspunkte" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="BNE Belege" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="SDG-Vorschläge" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Hinweise und Lücken" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="SDG-Unterziele" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Hinweise und Lücken" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Inhaltsfelder'!$A$1:$H$130</definedName>
@@ -24,8 +25,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Querbezüge belegt'!$A$1:$D$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Anknüpfungspunkte'!$A$1:$F$139</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'BNE Belege'!$A$1:$F$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'SDG-Vorschläge'!$A$1:$F$65</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Hinweise und Lücken'!$A$1:$B$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'SDG-Vorschläge'!$A$1:$G$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'SDG-Unterziele'!$A$1:$E$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Hinweise und Lücken'!$A$1:$B$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -642,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -730,7 +732,7 @@
         <v/>
       </c>
       <c r="E5" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A5)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A5)</f>
         <v/>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -768,7 +770,7 @@
         <v/>
       </c>
       <c r="E6" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A6)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A6)</f>
         <v/>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -806,7 +808,7 @@
         <v/>
       </c>
       <c r="E7" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A7)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A7)</f>
         <v/>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -844,7 +846,7 @@
         <v/>
       </c>
       <c r="E8" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A8)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A8)</f>
         <v/>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -882,7 +884,7 @@
         <v/>
       </c>
       <c r="E9" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A9)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A9)</f>
         <v/>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -920,7 +922,7 @@
         <v/>
       </c>
       <c r="E10" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A10)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A10)</f>
         <v/>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -958,7 +960,7 @@
         <v/>
       </c>
       <c r="E11" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A11)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A11)</f>
         <v/>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -986,7 +988,7 @@
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A12)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A12)</f>
         <v/>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -1024,7 +1026,7 @@
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A13)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A13)</f>
         <v/>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1062,7 +1064,7 @@
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A14)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A14)</f>
         <v/>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -1100,7 +1102,7 @@
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A15)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A15)</f>
         <v/>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1138,7 +1140,7 @@
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A16)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A16)</f>
         <v/>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1176,7 +1178,7 @@
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A17)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A17)</f>
         <v/>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1214,7 +1216,7 @@
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A18)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A18)</f>
         <v/>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1247,7 +1249,7 @@
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A19)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A19)</f>
         <v/>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1285,7 +1287,7 @@
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A20)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A20)</f>
         <v/>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1323,7 +1325,7 @@
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIF('SDG-Vorschläge'!C:C,A21)</f>
+        <f>COUNTIF('SDG-Vorschläge'!D:D,A21)</f>
         <v/>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1452,17 +1454,29 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Zuordnung von Inhaltsfeldern zu den 17 Nachhaltigkeitszielen, zu prüfen</t>
+          <t>Zuordnung von Inhaltsfeldern zu den 17 Nachhaltigkeitszielen und ihren Unterzielen, zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="23" t="inlineStr">
         <is>
+          <t>SDG-Unterziele</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Ausgewählte Unterziele mit Schulbezug im amtlichen deutschen Wortlaut</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="23" t="inlineStr">
+        <is>
           <t>Hinweise und Lücken</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>Was fehlt oder abweicht</t>
         </is>
@@ -1523,6 +1537,205 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>Punkt</t>
+        </is>
+      </c>
+      <c r="B1" s="25" t="inlineStr">
+        <is>
+          <t>Hinweis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>Bildungsgang</t>
+        </is>
+      </c>
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>Inhaltsfelder sind für 17 Fächer in allen drei KC-Fassungen erfasst (Hauptschule, Realschule, Gymnasium). Schwerpunkte gibt es für alle Fächer (teils automatisch ausgelesen, siehe Spalte Hinweis); Kompetenzbereiche nur Pilotfächer in der Gymnasialfassung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="26" t="inlineStr">
+        <is>
+          <t>Haupt- und Realschule</t>
+        </is>
+      </c>
+      <c r="B3" s="26" t="inlineStr">
+        <is>
+          <t>Biologie, Chemie, Physik: Übersichtstabelle Kap. 7.3 bzw. 7.2, Stufen bis Jg. 5/6 bzw. 1. Lernjahr bzw. Hälfte des Stundenkontingents und zusätzlich bis Abschluss Jg. 9 (HS) oder 10 (RS). Erdkunde: Kap. 7.1 (Ende Jg. 6), Kap. 7.2 entfällt laut KC. PoWi: Kap. 7 entfällt laut KC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>Fächerauswahl</t>
+        </is>
+      </c>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>Aufgenommen sind die Fächer einer IGS 5 bis 10. Latein, Griechisch, Chinesisch, Arabisch sowie alevitische, jüdische und islamische Religion fehlen noch. Informatik gibt es nur als KC für den Wahlunterricht am Gymnasium.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>Moderne Fremdsprachen</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>Ein gemeinsames KC für alle modernen Fremdsprachen. Die Inhaltsfelder sind drei Lebenswelten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>Kunst</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>Die Zuordnung der neun Inhaltsfelder zu den drei Kernbereichen steht nur in Abb. 2 (Kap. 5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>Evangelische und Katholische Religion liegen in der neuen KC-Fassung von 2026 vor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>BNE ist nach § 6 Abs. 4 HSchG ein Aufgabengebiet. Die KC von 2011 nennen BNE nicht ausdrücklich. Als Beleg zählt nur, wo das KC selbst Nachhaltigkeit nennt (Blatt 'BNE Belege'). Die SDG-Zuordnung ist ein Vorschlag.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>Stufung</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Die Stufen sind nicht einheitlich: Biologie 'bis Ende 5/6', Chemie '1. Lernjahr', Physik 'nach ca. der Hälfte des Stundenkontingents', jeweils plus 'bis Ende 9/10'. Erdkunde und Politik und Wirtschaft haben im Gymnasium-KC keine Stufung. Die Zuordnung zu Jahrgängen hängt an der Stundentafel bzw. am Schulcurriculum.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>Jahrgang 8</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Biologie, Chemie, Physik, Erdkunde und PoWi weisen für das Gymnasium ausdrücklich keine Kompetenzerwartungen für Jahrgang 6/8 bzw. 8 aus (jeweils Kap. 7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>Erdkunde, PoWi</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>Die Einträge im Blatt 'Schwerpunkte' sind Stichworte aus den Inhaltsfeldbeschreibungen (Kap. 6), da es keine Schwerpunkt-Tabelle gibt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>PoWi</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Im PDF ist der rechte Teil der quer gesetzten Tabellen beim Auslesen abgeschnitten. Stichworte bitte am Original prüfen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>Grafiken</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>Abbildungen (z. B. Basiskonzept-Zuordnung Physik, Verzahnung Erdkunde/PoWi/Geschichte) ließen sich nicht als Text auslesen und fehlen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>Wortlaut</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Schwerpunkte sind teils gekürzt oder zusammengefasst. Für verbindliche Formulierungen gilt das Original (Seitenangabe je Zeile).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>Anknüpfungspunkte</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>Das Blatt 'Anknüpfungspunkte' enthält Vorschläge auf Basis gemeinsamer Stichworte. Sie stehen so nicht im KC und sind fachlich zu prüfen.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B15"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -72857,15 +73070,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -72881,20 +73095,25 @@
       </c>
       <c r="C1" s="25" t="inlineStr">
         <is>
+          <t>Unterziel</t>
+        </is>
+      </c>
+      <c r="D1" s="25" t="inlineStr">
+        <is>
           <t>Fach</t>
         </is>
       </c>
-      <c r="D1" s="25" t="inlineStr">
+      <c r="E1" s="25" t="inlineStr">
         <is>
           <t>Inhaltsfeld</t>
         </is>
       </c>
-      <c r="E1" s="25" t="inlineStr">
+      <c r="F1" s="25" t="inlineStr">
         <is>
           <t>Stichwort</t>
         </is>
       </c>
-      <c r="F1" s="25" t="inlineStr">
+      <c r="G1" s="25" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -72909,22 +73128,27 @@
           <t>Keine Armut</t>
         </is>
       </c>
-      <c r="C2" s="31" t="inlineStr">
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="D2" s="31" t="inlineStr">
         <is>
           <t>Politik und Wirtschaft</t>
         </is>
       </c>
-      <c r="D2" s="26" t="inlineStr">
+      <c r="E2" s="26" t="inlineStr">
         <is>
           <t>Wirtschaft</t>
         </is>
       </c>
-      <c r="E2" s="26" t="inlineStr">
+      <c r="F2" s="26" t="inlineStr">
         <is>
           <t>Einkommen und Verteilung</t>
         </is>
       </c>
-      <c r="F2" s="26" t="inlineStr">
+      <c r="G2" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -72939,22 +73163,27 @@
           <t>Keine Armut</t>
         </is>
       </c>
-      <c r="C3" s="31" t="inlineStr">
+      <c r="C3" s="26" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="D3" s="31" t="inlineStr">
         <is>
           <t>Politik und Wirtschaft</t>
         </is>
       </c>
-      <c r="D3" s="26" t="inlineStr">
+      <c r="E3" s="26" t="inlineStr">
         <is>
           <t>Internationale Beziehungen und Globalisierung</t>
         </is>
       </c>
-      <c r="E3" s="26" t="inlineStr">
+      <c r="F3" s="26" t="inlineStr">
         <is>
           <t>Globale Entwicklungsunterschiede</t>
         </is>
       </c>
-      <c r="F3" s="26" t="inlineStr">
+      <c r="G3" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -72969,22 +73198,27 @@
           <t>Keine Armut</t>
         </is>
       </c>
-      <c r="C4" s="30" t="inlineStr">
+      <c r="C4" s="26" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="D4" s="30" t="inlineStr">
         <is>
           <t>Erdkunde</t>
         </is>
       </c>
-      <c r="D4" s="26" t="inlineStr">
+      <c r="E4" s="26" t="inlineStr">
         <is>
           <t>Mensch/Gesellschaft</t>
         </is>
       </c>
-      <c r="E4" s="26" t="inlineStr">
+      <c r="F4" s="26" t="inlineStr">
         <is>
           <t>Lebensbedingungen in verschiedenen Räumen</t>
         </is>
       </c>
-      <c r="F4" s="26" t="inlineStr">
+      <c r="G4" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -72999,22 +73233,27 @@
           <t>Keine Armut</t>
         </is>
       </c>
-      <c r="C5" s="32" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="D5" s="32" t="inlineStr">
         <is>
           <t>Geschichte</t>
         </is>
       </c>
-      <c r="D5" s="26" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>Epochenbezug Neuzeit</t>
         </is>
       </c>
-      <c r="E5" s="26" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
         <is>
           <t>Industrielle Revolutionen und Soziale Frage</t>
         </is>
       </c>
-      <c r="F5" s="26" t="inlineStr">
+      <c r="G5" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73029,22 +73268,27 @@
           <t>Keine Armut</t>
         </is>
       </c>
-      <c r="C6" s="33" t="inlineStr">
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="D6" s="33" t="inlineStr">
         <is>
           <t>Arbeitslehre</t>
         </is>
       </c>
-      <c r="D6" s="26" t="inlineStr">
+      <c r="E6" s="26" t="inlineStr">
         <is>
           <t>Ökonomisch geprägte Situationen und Strukturen des Zusammenlebens</t>
         </is>
       </c>
-      <c r="E6" s="26" t="inlineStr">
+      <c r="F6" s="26" t="inlineStr">
         <is>
           <t>Einkommen und soziale Sicherung</t>
         </is>
       </c>
-      <c r="F6" s="26" t="inlineStr">
+      <c r="G6" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73059,22 +73303,27 @@
           <t>Kein Hunger</t>
         </is>
       </c>
-      <c r="C7" s="27" t="inlineStr">
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="inlineStr">
         <is>
           <t>Biologie</t>
         </is>
       </c>
-      <c r="D7" s="26" t="inlineStr">
+      <c r="E7" s="26" t="inlineStr">
         <is>
           <t>Stoffwechsel und Regelmechanismen</t>
         </is>
       </c>
-      <c r="E7" s="26" t="inlineStr">
+      <c r="F7" s="26" t="inlineStr">
         <is>
           <t>Ausgewogene Ernährung</t>
         </is>
       </c>
-      <c r="F7" s="26" t="inlineStr">
+      <c r="G7" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73089,22 +73338,27 @@
           <t>Kein Hunger</t>
         </is>
       </c>
-      <c r="C8" s="30" t="inlineStr">
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="D8" s="30" t="inlineStr">
         <is>
           <t>Erdkunde</t>
         </is>
       </c>
-      <c r="D8" s="26" t="inlineStr">
+      <c r="E8" s="26" t="inlineStr">
         <is>
           <t>Umwelt-Gesellschaft-Beziehungen und globale Probleme</t>
         </is>
       </c>
-      <c r="E8" s="26" t="inlineStr">
+      <c r="F8" s="26" t="inlineStr">
         <is>
           <t>Ressourcensicherung</t>
         </is>
       </c>
-      <c r="F8" s="26" t="inlineStr">
+      <c r="G8" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73119,22 +73373,27 @@
           <t>Gesundheit und Wohlergehen</t>
         </is>
       </c>
-      <c r="C9" s="27" t="inlineStr">
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
         <is>
           <t>Biologie</t>
         </is>
       </c>
-      <c r="D9" s="26" t="inlineStr">
+      <c r="E9" s="26" t="inlineStr">
         <is>
           <t>Funktionsteilung im Organismus</t>
         </is>
       </c>
-      <c r="E9" s="26" t="inlineStr">
+      <c r="F9" s="26" t="inlineStr">
         <is>
           <t>Immunsystem und Infektionskrankheiten</t>
         </is>
       </c>
-      <c r="F9" s="26" t="inlineStr">
+      <c r="G9" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73149,22 +73408,27 @@
           <t>Gesundheit und Wohlergehen</t>
         </is>
       </c>
-      <c r="C10" s="27" t="inlineStr">
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
         <is>
           <t>Biologie</t>
         </is>
       </c>
-      <c r="D10" s="26" t="inlineStr">
+      <c r="E10" s="26" t="inlineStr">
         <is>
           <t>Sexualität des Menschen</t>
         </is>
       </c>
-      <c r="E10" s="26" t="inlineStr">
+      <c r="F10" s="26" t="inlineStr">
         <is>
           <t>Gesundheitserziehung</t>
         </is>
       </c>
-      <c r="F10" s="26" t="inlineStr">
+      <c r="G10" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73179,22 +73443,27 @@
           <t>Gesundheit und Wohlergehen</t>
         </is>
       </c>
-      <c r="C11" s="39" t="inlineStr">
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="D11" s="39" t="inlineStr">
         <is>
           <t>Sport</t>
         </is>
       </c>
-      <c r="D11" s="26" t="inlineStr">
+      <c r="E11" s="26" t="inlineStr">
         <is>
           <t>Den Körper trainieren, die Fitness verbessern</t>
         </is>
       </c>
-      <c r="E11" s="26" t="inlineStr">
+      <c r="F11" s="26" t="inlineStr">
         <is>
           <t>Fitness und Gesundheit</t>
         </is>
       </c>
-      <c r="F11" s="26" t="inlineStr">
+      <c r="G11" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73209,22 +73478,27 @@
           <t>Gesundheit und Wohlergehen</t>
         </is>
       </c>
-      <c r="C12" s="33" t="inlineStr">
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="D12" s="33" t="inlineStr">
         <is>
           <t>Arbeitslehre</t>
         </is>
       </c>
-      <c r="D12" s="26" t="inlineStr">
+      <c r="E12" s="26" t="inlineStr">
         <is>
           <t>Erhalt der psychischen und physischen Gesundheit</t>
         </is>
       </c>
-      <c r="E12" s="26" t="inlineStr">
+      <c r="F12" s="26" t="inlineStr">
         <is>
           <t>Gesundheit im Arbeitsleben</t>
         </is>
       </c>
-      <c r="F12" s="26" t="inlineStr">
+      <c r="G12" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73239,22 +73513,27 @@
           <t>Hochwertige Bildung</t>
         </is>
       </c>
-      <c r="C13" s="33" t="inlineStr">
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="D13" s="33" t="inlineStr">
         <is>
           <t>Arbeitslehre</t>
         </is>
       </c>
-      <c r="D13" s="26" t="inlineStr">
+      <c r="E13" s="26" t="inlineStr">
         <is>
           <t>Berufswegeplanung</t>
         </is>
       </c>
-      <c r="E13" s="26" t="inlineStr">
+      <c r="F13" s="26" t="inlineStr">
         <is>
           <t>Bildungs- und Berufswege</t>
         </is>
       </c>
-      <c r="F13" s="26" t="inlineStr">
+      <c r="G13" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73269,22 +73548,27 @@
           <t>Geschlechtergleichheit</t>
         </is>
       </c>
-      <c r="C14" s="27" t="inlineStr">
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
         <is>
           <t>Biologie</t>
         </is>
       </c>
-      <c r="D14" s="26" t="inlineStr">
+      <c r="E14" s="26" t="inlineStr">
         <is>
           <t>Sexualität des Menschen</t>
         </is>
       </c>
-      <c r="E14" s="26" t="inlineStr">
+      <c r="F14" s="26" t="inlineStr">
         <is>
           <t>Geschlechterrollen</t>
         </is>
       </c>
-      <c r="F14" s="26" t="inlineStr">
+      <c r="G14" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73299,22 +73583,27 @@
           <t>Geschlechtergleichheit</t>
         </is>
       </c>
-      <c r="C15" s="31" t="inlineStr">
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
+      <c r="D15" s="31" t="inlineStr">
         <is>
           <t>Politik und Wirtschaft</t>
         </is>
       </c>
-      <c r="D15" s="26" t="inlineStr">
+      <c r="E15" s="26" t="inlineStr">
         <is>
           <t>Individuum und Gesellschaft</t>
         </is>
       </c>
-      <c r="E15" s="26" t="inlineStr">
+      <c r="F15" s="26" t="inlineStr">
         <is>
           <t>Gleichberechtigung</t>
         </is>
       </c>
-      <c r="F15" s="26" t="inlineStr">
+      <c r="G15" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73329,22 +73618,27 @@
           <t>Geschlechtergleichheit</t>
         </is>
       </c>
-      <c r="C16" s="40" t="inlineStr">
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="D16" s="40" t="inlineStr">
         <is>
           <t>Ethik</t>
         </is>
       </c>
-      <c r="D16" s="26" t="inlineStr">
+      <c r="E16" s="26" t="inlineStr">
         <is>
           <t>Freiheit und Würde</t>
         </is>
       </c>
-      <c r="E16" s="26" t="inlineStr">
+      <c r="F16" s="26" t="inlineStr">
         <is>
           <t>Würde unabhängig von Herkunft, Geschlecht, Alter</t>
         </is>
       </c>
-      <c r="F16" s="26" t="inlineStr">
+      <c r="G16" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73359,22 +73653,27 @@
           <t>Geschlechtergleichheit</t>
         </is>
       </c>
-      <c r="C17" s="32" t="inlineStr">
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="D17" s="32" t="inlineStr">
         <is>
           <t>Geschichte</t>
         </is>
       </c>
-      <c r="D17" s="26" t="inlineStr">
+      <c r="E17" s="26" t="inlineStr">
         <is>
           <t>Alltagskulturen</t>
         </is>
       </c>
-      <c r="E17" s="26" t="inlineStr">
+      <c r="F17" s="26" t="inlineStr">
         <is>
           <t>Geschlecht und Sexualität im Wandel</t>
         </is>
       </c>
-      <c r="F17" s="26" t="inlineStr">
+      <c r="G17" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73389,22 +73688,27 @@
           <t>Sauberes Wasser und Sanitäreinrichtungen</t>
         </is>
       </c>
-      <c r="C18" s="28" t="inlineStr">
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="D18" s="28" t="inlineStr">
         <is>
           <t>Chemie</t>
         </is>
       </c>
-      <c r="D18" s="26" t="inlineStr">
+      <c r="E18" s="26" t="inlineStr">
         <is>
           <t>Welt der Stoffe – Identifikation und Ordnung von Stoffen</t>
         </is>
       </c>
-      <c r="E18" s="26" t="inlineStr">
+      <c r="F18" s="26" t="inlineStr">
         <is>
           <t>Luft und Wasser</t>
         </is>
       </c>
-      <c r="F18" s="26" t="inlineStr">
+      <c r="G18" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73419,22 +73723,27 @@
           <t>Sauberes Wasser und Sanitäreinrichtungen</t>
         </is>
       </c>
-      <c r="C19" s="28" t="inlineStr">
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="D19" s="28" t="inlineStr">
         <is>
           <t>Chemie</t>
         </is>
       </c>
-      <c r="D19" s="26" t="inlineStr">
+      <c r="E19" s="26" t="inlineStr">
         <is>
           <t>Schatzkiste der Natur – Chemie in Alltag und Technik</t>
         </is>
       </c>
-      <c r="E19" s="26" t="inlineStr">
+      <c r="F19" s="26" t="inlineStr">
         <is>
           <t>Luft, Wasser, Boden</t>
         </is>
       </c>
-      <c r="F19" s="26" t="inlineStr">
+      <c r="G19" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73449,22 +73758,27 @@
           <t>Sauberes Wasser und Sanitäreinrichtungen</t>
         </is>
       </c>
-      <c r="C20" s="30" t="inlineStr">
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>6.6</t>
+        </is>
+      </c>
+      <c r="D20" s="30" t="inlineStr">
         <is>
           <t>Erdkunde</t>
         </is>
       </c>
-      <c r="D20" s="26" t="inlineStr">
+      <c r="E20" s="26" t="inlineStr">
         <is>
           <t>Natur/Umwelt</t>
         </is>
       </c>
-      <c r="E20" s="26" t="inlineStr">
+      <c r="F20" s="26" t="inlineStr">
         <is>
           <t>Wasser als Naturfaktor</t>
         </is>
       </c>
-      <c r="F20" s="26" t="inlineStr">
+      <c r="G20" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73479,22 +73793,27 @@
           <t>Bezahlbare und saubere Energie</t>
         </is>
       </c>
-      <c r="C21" s="29" t="inlineStr">
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="D21" s="29" t="inlineStr">
         <is>
           <t>Physik</t>
         </is>
       </c>
-      <c r="D21" s="26" t="inlineStr">
+      <c r="E21" s="26" t="inlineStr">
         <is>
           <t>Energie in Umwelt und Technik</t>
         </is>
       </c>
-      <c r="E21" s="26" t="inlineStr">
+      <c r="F21" s="26" t="inlineStr">
         <is>
           <t>Energieformen und Energieumwandlung</t>
         </is>
       </c>
-      <c r="F21" s="26" t="inlineStr">
+      <c r="G21" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73509,22 +73828,27 @@
           <t>Bezahlbare und saubere Energie</t>
         </is>
       </c>
-      <c r="C22" s="29" t="inlineStr">
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="D22" s="29" t="inlineStr">
         <is>
           <t>Physik</t>
         </is>
       </c>
-      <c r="D22" s="26" t="inlineStr">
+      <c r="E22" s="26" t="inlineStr">
         <is>
           <t>Zukunftssichere Energieversorgung</t>
         </is>
       </c>
-      <c r="E22" s="26" t="inlineStr">
+      <c r="F22" s="26" t="inlineStr">
         <is>
           <t>Regenerative und erschöpfbare Energien</t>
         </is>
       </c>
-      <c r="F22" s="26" t="inlineStr">
+      <c r="G22" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73539,22 +73863,27 @@
           <t>Bezahlbare und saubere Energie</t>
         </is>
       </c>
-      <c r="C23" s="28" t="inlineStr">
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="D23" s="28" t="inlineStr">
         <is>
           <t>Chemie</t>
         </is>
       </c>
-      <c r="D23" s="26" t="inlineStr">
+      <c r="E23" s="26" t="inlineStr">
         <is>
           <t>Verwandlungen – Chemische Reaktion</t>
         </is>
       </c>
-      <c r="E23" s="26" t="inlineStr">
+      <c r="F23" s="26" t="inlineStr">
         <is>
           <t>Energieumsatz bei Reaktionen</t>
         </is>
       </c>
-      <c r="F23" s="26" t="inlineStr">
+      <c r="G23" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73569,22 +73898,27 @@
           <t>Bezahlbare und saubere Energie</t>
         </is>
       </c>
-      <c r="C24" s="28" t="inlineStr">
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="D24" s="28" t="inlineStr">
         <is>
           <t>Chemie</t>
         </is>
       </c>
-      <c r="D24" s="26" t="inlineStr">
+      <c r="E24" s="26" t="inlineStr">
         <is>
           <t>Magie des Kohlenstoffs – Organische Verbindungen</t>
         </is>
       </c>
-      <c r="E24" s="26" t="inlineStr">
+      <c r="F24" s="26" t="inlineStr">
         <is>
           <t>Energieträger</t>
         </is>
       </c>
-      <c r="F24" s="26" t="inlineStr">
+      <c r="G24" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73599,22 +73933,27 @@
           <t>Menschenwürdige Arbeit und Wirtschaftswachstum</t>
         </is>
       </c>
-      <c r="C25" s="33" t="inlineStr">
+      <c r="C25" s="26" t="inlineStr">
+        <is>
+          <t>8.8</t>
+        </is>
+      </c>
+      <c r="D25" s="33" t="inlineStr">
         <is>
           <t>Arbeitslehre</t>
         </is>
       </c>
-      <c r="D25" s="26" t="inlineStr">
+      <c r="E25" s="26" t="inlineStr">
         <is>
           <t>Organisation von Arbeit</t>
         </is>
       </c>
-      <c r="E25" s="26" t="inlineStr">
+      <c r="F25" s="26" t="inlineStr">
         <is>
           <t>Menschenwürdige Arbeitsbedingungen</t>
         </is>
       </c>
-      <c r="F25" s="26" t="inlineStr">
+      <c r="G25" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73629,22 +73968,27 @@
           <t>Menschenwürdige Arbeit und Wirtschaftswachstum</t>
         </is>
       </c>
-      <c r="C26" s="33" t="inlineStr">
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D26" s="33" t="inlineStr">
         <is>
           <t>Arbeitslehre</t>
         </is>
       </c>
-      <c r="D26" s="26" t="inlineStr">
+      <c r="E26" s="26" t="inlineStr">
         <is>
           <t>Zukunft der Arbeit</t>
         </is>
       </c>
-      <c r="E26" s="26" t="inlineStr">
+      <c r="F26" s="26" t="inlineStr">
         <is>
           <t>Zukunft der Erwerbsarbeit</t>
         </is>
       </c>
-      <c r="F26" s="26" t="inlineStr">
+      <c r="G26" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73659,22 +74003,27 @@
           <t>Menschenwürdige Arbeit und Wirtschaftswachstum</t>
         </is>
       </c>
-      <c r="C27" s="31" t="inlineStr">
+      <c r="C27" s="26" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D27" s="31" t="inlineStr">
         <is>
           <t>Politik und Wirtschaft</t>
         </is>
       </c>
-      <c r="D27" s="26" t="inlineStr">
+      <c r="E27" s="26" t="inlineStr">
         <is>
           <t>Wirtschaft</t>
         </is>
       </c>
-      <c r="E27" s="26" t="inlineStr">
+      <c r="F27" s="26" t="inlineStr">
         <is>
           <t>Wirtschaftsordnung und Arbeit</t>
         </is>
       </c>
-      <c r="F27" s="26" t="inlineStr">
+      <c r="G27" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73689,22 +74038,27 @@
           <t>Menschenwürdige Arbeit und Wirtschaftswachstum</t>
         </is>
       </c>
-      <c r="C28" s="32" t="inlineStr">
+      <c r="C28" s="26" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D28" s="32" t="inlineStr">
         <is>
           <t>Geschichte</t>
         </is>
       </c>
-      <c r="D28" s="26" t="inlineStr">
+      <c r="E28" s="26" t="inlineStr">
         <is>
           <t>Wirtschaft</t>
         </is>
       </c>
-      <c r="E28" s="26" t="inlineStr">
+      <c r="F28" s="26" t="inlineStr">
         <is>
           <t>Wandel von Arbeit und Wirtschaft</t>
         </is>
       </c>
-      <c r="F28" s="26" t="inlineStr">
+      <c r="G28" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73719,22 +74073,27 @@
           <t>Industrie, Innovation und Infrastruktur</t>
         </is>
       </c>
-      <c r="C29" s="29" t="inlineStr">
+      <c r="C29" s="26" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="D29" s="29" t="inlineStr">
         <is>
           <t>Physik</t>
         </is>
       </c>
-      <c r="D29" s="26" t="inlineStr">
+      <c r="E29" s="26" t="inlineStr">
         <is>
           <t>Technik im Dienst des Menschen</t>
         </is>
       </c>
-      <c r="E29" s="26" t="inlineStr">
+      <c r="F29" s="26" t="inlineStr">
         <is>
           <t>Technik und Innovation</t>
         </is>
       </c>
-      <c r="F29" s="26" t="inlineStr">
+      <c r="G29" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73749,22 +74108,27 @@
           <t>Industrie, Innovation und Infrastruktur</t>
         </is>
       </c>
-      <c r="C30" s="33" t="inlineStr">
+      <c r="C30" s="26" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="D30" s="33" t="inlineStr">
         <is>
           <t>Arbeitslehre</t>
         </is>
       </c>
-      <c r="D30" s="26" t="inlineStr">
+      <c r="E30" s="26" t="inlineStr">
         <is>
           <t>Technische Systeme und Prozesse</t>
         </is>
       </c>
-      <c r="E30" s="26" t="inlineStr">
+      <c r="F30" s="26" t="inlineStr">
         <is>
           <t>Technische Systeme</t>
         </is>
       </c>
-      <c r="F30" s="26" t="inlineStr">
+      <c r="G30" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73779,22 +74143,27 @@
           <t>Industrie, Innovation und Infrastruktur</t>
         </is>
       </c>
-      <c r="C31" s="43" t="inlineStr">
+      <c r="C31" s="26" t="inlineStr">
+        <is>
+          <t>9.c</t>
+        </is>
+      </c>
+      <c r="D31" s="43" t="inlineStr">
         <is>
           <t>Informatik</t>
         </is>
       </c>
-      <c r="D31" s="26" t="inlineStr">
+      <c r="E31" s="26" t="inlineStr">
         <is>
           <t>Hardware und Rechnerarchitektur</t>
         </is>
       </c>
-      <c r="E31" s="26" t="inlineStr">
+      <c r="F31" s="26" t="inlineStr">
         <is>
           <t>Digitale Infrastruktur</t>
         </is>
       </c>
-      <c r="F31" s="26" t="inlineStr">
+      <c r="G31" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73809,22 +74178,27 @@
           <t>Industrie, Innovation und Infrastruktur</t>
         </is>
       </c>
-      <c r="C32" s="43" t="inlineStr">
+      <c r="C32" s="26" t="inlineStr">
+        <is>
+          <t>9.c</t>
+        </is>
+      </c>
+      <c r="D32" s="43" t="inlineStr">
         <is>
           <t>Informatik</t>
         </is>
       </c>
-      <c r="D32" s="26" t="inlineStr">
+      <c r="E32" s="26" t="inlineStr">
         <is>
           <t>Internet und HTML</t>
         </is>
       </c>
-      <c r="E32" s="26" t="inlineStr">
+      <c r="F32" s="26" t="inlineStr">
         <is>
           <t>Digitale Infrastruktur</t>
         </is>
       </c>
-      <c r="F32" s="26" t="inlineStr">
+      <c r="G32" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73839,22 +74213,27 @@
           <t>Weniger Ungleichheiten</t>
         </is>
       </c>
-      <c r="C33" s="31" t="inlineStr">
+      <c r="C33" s="26" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="D33" s="31" t="inlineStr">
         <is>
           <t>Politik und Wirtschaft</t>
         </is>
       </c>
-      <c r="D33" s="26" t="inlineStr">
+      <c r="E33" s="26" t="inlineStr">
         <is>
           <t>Individuum und Gesellschaft</t>
         </is>
       </c>
-      <c r="E33" s="26" t="inlineStr">
+      <c r="F33" s="26" t="inlineStr">
         <is>
           <t>Soziale Ungleichheit</t>
         </is>
       </c>
-      <c r="F33" s="26" t="inlineStr">
+      <c r="G33" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73869,22 +74248,27 @@
           <t>Weniger Ungleichheiten</t>
         </is>
       </c>
-      <c r="C34" s="40" t="inlineStr">
+      <c r="C34" s="26" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="D34" s="40" t="inlineStr">
         <is>
           <t>Ethik</t>
         </is>
       </c>
-      <c r="D34" s="26" t="inlineStr">
+      <c r="E34" s="26" t="inlineStr">
         <is>
           <t>Recht und Gerechtigkeit</t>
         </is>
       </c>
-      <c r="E34" s="26" t="inlineStr">
+      <c r="F34" s="26" t="inlineStr">
         <is>
           <t>Gerechtigkeitsvorstellungen</t>
         </is>
       </c>
-      <c r="F34" s="26" t="inlineStr">
+      <c r="G34" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73899,22 +74283,27 @@
           <t>Weniger Ungleichheiten</t>
         </is>
       </c>
-      <c r="C35" s="32" t="inlineStr">
+      <c r="C35" s="26" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="D35" s="32" t="inlineStr">
         <is>
           <t>Geschichte</t>
         </is>
       </c>
-      <c r="D35" s="26" t="inlineStr">
+      <c r="E35" s="26" t="inlineStr">
         <is>
           <t>Eigenes und Fremdes</t>
         </is>
       </c>
-      <c r="E35" s="26" t="inlineStr">
+      <c r="F35" s="26" t="inlineStr">
         <is>
           <t>Umgang mit dem Fremden</t>
         </is>
       </c>
-      <c r="F35" s="26" t="inlineStr">
+      <c r="G35" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73929,22 +74318,27 @@
           <t>Weniger Ungleichheiten</t>
         </is>
       </c>
-      <c r="C36" s="36" t="inlineStr">
+      <c r="C36" s="26" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="D36" s="36" t="inlineStr">
         <is>
           <t>Moderne Fremdsprachen</t>
         </is>
       </c>
-      <c r="D36" s="26" t="inlineStr">
+      <c r="E36" s="26" t="inlineStr">
         <is>
           <t>Öffentlich-gesellschaftliche Lebenswelten „Ich und die Gesellschaft“</t>
         </is>
       </c>
-      <c r="E36" s="26" t="inlineStr">
+      <c r="F36" s="26" t="inlineStr">
         <is>
           <t>Gesellschaft in anderen Ländern</t>
         </is>
       </c>
-      <c r="F36" s="26" t="inlineStr">
+      <c r="G36" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73959,22 +74353,27 @@
           <t>Nachhaltige Städte und Gemeinden</t>
         </is>
       </c>
-      <c r="C37" s="30" t="inlineStr">
+      <c r="C37" s="26" t="inlineStr">
+        <is>
+          <t>11.6</t>
+        </is>
+      </c>
+      <c r="D37" s="30" t="inlineStr">
         <is>
           <t>Erdkunde</t>
         </is>
       </c>
-      <c r="D37" s="26" t="inlineStr">
+      <c r="E37" s="26" t="inlineStr">
         <is>
           <t>Geographie auf regionaler Ebene</t>
         </is>
       </c>
-      <c r="E37" s="26" t="inlineStr">
+      <c r="F37" s="26" t="inlineStr">
         <is>
           <t>Stadt und Region</t>
         </is>
       </c>
-      <c r="F37" s="26" t="inlineStr">
+      <c r="G37" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -73989,22 +74388,27 @@
           <t>Nachhaltige Städte und Gemeinden</t>
         </is>
       </c>
-      <c r="C38" s="29" t="inlineStr">
+      <c r="C38" s="26" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="D38" s="29" t="inlineStr">
         <is>
           <t>Physik</t>
         </is>
       </c>
-      <c r="D38" s="26" t="inlineStr">
+      <c r="E38" s="26" t="inlineStr">
         <is>
           <t>Fortbewegung und Mobilität</t>
         </is>
       </c>
-      <c r="E38" s="26" t="inlineStr">
+      <c r="F38" s="26" t="inlineStr">
         <is>
           <t>Mobilität</t>
         </is>
       </c>
-      <c r="F38" s="26" t="inlineStr">
+      <c r="G38" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74019,22 +74423,27 @@
           <t>Nachhaltige Städte und Gemeinden</t>
         </is>
       </c>
-      <c r="C39" s="32" t="inlineStr">
+      <c r="C39" s="26" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="D39" s="32" t="inlineStr">
         <is>
           <t>Geschichte</t>
         </is>
       </c>
-      <c r="D39" s="26" t="inlineStr">
+      <c r="E39" s="26" t="inlineStr">
         <is>
           <t>Epochenbezug Mittelalter</t>
         </is>
       </c>
-      <c r="E39" s="26" t="inlineStr">
+      <c r="F39" s="26" t="inlineStr">
         <is>
           <t>Städte als Triebkraft der Entwicklung</t>
         </is>
       </c>
-      <c r="F39" s="26" t="inlineStr">
+      <c r="G39" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74049,22 +74458,27 @@
           <t>Nachhaltige Städte und Gemeinden</t>
         </is>
       </c>
-      <c r="C40" s="32" t="inlineStr">
+      <c r="C40" s="26" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="D40" s="32" t="inlineStr">
         <is>
           <t>Geschichte</t>
         </is>
       </c>
-      <c r="D40" s="26" t="inlineStr">
+      <c r="E40" s="26" t="inlineStr">
         <is>
           <t>Bewältigung und Nutzung von Räumen</t>
         </is>
       </c>
-      <c r="E40" s="26" t="inlineStr">
+      <c r="F40" s="26" t="inlineStr">
         <is>
           <t>Raumnutzung</t>
         </is>
       </c>
-      <c r="F40" s="26" t="inlineStr">
+      <c r="G40" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74079,22 +74493,27 @@
           <t>Nachhaltige/r Konsum und Produktion</t>
         </is>
       </c>
-      <c r="C41" s="31" t="inlineStr">
+      <c r="C41" s="26" t="inlineStr">
+        <is>
+          <t>12.8</t>
+        </is>
+      </c>
+      <c r="D41" s="31" t="inlineStr">
         <is>
           <t>Politik und Wirtschaft</t>
         </is>
       </c>
-      <c r="D41" s="26" t="inlineStr">
+      <c r="E41" s="26" t="inlineStr">
         <is>
           <t>Wirtschaft</t>
         </is>
       </c>
-      <c r="E41" s="26" t="inlineStr">
+      <c r="F41" s="26" t="inlineStr">
         <is>
           <t>Konsumentenentscheidungen</t>
         </is>
       </c>
-      <c r="F41" s="26" t="inlineStr">
+      <c r="G41" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74109,22 +74528,27 @@
           <t>Nachhaltige/r Konsum und Produktion</t>
         </is>
       </c>
-      <c r="C42" s="28" t="inlineStr">
+      <c r="C42" s="26" t="inlineStr">
+        <is>
+          <t>12.4</t>
+        </is>
+      </c>
+      <c r="D42" s="28" t="inlineStr">
         <is>
           <t>Chemie</t>
         </is>
       </c>
-      <c r="D42" s="26" t="inlineStr">
+      <c r="E42" s="26" t="inlineStr">
         <is>
           <t>Schatzkiste der Natur – Chemie in Alltag und Technik</t>
         </is>
       </c>
-      <c r="E42" s="26" t="inlineStr">
+      <c r="F42" s="26" t="inlineStr">
         <is>
           <t>Stoffe in Alltag und Technik</t>
         </is>
       </c>
-      <c r="F42" s="26" t="inlineStr">
+      <c r="G42" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74139,22 +74563,27 @@
           <t>Nachhaltige/r Konsum und Produktion</t>
         </is>
       </c>
-      <c r="C43" s="28" t="inlineStr">
+      <c r="C43" s="26" t="inlineStr">
+        <is>
+          <t>12.5</t>
+        </is>
+      </c>
+      <c r="D43" s="28" t="inlineStr">
         <is>
           <t>Chemie</t>
         </is>
       </c>
-      <c r="D43" s="26" t="inlineStr">
+      <c r="E43" s="26" t="inlineStr">
         <is>
           <t>Magie des Kohlenstoffs – Organische Verbindungen</t>
         </is>
       </c>
-      <c r="E43" s="26" t="inlineStr">
+      <c r="F43" s="26" t="inlineStr">
         <is>
           <t>Kunststoffe und Rohstoffe</t>
         </is>
       </c>
-      <c r="F43" s="26" t="inlineStr">
+      <c r="G43" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74169,22 +74598,27 @@
           <t>Nachhaltige/r Konsum und Produktion</t>
         </is>
       </c>
-      <c r="C44" s="33" t="inlineStr">
+      <c r="C44" s="26" t="inlineStr">
+        <is>
+          <t>12.8</t>
+        </is>
+      </c>
+      <c r="D44" s="33" t="inlineStr">
         <is>
           <t>Arbeitslehre</t>
         </is>
       </c>
-      <c r="D44" s="26" t="inlineStr">
+      <c r="E44" s="26" t="inlineStr">
         <is>
           <t>Ökonomisch geprägte Situationen und Strukturen des Zusammenlebens</t>
         </is>
       </c>
-      <c r="E44" s="26" t="inlineStr">
+      <c r="F44" s="26" t="inlineStr">
         <is>
           <t>Verwendung von Einkommen</t>
         </is>
       </c>
-      <c r="F44" s="26" t="inlineStr">
+      <c r="G44" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74199,22 +74633,27 @@
           <t>Maßnahmen zum Klimaschutz</t>
         </is>
       </c>
-      <c r="C45" s="29" t="inlineStr">
+      <c r="C45" s="26" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="D45" s="29" t="inlineStr">
         <is>
           <t>Physik</t>
         </is>
       </c>
-      <c r="D45" s="26" t="inlineStr">
+      <c r="E45" s="26" t="inlineStr">
         <is>
           <t>Wettererscheinungen und Klima</t>
         </is>
       </c>
-      <c r="E45" s="26" t="inlineStr">
+      <c r="F45" s="26" t="inlineStr">
         <is>
           <t>Wetter und Klima</t>
         </is>
       </c>
-      <c r="F45" s="26" t="inlineStr">
+      <c r="G45" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74229,22 +74668,27 @@
           <t>Maßnahmen zum Klimaschutz</t>
         </is>
       </c>
-      <c r="C46" s="30" t="inlineStr">
+      <c r="C46" s="26" t="inlineStr">
+        <is>
+          <t>13.1</t>
+        </is>
+      </c>
+      <c r="D46" s="30" t="inlineStr">
         <is>
           <t>Erdkunde</t>
         </is>
       </c>
-      <c r="D46" s="26" t="inlineStr">
+      <c r="E46" s="26" t="inlineStr">
         <is>
           <t>Umwelt-Gesellschaft-Beziehungen und globale Probleme</t>
         </is>
       </c>
-      <c r="E46" s="26" t="inlineStr">
+      <c r="F46" s="26" t="inlineStr">
         <is>
           <t>Globale Probleme</t>
         </is>
       </c>
-      <c r="F46" s="26" t="inlineStr">
+      <c r="G46" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74259,22 +74703,27 @@
           <t>Maßnahmen zum Klimaschutz</t>
         </is>
       </c>
-      <c r="C47" s="30" t="inlineStr">
+      <c r="C47" s="26" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="D47" s="30" t="inlineStr">
         <is>
           <t>Erdkunde</t>
         </is>
       </c>
-      <c r="D47" s="26" t="inlineStr">
+      <c r="E47" s="26" t="inlineStr">
         <is>
           <t>Natur/Umwelt</t>
         </is>
       </c>
-      <c r="E47" s="26" t="inlineStr">
+      <c r="F47" s="26" t="inlineStr">
         <is>
           <t>Klima als Naturfaktor</t>
         </is>
       </c>
-      <c r="F47" s="26" t="inlineStr">
+      <c r="G47" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74289,22 +74738,27 @@
           <t>Maßnahmen zum Klimaschutz</t>
         </is>
       </c>
-      <c r="C48" s="27" t="inlineStr">
+      <c r="C48" s="26" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="D48" s="27" t="inlineStr">
         <is>
           <t>Biologie</t>
         </is>
       </c>
-      <c r="D48" s="26" t="inlineStr">
+      <c r="E48" s="26" t="inlineStr">
         <is>
           <t>Stoffwechsel und Regelmechanismen</t>
         </is>
       </c>
-      <c r="E48" s="26" t="inlineStr">
+      <c r="F48" s="26" t="inlineStr">
         <is>
           <t>Kohlenstoffkreislauf</t>
         </is>
       </c>
-      <c r="F48" s="26" t="inlineStr">
+      <c r="G48" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74319,22 +74773,27 @@
           <t>Leben unter Wasser</t>
         </is>
       </c>
-      <c r="C49" s="27" t="inlineStr">
+      <c r="C49" s="26" t="inlineStr">
+        <is>
+          <t>14.2</t>
+        </is>
+      </c>
+      <c r="D49" s="27" t="inlineStr">
         <is>
           <t>Biologie</t>
         </is>
       </c>
-      <c r="D49" s="26" t="inlineStr">
+      <c r="E49" s="26" t="inlineStr">
         <is>
           <t>Wechselwirkungen in Ökosystemen</t>
         </is>
       </c>
-      <c r="E49" s="26" t="inlineStr">
+      <c r="F49" s="26" t="inlineStr">
         <is>
           <t>Gewässer als Ökosystem</t>
         </is>
       </c>
-      <c r="F49" s="26" t="inlineStr">
+      <c r="G49" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74349,22 +74808,27 @@
           <t>Leben an Land</t>
         </is>
       </c>
-      <c r="C50" s="27" t="inlineStr">
+      <c r="C50" s="26" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="D50" s="27" t="inlineStr">
         <is>
           <t>Biologie</t>
         </is>
       </c>
-      <c r="D50" s="26" t="inlineStr">
+      <c r="E50" s="26" t="inlineStr">
         <is>
           <t>Wechselwirkungen in Ökosystemen</t>
         </is>
       </c>
-      <c r="E50" s="26" t="inlineStr">
+      <c r="F50" s="26" t="inlineStr">
         <is>
           <t>Gefährdung von Ökosystemen</t>
         </is>
       </c>
-      <c r="F50" s="26" t="inlineStr">
+      <c r="G50" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74379,22 +74843,27 @@
           <t>Leben an Land</t>
         </is>
       </c>
-      <c r="C51" s="27" t="inlineStr">
+      <c r="C51" s="26" t="inlineStr">
+        <is>
+          <t>15.5</t>
+        </is>
+      </c>
+      <c r="D51" s="27" t="inlineStr">
         <is>
           <t>Biologie</t>
         </is>
       </c>
-      <c r="D51" s="26" t="inlineStr">
+      <c r="E51" s="26" t="inlineStr">
         <is>
           <t>Vielfalt, Veränderung und Abstammung von Lebewesen</t>
         </is>
       </c>
-      <c r="E51" s="26" t="inlineStr">
+      <c r="F51" s="26" t="inlineStr">
         <is>
           <t>Artenvielfalt und Artensterben</t>
         </is>
       </c>
-      <c r="F51" s="26" t="inlineStr">
+      <c r="G51" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74409,22 +74878,27 @@
           <t>Leben an Land</t>
         </is>
       </c>
-      <c r="C52" s="30" t="inlineStr">
+      <c r="C52" s="26" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="D52" s="30" t="inlineStr">
         <is>
           <t>Erdkunde</t>
         </is>
       </c>
-      <c r="D52" s="26" t="inlineStr">
+      <c r="E52" s="26" t="inlineStr">
         <is>
           <t>Natur/Umwelt</t>
         </is>
       </c>
-      <c r="E52" s="26" t="inlineStr">
+      <c r="F52" s="26" t="inlineStr">
         <is>
           <t>Naturräume</t>
         </is>
       </c>
-      <c r="F52" s="26" t="inlineStr">
+      <c r="G52" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74439,22 +74913,27 @@
           <t>Leben an Land</t>
         </is>
       </c>
-      <c r="C53" s="40" t="inlineStr">
+      <c r="C53" s="26" t="inlineStr">
+        <is>
+          <t>15.5</t>
+        </is>
+      </c>
+      <c r="D53" s="40" t="inlineStr">
         <is>
           <t>Ethik</t>
         </is>
       </c>
-      <c r="D53" s="26" t="inlineStr">
+      <c r="E53" s="26" t="inlineStr">
         <is>
           <t>Mensch, Natur und Technik</t>
         </is>
       </c>
-      <c r="E53" s="26" t="inlineStr">
+      <c r="F53" s="26" t="inlineStr">
         <is>
           <t>Verantwortung für Lebewesen und Natur</t>
         </is>
       </c>
-      <c r="F53" s="26" t="inlineStr">
+      <c r="G53" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74469,22 +74948,27 @@
           <t>Leben an Land</t>
         </is>
       </c>
-      <c r="C54" s="37" t="inlineStr">
+      <c r="C54" s="26" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="D54" s="37" t="inlineStr">
         <is>
           <t>Kunst</t>
         </is>
       </c>
-      <c r="D54" s="26" t="inlineStr">
+      <c r="E54" s="26" t="inlineStr">
         <is>
           <t>Wahrnehmung der Umwelt</t>
         </is>
       </c>
-      <c r="E54" s="26" t="inlineStr">
+      <c r="F54" s="26" t="inlineStr">
         <is>
           <t>Haltung zur Umwelt</t>
         </is>
       </c>
-      <c r="F54" s="26" t="inlineStr">
+      <c r="G54" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74499,22 +74983,27 @@
           <t>Frieden, Gerechtigkeit und starke Institutionen</t>
         </is>
       </c>
-      <c r="C55" s="31" t="inlineStr">
+      <c r="C55" s="26" t="inlineStr">
+        <is>
+          <t>16.7</t>
+        </is>
+      </c>
+      <c r="D55" s="31" t="inlineStr">
         <is>
           <t>Politik und Wirtschaft</t>
         </is>
       </c>
-      <c r="D55" s="26" t="inlineStr">
+      <c r="E55" s="26" t="inlineStr">
         <is>
           <t>Demokratie</t>
         </is>
       </c>
-      <c r="E55" s="26" t="inlineStr">
+      <c r="F55" s="26" t="inlineStr">
         <is>
           <t>Demokratische Institutionen</t>
         </is>
       </c>
-      <c r="F55" s="26" t="inlineStr">
+      <c r="G55" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74529,22 +75018,27 @@
           <t>Frieden, Gerechtigkeit und starke Institutionen</t>
         </is>
       </c>
-      <c r="C56" s="31" t="inlineStr">
+      <c r="C56" s="26" t="inlineStr">
+        <is>
+          <t>16.3</t>
+        </is>
+      </c>
+      <c r="D56" s="31" t="inlineStr">
         <is>
           <t>Politik und Wirtschaft</t>
         </is>
       </c>
-      <c r="D56" s="26" t="inlineStr">
+      <c r="E56" s="26" t="inlineStr">
         <is>
           <t>Recht und Rechtsprechung</t>
         </is>
       </c>
-      <c r="E56" s="26" t="inlineStr">
+      <c r="F56" s="26" t="inlineStr">
         <is>
           <t>Rechtsstaat</t>
         </is>
       </c>
-      <c r="F56" s="26" t="inlineStr">
+      <c r="G56" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74559,22 +75053,27 @@
           <t>Frieden, Gerechtigkeit und starke Institutionen</t>
         </is>
       </c>
-      <c r="C57" s="32" t="inlineStr">
+      <c r="C57" s="26" t="inlineStr">
+        <is>
+          <t>16.7</t>
+        </is>
+      </c>
+      <c r="D57" s="32" t="inlineStr">
         <is>
           <t>Geschichte</t>
         </is>
       </c>
-      <c r="D57" s="26" t="inlineStr">
+      <c r="E57" s="26" t="inlineStr">
         <is>
           <t>Herrschaft</t>
         </is>
       </c>
-      <c r="E57" s="26" t="inlineStr">
+      <c r="F57" s="26" t="inlineStr">
         <is>
           <t>Legitimation von Herrschaft</t>
         </is>
       </c>
-      <c r="F57" s="26" t="inlineStr">
+      <c r="G57" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74589,22 +75088,27 @@
           <t>Frieden, Gerechtigkeit und starke Institutionen</t>
         </is>
       </c>
-      <c r="C58" s="32" t="inlineStr">
+      <c r="C58" s="26" t="inlineStr">
+        <is>
+          <t>16.1</t>
+        </is>
+      </c>
+      <c r="D58" s="32" t="inlineStr">
         <is>
           <t>Geschichte</t>
         </is>
       </c>
-      <c r="D58" s="26" t="inlineStr">
+      <c r="E58" s="26" t="inlineStr">
         <is>
           <t>Epochenbezug Neueste Zeit</t>
         </is>
       </c>
-      <c r="E58" s="26" t="inlineStr">
+      <c r="F58" s="26" t="inlineStr">
         <is>
           <t>Friedenssicherung, totalitäre Systeme, Shoa</t>
         </is>
       </c>
-      <c r="F58" s="26" t="inlineStr">
+      <c r="G58" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74619,22 +75123,27 @@
           <t>Frieden, Gerechtigkeit und starke Institutionen</t>
         </is>
       </c>
-      <c r="C59" s="40" t="inlineStr">
+      <c r="C59" s="26" t="inlineStr">
+        <is>
+          <t>16.3</t>
+        </is>
+      </c>
+      <c r="D59" s="40" t="inlineStr">
         <is>
           <t>Ethik</t>
         </is>
       </c>
-      <c r="D59" s="26" t="inlineStr">
+      <c r="E59" s="26" t="inlineStr">
         <is>
           <t>Recht und Gerechtigkeit</t>
         </is>
       </c>
-      <c r="E59" s="26" t="inlineStr">
+      <c r="F59" s="26" t="inlineStr">
         <is>
           <t>Recht und Menschenrechte</t>
         </is>
       </c>
-      <c r="F59" s="26" t="inlineStr">
+      <c r="G59" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74649,22 +75158,23 @@
           <t>Frieden, Gerechtigkeit und starke Institutionen</t>
         </is>
       </c>
-      <c r="C60" s="41" t="inlineStr">
+      <c r="C60" s="26" t="inlineStr"/>
+      <c r="D60" s="41" t="inlineStr">
         <is>
           <t>Evangelische Religion</t>
         </is>
       </c>
-      <c r="D60" s="26" t="inlineStr">
+      <c r="E60" s="26" t="inlineStr">
         <is>
           <t>Ethik</t>
         </is>
       </c>
-      <c r="E60" s="26" t="inlineStr">
+      <c r="F60" s="26" t="inlineStr">
         <is>
           <t>Verantwortliches Handeln</t>
         </is>
       </c>
-      <c r="F60" s="26" t="inlineStr">
+      <c r="G60" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74679,22 +75189,27 @@
           <t>Partnerschaften zur Erreichung der Ziele</t>
         </is>
       </c>
-      <c r="C61" s="31" t="inlineStr">
+      <c r="C61" s="26" t="inlineStr">
+        <is>
+          <t>17.16</t>
+        </is>
+      </c>
+      <c r="D61" s="31" t="inlineStr">
         <is>
           <t>Politik und Wirtschaft</t>
         </is>
       </c>
-      <c r="D61" s="26" t="inlineStr">
+      <c r="E61" s="26" t="inlineStr">
         <is>
           <t>Internationale Beziehungen und Globalisierung</t>
         </is>
       </c>
-      <c r="E61" s="26" t="inlineStr">
+      <c r="F61" s="26" t="inlineStr">
         <is>
           <t>Internationale Zusammenarbeit</t>
         </is>
       </c>
-      <c r="F61" s="26" t="inlineStr">
+      <c r="G61" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74709,22 +75224,27 @@
           <t>Partnerschaften zur Erreichung der Ziele</t>
         </is>
       </c>
-      <c r="C62" s="36" t="inlineStr">
+      <c r="C62" s="26" t="inlineStr">
+        <is>
+          <t>17.16</t>
+        </is>
+      </c>
+      <c r="D62" s="36" t="inlineStr">
         <is>
           <t>Moderne Fremdsprachen</t>
         </is>
       </c>
-      <c r="D62" s="26" t="inlineStr">
+      <c r="E62" s="26" t="inlineStr">
         <is>
           <t>Kulturelle Lebenswelten „Ich und die Welt“</t>
         </is>
       </c>
-      <c r="E62" s="26" t="inlineStr">
+      <c r="F62" s="26" t="inlineStr">
         <is>
           <t>Interkulturelle Verständigung</t>
         </is>
       </c>
-      <c r="F62" s="26" t="inlineStr">
+      <c r="G62" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74739,22 +75259,23 @@
           <t>Partnerschaften zur Erreichung der Ziele</t>
         </is>
       </c>
-      <c r="C63" s="40" t="inlineStr">
+      <c r="C63" s="26" t="inlineStr"/>
+      <c r="D63" s="40" t="inlineStr">
         <is>
           <t>Ethik</t>
         </is>
       </c>
-      <c r="D63" s="26" t="inlineStr">
+      <c r="E63" s="26" t="inlineStr">
         <is>
           <t>Religionen, Weltbilder und Kulturen</t>
         </is>
       </c>
-      <c r="E63" s="26" t="inlineStr">
+      <c r="F63" s="26" t="inlineStr">
         <is>
           <t>Dialog der Kulturen</t>
         </is>
       </c>
-      <c r="F63" s="26" t="inlineStr">
+      <c r="G63" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74769,22 +75290,23 @@
           <t>Partnerschaften zur Erreichung der Ziele</t>
         </is>
       </c>
-      <c r="C64" s="41" t="inlineStr">
+      <c r="C64" s="26" t="inlineStr"/>
+      <c r="D64" s="41" t="inlineStr">
         <is>
           <t>Evangelische Religion</t>
         </is>
       </c>
-      <c r="D64" s="26" t="inlineStr">
+      <c r="E64" s="26" t="inlineStr">
         <is>
           <t>Religionen</t>
         </is>
       </c>
-      <c r="E64" s="26" t="inlineStr">
+      <c r="F64" s="26" t="inlineStr">
         <is>
           <t>Dialog der Religionen</t>
         </is>
       </c>
-      <c r="F64" s="26" t="inlineStr">
+      <c r="G64" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
@@ -74799,29 +75321,30 @@
           <t>Partnerschaften zur Erreichung der Ziele</t>
         </is>
       </c>
-      <c r="C65" s="42" t="inlineStr">
+      <c r="C65" s="26" t="inlineStr"/>
+      <c r="D65" s="42" t="inlineStr">
         <is>
           <t>Katholische Religion</t>
         </is>
       </c>
-      <c r="D65" s="26" t="inlineStr">
+      <c r="E65" s="26" t="inlineStr">
         <is>
           <t>Religionen</t>
         </is>
       </c>
-      <c r="E65" s="26" t="inlineStr">
+      <c r="F65" s="26" t="inlineStr">
         <is>
           <t>Dialog der Religionen</t>
         </is>
       </c>
-      <c r="F65" s="26" t="inlineStr">
+      <c r="G65" s="26" t="inlineStr">
         <is>
           <t>Vorschlag, fachlich zu prüfen</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F65"/>
+  <autoFilter ref="A1:G65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -74832,195 +75355,1620 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="100" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="25" t="inlineStr">
         <is>
-          <t>Punkt</t>
+          <t>SDG</t>
         </is>
       </c>
       <c r="B1" s="25" t="inlineStr">
         <is>
-          <t>Hinweis</t>
+          <t>Nachhaltigkeitsziel</t>
+        </is>
+      </c>
+      <c r="C1" s="25" t="inlineStr">
+        <is>
+          <t>Unterziel</t>
+        </is>
+      </c>
+      <c r="D1" s="25" t="inlineStr">
+        <is>
+          <t>Wortlaut (amtliche deutsche Fassung)</t>
+        </is>
+      </c>
+      <c r="E1" s="25" t="inlineStr">
+        <is>
+          <t>Quelle</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="26" t="inlineStr">
-        <is>
-          <t>Bildungsgang</t>
-        </is>
+      <c r="A2" s="26" t="n">
+        <v>1</v>
       </c>
       <c r="B2" s="26" t="inlineStr">
         <is>
-          <t>Inhaltsfelder sind für 17 Fächer in allen drei KC-Fassungen erfasst (Hauptschule, Realschule, Gymnasium). Schwerpunkte gibt es für alle Fächer (teils automatisch ausgelesen, siehe Spalte Hinweis); Kompetenzbereiche nur Pilotfächer in der Gymnasialfassung.</t>
+          <t>Keine Armut</t>
+        </is>
+      </c>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="D2" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 den Anteil der Männer, Frauen und Kinder jeden Alters, die in Armut in all ihren Dimensionen nach der jeweiligen nationalen Definition leben, mindestens um die Hälfte senken</t>
+        </is>
+      </c>
+      <c r="E2" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="26" t="inlineStr">
-        <is>
-          <t>Haupt- und Realschule</t>
-        </is>
+      <c r="A3" s="26" t="n">
+        <v>1</v>
       </c>
       <c r="B3" s="26" t="inlineStr">
         <is>
-          <t>Biologie, Chemie, Physik: Übersichtstabelle Kap. 7.3 bzw. 7.2, Stufen bis Jg. 5/6 bzw. 1. Lernjahr bzw. Hälfte des Stundenkontingents und zusätzlich bis Abschluss Jg. 9 (HS) oder 10 (RS). Erdkunde: Kap. 7.1 (Ende Jg. 6), Kap. 7.2 entfällt laut KC. PoWi: Kap. 7 entfällt laut KC.</t>
+          <t>Keine Armut</t>
+        </is>
+      </c>
+      <c r="C3" s="26" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="D3" s="26" t="inlineStr">
+        <is>
+          <t>Den nationalen Gegebenheiten entsprechende Sozialschutzsysteme und -maßnahmen für alle umsetzen, einschließlich eines Basisschutzes, und bis 2030 eine breite Versorgung der Armen und Schwachen erreichen</t>
+        </is>
+      </c>
+      <c r="E3" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="26" t="inlineStr">
-        <is>
-          <t>Fächerauswahl</t>
-        </is>
+      <c r="A4" s="26" t="n">
+        <v>1</v>
       </c>
       <c r="B4" s="26" t="inlineStr">
         <is>
-          <t>Aufgenommen sind die Fächer einer IGS 5 bis 10. Latein, Griechisch, Chinesisch, Arabisch sowie alevitische, jüdische und islamische Religion fehlen noch. Informatik gibt es nur als KC für den Wahlunterricht am Gymnasium.</t>
+          <t>Keine Armut</t>
+        </is>
+      </c>
+      <c r="C4" s="26" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="D4" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 die Widerstandsfähigkeit der Armen und der Menschen in prekären Situationen erhöhen und ihre Exposition und Anfälligkeit gegenüber klimabedingten Extremereignissen und anderen wirtschaftlichen, sozialen und ökologischen Schocks und Katastrophen verringern</t>
+        </is>
+      </c>
+      <c r="E4" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>Moderne Fremdsprachen</t>
-        </is>
+      <c r="A5" s="26" t="n">
+        <v>2</v>
       </c>
       <c r="B5" s="26" t="inlineStr">
         <is>
-          <t>Ein gemeinsames KC für alle modernen Fremdsprachen. Die Inhaltsfelder sind drei Lebenswelten.</t>
+          <t>Kein Hunger</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="D5" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 den Hunger beenden und sicherstellen, dass alle Menschen, insbesondere die Armen und Menschen in prekären Situationen, einschließlich Kleinkindern, ganzjährig Zugang zu sicheren, nährstoffreichen und ausreichenden Nahrungsmitteln haben</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr">
-        <is>
-          <t>Kunst</t>
-        </is>
+      <c r="A6" s="26" t="n">
+        <v>2</v>
       </c>
       <c r="B6" s="26" t="inlineStr">
         <is>
-          <t>Die Zuordnung der neun Inhaltsfelder zu den drei Kernbereichen steht nur in Abb. 2 (Kap. 5).</t>
+          <t>Kein Hunger</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 alle Formen der Fehlernährung beenden, einschließlich durch Erreichung der international vereinbarten Zielvorgaben in Bezug auf Wachstumshemmung und Auszehrung bei Kindern unter 5 Jahren bis 2025, und den Ernährungsbedürfnissen von heranwachsenden Mädchen, schwangeren und stillenden Frauen und älteren Menschen Rechnung tragen</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
-        <is>
-          <t>Religion</t>
-        </is>
+      <c r="A7" s="26" t="n">
+        <v>2</v>
       </c>
       <c r="B7" s="26" t="inlineStr">
         <is>
-          <t>Evangelische und Katholische Religion liegen in der neuen KC-Fassung von 2026 vor.</t>
+          <t>Kein Hunger</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 die Nachhaltigkeit der Systeme der Nahrungsmittelproduktion sicherstellen und resiliente landwirtschaftliche Methoden anwenden, die die Produktivität und den Ertrag steigern, zur Erhaltung der Ökosysteme beitragen, die Anpassungsfähigkeit an Klimaänderungen, extreme Wetterereignisse, Dürren, Überschwemmungen und andere Katastrophen erhöhen und die Flächen- und Bodenqualität schrittweise verbessern</t>
+        </is>
+      </c>
+      <c r="E7" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="26" t="inlineStr">
-        <is>
-          <t>BNE</t>
-        </is>
+      <c r="A8" s="26" t="n">
+        <v>3</v>
       </c>
       <c r="B8" s="26" t="inlineStr">
         <is>
-          <t>BNE ist nach § 6 Abs. 4 HSchG ein Aufgabengebiet. Die KC von 2011 nennen BNE nicht ausdrücklich. Als Beleg zählt nur, wo das KC selbst Nachhaltigkeit nennt (Blatt 'BNE Belege'). Die SDG-Zuordnung ist ein Vorschlag.</t>
+          <t>Gesundheit und Wohlergehen</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 die Aids-, Tuberkulose- und Malariaepidemien und die vernachlässigten Tropenkrankheiten beseitigen und Hepatitis, durch Wasser übertragene Krankheiten und andere übertragbare Krankheiten bekämpfen</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="26" t="inlineStr">
-        <is>
-          <t>Stufung</t>
-        </is>
+      <c r="A9" s="26" t="n">
+        <v>3</v>
       </c>
       <c r="B9" s="26" t="inlineStr">
         <is>
-          <t>Die Stufen sind nicht einheitlich: Biologie 'bis Ende 5/6', Chemie '1. Lernjahr', Physik 'nach ca. der Hälfte des Stundenkontingents', jeweils plus 'bis Ende 9/10'. Erdkunde und Politik und Wirtschaft haben im Gymnasium-KC keine Stufung. Die Zuordnung zu Jahrgängen hängt an der Stundentafel bzw. am Schulcurriculum.</t>
+          <t>Gesundheit und Wohlergehen</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 die vorzeitige Sterblichkeit aufgrund von nichtübertragbaren Krankheiten durch Prävention und Behandlung um ein Drittel senken und die psychische Gesundheit und das Wohlergehen fördern</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="26" t="inlineStr">
-        <is>
-          <t>Jahrgang 8</t>
-        </is>
+      <c r="A10" s="26" t="n">
+        <v>3</v>
       </c>
       <c r="B10" s="26" t="inlineStr">
         <is>
-          <t>Biologie, Chemie, Physik, Erdkunde und PoWi weisen für das Gymnasium ausdrücklich keine Kompetenzerwartungen für Jahrgang 6/8 bzw. 8 aus (jeweils Kap. 7).</t>
+          <t>Gesundheit und Wohlergehen</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="D10" s="26" t="inlineStr">
+        <is>
+          <t>Die Prävention und Behandlung des Substanzmissbrauchs, namentlich des Suchtstoffmissbrauchs und des schädlichen Gebrauchs von Alkohol, verstärken</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="26" t="inlineStr">
-        <is>
-          <t>Erdkunde, PoWi</t>
-        </is>
+      <c r="A11" s="26" t="n">
+        <v>3</v>
       </c>
       <c r="B11" s="26" t="inlineStr">
         <is>
-          <t>Die Einträge im Blatt 'Schwerpunkte' sind Stichworte aus den Inhaltsfeldbeschreibungen (Kap. 6), da es keine Schwerpunkt-Tabelle gibt.</t>
+          <t>Gesundheit und Wohlergehen</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>3.6</t>
+        </is>
+      </c>
+      <c r="D11" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2020 die Zahl der Todesfälle und Verletzungen infolge von Straßenverkehrsunfällen weltweit halbieren</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="26" t="inlineStr">
-        <is>
-          <t>PoWi</t>
-        </is>
+      <c r="A12" s="26" t="n">
+        <v>3</v>
       </c>
       <c r="B12" s="26" t="inlineStr">
         <is>
-          <t>Im PDF ist der rechte Teil der quer gesetzten Tabellen beim Auslesen abgeschnitten. Stichworte bitte am Original prüfen.</t>
+          <t>Gesundheit und Wohlergehen</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="D12" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 den allgemeinen Zugang zu sexual- und reproduktionsmedizinischer Versorgung, einschließlich Familienplanung, Information und Aufklärung, und die Einbeziehung der reproduktiven Gesundheit in nationale Strategien und Programme gewährleisten</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="26" t="inlineStr">
-        <is>
-          <t>Grafiken</t>
-        </is>
+      <c r="A13" s="26" t="n">
+        <v>4</v>
       </c>
       <c r="B13" s="26" t="inlineStr">
         <is>
-          <t>Abbildungen (z. B. Basiskonzept-Zuordnung Physik, Verzahnung Erdkunde/PoWi/Geschichte) ließen sich nicht als Text auslesen und fehlen.</t>
+          <t>Hochwertige Bildung</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="D13" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 sicherstellen, dass alle Mädchen und Jungen gleichberechtigt eine kostenlose und hochwertige Grund- und Sekundarschulbildung abschließen, die zu brauchbaren und effektiven Lernergebnissen führt</t>
+        </is>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="26" t="inlineStr">
-        <is>
-          <t>Wortlaut</t>
-        </is>
+      <c r="A14" s="26" t="n">
+        <v>4</v>
       </c>
       <c r="B14" s="26" t="inlineStr">
         <is>
-          <t>Schwerpunkte sind teils gekürzt oder zusammengefasst. Für verbindliche Formulierungen gilt das Original (Seitenangabe je Zeile).</t>
+          <t>Hochwertige Bildung</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="D14" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 die Zahl der Jugendlichen und Erwachsenen wesentlich erhöhen, die über die entsprechenden Qualifikationen einschließlich fachlicher und beruflicher Qualifikationen für eine Beschäftigung, eine menschenwürdige Arbeit und Unternehmertum verfügen</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="26" t="inlineStr">
-        <is>
-          <t>Anknüpfungspunkte</t>
-        </is>
+      <c r="A15" s="26" t="n">
+        <v>4</v>
       </c>
       <c r="B15" s="26" t="inlineStr">
         <is>
-          <t>Das Blatt 'Anknüpfungspunkte' enthält Vorschläge auf Basis gemeinsamer Stichworte. Sie stehen so nicht im KC und sind fachlich zu prüfen.</t>
+          <t>Hochwertige Bildung</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="D15" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 geschlechtsspezifische Disparitäten in der Bildung beseitigen und den gleichberechtigen Zugang der Schwachen in der Gesellschaft, namentlich von Menschen mit Behinderungen, Angehörigen indigener Völker und Kindern in prekären Situationen, zu allen Bildungs- und Ausbildungsebenen gewährleisten</t>
+        </is>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>Hochwertige Bildung</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="D16" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 sicherstellen, dass alle Lernenden die notwendigen Kenntnisse und Qualifikationen zur Förderung nachhaltiger Entwicklung erwerben, unter anderem durch Bildung für nachhaltige Entwicklung und nachhaltige Lebensweisen, Menschenrechte, Geschlechtergleichstellung, eine Kultur des Friedens und der Gewaltlosigkeit, Weltbürgerschaft und die Wertschätzung kultureller Vielfalt und des Beitrags der Kultur zu nachhaltiger Entwicklung</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>Geschlechtergleichheit</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="D17" s="26" t="inlineStr">
+        <is>
+          <t>Alle Formen der Diskriminierung von Frauen und Mädchen überall auf der Welt beenden</t>
+        </is>
+      </c>
+      <c r="E17" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>Geschlechtergleichheit</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="D18" s="26" t="inlineStr">
+        <is>
+          <t>Alle Formen von Gewalt gegen alle Frauen und Mädchen im öffentlichen und im privaten Bereich einschließlich des Menschenhandels und sexueller und anderer Formen der Ausbeutung beseitigen</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>Geschlechtergleichheit</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
+      <c r="D19" s="26" t="inlineStr">
+        <is>
+          <t>Die volle und wirksame Teilhabe von Frauen und ihre Chancengleichheit bei der Übernahme von Führungsrollen auf allen Ebenen der Entscheidungsfindung im politischen, wirtschaftlichen und öffentlichen Leben sicherstellen</t>
+        </is>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>Sauberes Wasser und Sanitäreinrichtungen</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="D20" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 den allgemeinen und gerechten Zugang zu einwandfreiem und bezahlbarem Trinkwasser für alle erreichen</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>Sauberes Wasser und Sanitäreinrichtungen</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="D21" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 die Wasserqualität durch Verringerung der Verschmutzung, Beendigung des Einbringens und Minimierung der Freisetzung gefährlicher Chemikalien und Stoffe, Halbierung des Anteils unbehandelten Abwassers und eine beträchtliche Steigerung der Wiederaufbereitung und gefahrlosen Wiederverwendung weltweit verbessern</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>Sauberes Wasser und Sanitäreinrichtungen</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>6.4</t>
+        </is>
+      </c>
+      <c r="D22" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 die Effizienz der Wassernutzung in allen Sektoren wesentlich steigern und eine nachhaltige Entnahme und Bereitstellung von Süßwasser gewährleisten, um der Wasserknappheit zu begegnen und die Zahl der unter Wasserknappheit leidenden Menschen erheblich zu verringern</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>Sauberes Wasser und Sanitäreinrichtungen</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>6.6</t>
+        </is>
+      </c>
+      <c r="D23" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2020 wasserverbundene Ökosysteme schützen und wiederherstellen, darunter Berge, Wälder, Feuchtgebiete, Flüsse, Grundwasserleiter und Seen</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="26" t="n">
+        <v>7</v>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>Bezahlbare und saubere Energie</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>7.1</t>
+        </is>
+      </c>
+      <c r="D24" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 den allgemeinen Zugang zu bezahlbaren, verlässlichen und modernen Energiedienstleistungen sichern</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="26" t="n">
+        <v>7</v>
+      </c>
+      <c r="B25" s="26" t="inlineStr">
+        <is>
+          <t>Bezahlbare und saubere Energie</t>
+        </is>
+      </c>
+      <c r="C25" s="26" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="D25" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 den Anteil erneuerbarer Energie am globalen Energiemix deutlich erhöhen</t>
+        </is>
+      </c>
+      <c r="E25" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="26" t="n">
+        <v>7</v>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>Bezahlbare und saubere Energie</t>
+        </is>
+      </c>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="D26" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 die weltweite Steigerungsrate der Energieeffizienz verdoppeln</t>
+        </is>
+      </c>
+      <c r="E26" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="B27" s="26" t="inlineStr">
+        <is>
+          <t>Menschenwürdige Arbeit und Wirtschaftswachstum</t>
+        </is>
+      </c>
+      <c r="C27" s="26" t="inlineStr">
+        <is>
+          <t>8.4</t>
+        </is>
+      </c>
+      <c r="D27" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 die weltweite Ressourceneffizienz in Konsum und Produktion Schritt für Schritt verbessern und die Entkopplung von Wirtschaftswachstum und Umweltzerstörung anstreben, im Einklang mit dem Zehnjahres-Programmrahmen für nachhaltige Konsum- und Produktionsmuster, wobei die entwickelten Länder die Führung übernehmen</t>
+        </is>
+      </c>
+      <c r="E27" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="B28" s="26" t="inlineStr">
+        <is>
+          <t>Menschenwürdige Arbeit und Wirtschaftswachstum</t>
+        </is>
+      </c>
+      <c r="C28" s="26" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D28" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 produktive Vollbeschäftigung und menschenwürdige Arbeit für alle Frauen und Männer, einschließlich junger Menschen und Menschen mit Behinderungen, sowie gleiches Entgelt für gleichwertige Arbeit erreichen</t>
+        </is>
+      </c>
+      <c r="E28" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="B29" s="26" t="inlineStr">
+        <is>
+          <t>Menschenwürdige Arbeit und Wirtschaftswachstum</t>
+        </is>
+      </c>
+      <c r="C29" s="26" t="inlineStr">
+        <is>
+          <t>8.6</t>
+        </is>
+      </c>
+      <c r="D29" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2020 den Anteil junger Menschen, die sich weder in Schul- oder Berufsausbildung noch in Erwerbstätigkeit befinden, erheblich verringern</t>
+        </is>
+      </c>
+      <c r="E29" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="B30" s="26" t="inlineStr">
+        <is>
+          <t>Menschenwürdige Arbeit und Wirtschaftswachstum</t>
+        </is>
+      </c>
+      <c r="C30" s="26" t="inlineStr">
+        <is>
+          <t>8.7</t>
+        </is>
+      </c>
+      <c r="D30" s="26" t="inlineStr">
+        <is>
+          <t>Sofortige und wirksame Maßnahmen ergreifen, um Zwangsarbeit abzuschaffen, moderne Sklaverei und Menschenhandel zu beenden und das Verbot und die Beseitigung der schlimmsten Formen der Kinderarbeit, einschließlich der Einziehung und des Einsatzes von Kindersoldatinnen und -soldaten, sicherzustellen, und bis 2025 jeder Form von Kinderarbeit ein Ende setzen</t>
+        </is>
+      </c>
+      <c r="E30" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="B31" s="26" t="inlineStr">
+        <is>
+          <t>Menschenwürdige Arbeit und Wirtschaftswachstum</t>
+        </is>
+      </c>
+      <c r="C31" s="26" t="inlineStr">
+        <is>
+          <t>8.8</t>
+        </is>
+      </c>
+      <c r="D31" s="26" t="inlineStr">
+        <is>
+          <t>Die Arbeitsrechte schützen und sichere Arbeitsumgebungen für alle Erwerbstätigen, einschließlich der Arbeitsmigranten und insbesondere der Arbeitsmigrantinnen, und der Menschen in prekärer Erwerbstätigkeit, fördern</t>
+        </is>
+      </c>
+      <c r="E31" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="26" t="n">
+        <v>9</v>
+      </c>
+      <c r="B32" s="26" t="inlineStr">
+        <is>
+          <t>Industrie, Innovation und Infrastruktur</t>
+        </is>
+      </c>
+      <c r="C32" s="26" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="D32" s="26" t="inlineStr">
+        <is>
+          <t>Eine hochwertige, verlässliche, nachhaltige und widerstandsfähige Infrastruktur aufbauen, einschließlich regionaler und grenzüberschreitender Infrastruktur, um die wirtschaftliche Entwicklung und das menschliche Wohlergehen zu unterstützen, und dabei den Schwerpunkt auf einen erschwinglichen und gleichberechtigten Zugang für alle legen</t>
+        </is>
+      </c>
+      <c r="E32" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="26" t="n">
+        <v>9</v>
+      </c>
+      <c r="B33" s="26" t="inlineStr">
+        <is>
+          <t>Industrie, Innovation und Infrastruktur</t>
+        </is>
+      </c>
+      <c r="C33" s="26" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="D33" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 die Infrastruktur modernisieren und die Industrien nachrüsten, um sie nachhaltig zu machen, mit effizienterem Ressourceneinsatz und unter vermehrter Nutzung sauberer und umweltverträglicher Technologien und Industrieprozesse, wobei alle Länder Maßnahmen entsprechend ihren jeweiligen Kapazitäten ergreifen</t>
+        </is>
+      </c>
+      <c r="E33" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="26" t="n">
+        <v>9</v>
+      </c>
+      <c r="B34" s="26" t="inlineStr">
+        <is>
+          <t>Industrie, Innovation und Infrastruktur</t>
+        </is>
+      </c>
+      <c r="C34" s="26" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="D34" s="26" t="inlineStr">
+        <is>
+          <t>Die wissenschaftliche Forschung verbessern und die technologischen Kapazitäten der Industriesektoren in allen Ländern und insbesondere in den Entwicklungsländern ausbauen und zu diesem Zweck bis 2030 unter anderem Innovationen fördern und die Anzahl der im Bereich Forschung und Entwicklung tätigen Personen je 1 Million Menschen sowie die öffentlichen und privaten Ausgaben für Forschung und Entwicklung beträchtlich erhöhen</t>
+        </is>
+      </c>
+      <c r="E34" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="26" t="n">
+        <v>9</v>
+      </c>
+      <c r="B35" s="26" t="inlineStr">
+        <is>
+          <t>Industrie, Innovation und Infrastruktur</t>
+        </is>
+      </c>
+      <c r="C35" s="26" t="inlineStr">
+        <is>
+          <t>9.c</t>
+        </is>
+      </c>
+      <c r="D35" s="26" t="inlineStr">
+        <is>
+          <t>Den Zugang zur Informations- und Kommunikationstechnologie erheblich erweitern sowie anstreben, in den am wenigsten entwickelten Ländern bis 2020 einen allgemeinen und erschwinglichen Zugang zum Internet bereitzustellen</t>
+        </is>
+      </c>
+      <c r="E35" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="B36" s="26" t="inlineStr">
+        <is>
+          <t>Weniger Ungleichheiten</t>
+        </is>
+      </c>
+      <c r="C36" s="26" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="D36" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 alle Menschen unabhängig von Alter, Geschlecht, Behinderung, „Rasse“, Ethnizität, Herkunft, Religion oder wirtschaftlichem oder sonstigem Status zu Selbstbestimmung befähigen und ihre soziale, wirtschaftliche und politische Inklusion fördern</t>
+        </is>
+      </c>
+      <c r="E36" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="B37" s="26" t="inlineStr">
+        <is>
+          <t>Weniger Ungleichheiten</t>
+        </is>
+      </c>
+      <c r="C37" s="26" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="D37" s="26" t="inlineStr">
+        <is>
+          <t>Chancengleichheit gewährleisten und Ungleichheit der Ergebnisse reduzieren, namentlich durch die Abschaffung diskriminierender Gesetze, Politiken und Praktiken und die Förderung geeigneter gesetzgeberischer, politischer und sonstiger Maßnahmen in dieser Hinsicht</t>
+        </is>
+      </c>
+      <c r="E37" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="B38" s="26" t="inlineStr">
+        <is>
+          <t>Weniger Ungleichheiten</t>
+        </is>
+      </c>
+      <c r="C38" s="26" t="inlineStr">
+        <is>
+          <t>10.7</t>
+        </is>
+      </c>
+      <c r="D38" s="26" t="inlineStr">
+        <is>
+          <t>Eine geordnete, sichere, reguläre und verantwortungsvolle Migration und Mobilität von Menschen ermöglichen, unter anderem durch die Anwendung einer planvollen und gut gesteuerten Migrationspolitik</t>
+        </is>
+      </c>
+      <c r="E38" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="26" t="n">
+        <v>11</v>
+      </c>
+      <c r="B39" s="26" t="inlineStr">
+        <is>
+          <t>Nachhaltige Städte und Gemeinden</t>
+        </is>
+      </c>
+      <c r="C39" s="26" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="D39" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 den Zugang zu sicheren, bezahlbaren, zugänglichen und nachhaltigen Verkehrssystemen für alle ermöglichen und die Sicherheit im Straßenverkehr verbessern, insbesondere durch den Ausbau des öffentlichen Verkehrs, mit besonderem Augenmerk auf den Bedürfnissen von Menschen in prekären Situationen, Frauen, Kindern, Menschen mit Behinderungen und älteren Menschen</t>
+        </is>
+      </c>
+      <c r="E39" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="26" t="n">
+        <v>11</v>
+      </c>
+      <c r="B40" s="26" t="inlineStr">
+        <is>
+          <t>Nachhaltige Städte und Gemeinden</t>
+        </is>
+      </c>
+      <c r="C40" s="26" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="D40" s="26" t="inlineStr">
+        <is>
+          <t>Die Anstrengungen zum Schutz und zur Wahrung des Weltkultur- und -naturerbes verstärken</t>
+        </is>
+      </c>
+      <c r="E40" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="26" t="n">
+        <v>11</v>
+      </c>
+      <c r="B41" s="26" t="inlineStr">
+        <is>
+          <t>Nachhaltige Städte und Gemeinden</t>
+        </is>
+      </c>
+      <c r="C41" s="26" t="inlineStr">
+        <is>
+          <t>11.6</t>
+        </is>
+      </c>
+      <c r="D41" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 die von den Städten ausgehende Umweltbelastung pro Kopf senken, unter anderem mit besonderer Aufmerksamkeit auf der Luftqualität und der kommunalen und sonstigen Abfallbehandlung</t>
+        </is>
+      </c>
+      <c r="E41" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="26" t="n">
+        <v>11</v>
+      </c>
+      <c r="B42" s="26" t="inlineStr">
+        <is>
+          <t>Nachhaltige Städte und Gemeinden</t>
+        </is>
+      </c>
+      <c r="C42" s="26" t="inlineStr">
+        <is>
+          <t>11.7</t>
+        </is>
+      </c>
+      <c r="D42" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 den allgemeinen Zugang zu sicheren, inklusiven und zugänglichen Grünflächen und öffentlichen Räumen gewährleisten, insbesondere für Frauen und Kinder, ältere Menschen und Menschen mit Behinderungen</t>
+        </is>
+      </c>
+      <c r="E42" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="26" t="n">
+        <v>12</v>
+      </c>
+      <c r="B43" s="26" t="inlineStr">
+        <is>
+          <t>Nachhaltige/r Konsum und Produktion</t>
+        </is>
+      </c>
+      <c r="C43" s="26" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="D43" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 die nachhaltige Bewirtschaftung und effiziente Nutzung der natürlichen Ressourcen erreichen</t>
+        </is>
+      </c>
+      <c r="E43" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="26" t="n">
+        <v>12</v>
+      </c>
+      <c r="B44" s="26" t="inlineStr">
+        <is>
+          <t>Nachhaltige/r Konsum und Produktion</t>
+        </is>
+      </c>
+      <c r="C44" s="26" t="inlineStr">
+        <is>
+          <t>12.3</t>
+        </is>
+      </c>
+      <c r="D44" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 die weltweiten Lebensmittelabfälle pro Kopf auf Einzelhandels- und Verbraucherebene halbieren und die entlang der Produktions- und Lieferkette entstehenden Lebensmittelverluste einschließlich Nachernteverlusten verringern</t>
+        </is>
+      </c>
+      <c r="E44" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="26" t="n">
+        <v>12</v>
+      </c>
+      <c r="B45" s="26" t="inlineStr">
+        <is>
+          <t>Nachhaltige/r Konsum und Produktion</t>
+        </is>
+      </c>
+      <c r="C45" s="26" t="inlineStr">
+        <is>
+          <t>12.4</t>
+        </is>
+      </c>
+      <c r="D45" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2020 einen umweltverträglichen Umgang mit Chemikalien und allen Abfällen während ihres gesamten Lebenszyklus in Übereinstimmung mit den vereinbarten internationalen Rahmenregelungen erreichen und ihre Freisetzung in Luft, Wasser und Boden erheblich verringern, um ihre nachteiligen Auswirkungen auf die menschliche Gesundheit und die Umwelt auf ein Mindestmaß zu beschränken</t>
+        </is>
+      </c>
+      <c r="E45" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="26" t="n">
+        <v>12</v>
+      </c>
+      <c r="B46" s="26" t="inlineStr">
+        <is>
+          <t>Nachhaltige/r Konsum und Produktion</t>
+        </is>
+      </c>
+      <c r="C46" s="26" t="inlineStr">
+        <is>
+          <t>12.5</t>
+        </is>
+      </c>
+      <c r="D46" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 das Abfallaufkommen durch Vermeidung, Verminderung, Recycling und Wiederverwendung deutlich verringern</t>
+        </is>
+      </c>
+      <c r="E46" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="26" t="n">
+        <v>12</v>
+      </c>
+      <c r="B47" s="26" t="inlineStr">
+        <is>
+          <t>Nachhaltige/r Konsum und Produktion</t>
+        </is>
+      </c>
+      <c r="C47" s="26" t="inlineStr">
+        <is>
+          <t>12.8</t>
+        </is>
+      </c>
+      <c r="D47" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2030 sicherstellen, dass die Menschen überall über einschlägige Informationen und das Bewusstsein für nachhaltige Entwicklung und eine Lebensweise in Harmonie mit der Natur verfügen</t>
+        </is>
+      </c>
+      <c r="E47" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="26" t="n">
+        <v>13</v>
+      </c>
+      <c r="B48" s="26" t="inlineStr">
+        <is>
+          <t>Maßnahmen zum Klimaschutz</t>
+        </is>
+      </c>
+      <c r="C48" s="26" t="inlineStr">
+        <is>
+          <t>13.1</t>
+        </is>
+      </c>
+      <c r="D48" s="26" t="inlineStr">
+        <is>
+          <t>Die Widerstandskraft und die Anpassungsfähigkeit gegenüber klimabedingten Gefahren und Naturkatastrophen in allen Ländern stärken</t>
+        </is>
+      </c>
+      <c r="E48" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="26" t="n">
+        <v>13</v>
+      </c>
+      <c r="B49" s="26" t="inlineStr">
+        <is>
+          <t>Maßnahmen zum Klimaschutz</t>
+        </is>
+      </c>
+      <c r="C49" s="26" t="inlineStr">
+        <is>
+          <t>13.2</t>
+        </is>
+      </c>
+      <c r="D49" s="26" t="inlineStr">
+        <is>
+          <t>Klimaschutzmaßnahmen in die nationalen Politiken, Strategien und Planungen einbeziehen</t>
+        </is>
+      </c>
+      <c r="E49" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="26" t="n">
+        <v>13</v>
+      </c>
+      <c r="B50" s="26" t="inlineStr">
+        <is>
+          <t>Maßnahmen zum Klimaschutz</t>
+        </is>
+      </c>
+      <c r="C50" s="26" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="D50" s="26" t="inlineStr">
+        <is>
+          <t>Die Aufklärung und Sensibilisierung sowie die personellen und institutionellen Kapazitäten im Bereich der Abschwächung des Klimawandels, der Klimaanpassung, der Reduzierung der Klimaauswirkungen sowie der Frühwarnung verbessern</t>
+        </is>
+      </c>
+      <c r="E50" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="26" t="n">
+        <v>14</v>
+      </c>
+      <c r="B51" s="26" t="inlineStr">
+        <is>
+          <t>Leben unter Wasser</t>
+        </is>
+      </c>
+      <c r="C51" s="26" t="inlineStr">
+        <is>
+          <t>14.1</t>
+        </is>
+      </c>
+      <c r="D51" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2025 alle Arten der Meeresverschmutzung, insbesondere durch vom Lande ausgehende Tätigkeiten und namentlich Meeresmüll und Nährstoffbelastung, verhüten und erheblich verringern</t>
+        </is>
+      </c>
+      <c r="E51" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="26" t="n">
+        <v>14</v>
+      </c>
+      <c r="B52" s="26" t="inlineStr">
+        <is>
+          <t>Leben unter Wasser</t>
+        </is>
+      </c>
+      <c r="C52" s="26" t="inlineStr">
+        <is>
+          <t>14.2</t>
+        </is>
+      </c>
+      <c r="D52" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2020 die Meeres- und Küstenökosysteme nachhaltig bewirtschaften und schützen, um unter anderem durch Stärkung ihrer Resilienz erhebliche nachteilige Auswirkungen zu vermeiden, und Maßnahmen zu ihrer Wiederherstellung ergreifen, damit die Meere wieder gesund und produktiv werden</t>
+        </is>
+      </c>
+      <c r="E52" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="26" t="n">
+        <v>14</v>
+      </c>
+      <c r="B53" s="26" t="inlineStr">
+        <is>
+          <t>Leben unter Wasser</t>
+        </is>
+      </c>
+      <c r="C53" s="26" t="inlineStr">
+        <is>
+          <t>14.4</t>
+        </is>
+      </c>
+      <c r="D53" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2020 die Fangtätigkeit wirksam regeln und die Überfischung, die illegale, ungemeldete und unregulierte Fischerei und zerstörerische Fangpraktiken beenden und wissenschaftlich fundierte Bewirtschaftungspläne umsetzen, um die Fischbestände in kürzestmöglicher Zeit mindestens auf einen Stand zurückzuführen, der den höchstmöglichen Dauerertrag unter Berücksichtigung ihrer biologischen Merkmale sichert</t>
+        </is>
+      </c>
+      <c r="E53" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="26" t="n">
+        <v>15</v>
+      </c>
+      <c r="B54" s="26" t="inlineStr">
+        <is>
+          <t>Leben an Land</t>
+        </is>
+      </c>
+      <c r="C54" s="26" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="D54" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2020 im Einklang mit den Verpflichtungen aus internationalen Übereinkünften die Erhaltung, Wiederherstellung und nachhaltige Nutzung der Land- und Binnensüßwasser-Ökosysteme und ihrer Dienstleistungen, insbesondere der Wälder, der Feuchtgebiete, der Berge und der Trockengebiete, gewährleisten</t>
+        </is>
+      </c>
+      <c r="E54" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="26" t="n">
+        <v>15</v>
+      </c>
+      <c r="B55" s="26" t="inlineStr">
+        <is>
+          <t>Leben an Land</t>
+        </is>
+      </c>
+      <c r="C55" s="26" t="inlineStr">
+        <is>
+          <t>15.2</t>
+        </is>
+      </c>
+      <c r="D55" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2020 die nachhaltige Bewirtschaftung aller Waldarten fördern, die Entwaldung beenden, geschädigte Wälder wiederherstellen und die Aufforstung und Wiederaufforstung weltweit beträchtlich erhöhen</t>
+        </is>
+      </c>
+      <c r="E55" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="26" t="n">
+        <v>15</v>
+      </c>
+      <c r="B56" s="26" t="inlineStr">
+        <is>
+          <t>Leben an Land</t>
+        </is>
+      </c>
+      <c r="C56" s="26" t="inlineStr">
+        <is>
+          <t>15.5</t>
+        </is>
+      </c>
+      <c r="D56" s="26" t="inlineStr">
+        <is>
+          <t>Umgehende und bedeutende Maßnahmen ergreifen, um die Verschlechterung der natürlichen Lebensräume zu verringern, dem Verlust der biologischen Vielfalt ein Ende zu setzen und bis 2020 die bedrohten Arten zu schützen und ihr Aussterben zu verhindern</t>
+        </is>
+      </c>
+      <c r="E56" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="26" t="n">
+        <v>15</v>
+      </c>
+      <c r="B57" s="26" t="inlineStr">
+        <is>
+          <t>Leben an Land</t>
+        </is>
+      </c>
+      <c r="C57" s="26" t="inlineStr">
+        <is>
+          <t>15.8</t>
+        </is>
+      </c>
+      <c r="D57" s="26" t="inlineStr">
+        <is>
+          <t>Bis 2020 Maßnahmen einführen, um das Einbringen invasiver gebietsfremder Arten zu verhindern, ihre Auswirkungen auf die Land- und Wasserökosysteme deutlich zu reduzieren und die prioritären Arten zu kontrollieren oder zu beseitigen</t>
+        </is>
+      </c>
+      <c r="E57" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="26" t="n">
+        <v>16</v>
+      </c>
+      <c r="B58" s="26" t="inlineStr">
+        <is>
+          <t>Frieden, Gerechtigkeit und starke Institutionen</t>
+        </is>
+      </c>
+      <c r="C58" s="26" t="inlineStr">
+        <is>
+          <t>16.1</t>
+        </is>
+      </c>
+      <c r="D58" s="26" t="inlineStr">
+        <is>
+          <t>Alle Formen der Gewalt und die gewaltbedingte Sterblichkeit überall deutlich verringern</t>
+        </is>
+      </c>
+      <c r="E58" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="26" t="n">
+        <v>16</v>
+      </c>
+      <c r="B59" s="26" t="inlineStr">
+        <is>
+          <t>Frieden, Gerechtigkeit und starke Institutionen</t>
+        </is>
+      </c>
+      <c r="C59" s="26" t="inlineStr">
+        <is>
+          <t>16.3</t>
+        </is>
+      </c>
+      <c r="D59" s="26" t="inlineStr">
+        <is>
+          <t>Die Rechtsstaatlichkeit auf nationaler und internationaler Ebene fördern und den gleichberechtigten Zugang aller zur Justiz gewährleisten</t>
+        </is>
+      </c>
+      <c r="E59" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="26" t="n">
+        <v>16</v>
+      </c>
+      <c r="B60" s="26" t="inlineStr">
+        <is>
+          <t>Frieden, Gerechtigkeit und starke Institutionen</t>
+        </is>
+      </c>
+      <c r="C60" s="26" t="inlineStr">
+        <is>
+          <t>16.7</t>
+        </is>
+      </c>
+      <c r="D60" s="26" t="inlineStr">
+        <is>
+          <t>Dafür sorgen, dass die Entscheidungsfindung auf allen Ebenen bedarfsorientiert, inklusiv, partizipatorisch und repräsentativ ist</t>
+        </is>
+      </c>
+      <c r="E60" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="26" t="n">
+        <v>16</v>
+      </c>
+      <c r="B61" s="26" t="inlineStr">
+        <is>
+          <t>Frieden, Gerechtigkeit und starke Institutionen</t>
+        </is>
+      </c>
+      <c r="C61" s="26" t="inlineStr">
+        <is>
+          <t>16.10</t>
+        </is>
+      </c>
+      <c r="D61" s="26" t="inlineStr">
+        <is>
+          <t>Den öffentlichen Zugang zu Informationen gewährleisten und die Grundfreiheiten schützen, im Einklang mit den nationalen Rechtsvorschriften und völkerrechtlichen Übereinkünften</t>
+        </is>
+      </c>
+      <c r="E61" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="26" t="n">
+        <v>17</v>
+      </c>
+      <c r="B62" s="26" t="inlineStr">
+        <is>
+          <t>Partnerschaften zur Erreichung der Ziele</t>
+        </is>
+      </c>
+      <c r="C62" s="26" t="inlineStr">
+        <is>
+          <t>17.6</t>
+        </is>
+      </c>
+      <c r="D62" s="26" t="inlineStr">
+        <is>
+          <t>Die regionale und internationale Nord-Süd- und Süd-Süd-Zusammenarbeit und Dreieckskooperation im Bereich Wissenschaft, Technologie und Innovation und den Zugang dazu verbessern und den Austausch von Wissen zu einvernehmlich festgelegten Bedingungen verstärken, unter anderem durch eine bessere Abstimmung zwischen den vorhandenen Mechanismen, insbesondere auf Ebene der Vereinten Nationen, und durch einen globalen Mechanismus zur Technologieförderung</t>
+        </is>
+      </c>
+      <c r="E62" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="26" t="n">
+        <v>17</v>
+      </c>
+      <c r="B63" s="26" t="inlineStr">
+        <is>
+          <t>Partnerschaften zur Erreichung der Ziele</t>
+        </is>
+      </c>
+      <c r="C63" s="26" t="inlineStr">
+        <is>
+          <t>17.16</t>
+        </is>
+      </c>
+      <c r="D63" s="26" t="inlineStr">
+        <is>
+          <t>Die Globale Partnerschaft für nachhaltige Entwicklung ausbauen, ergänzt durch Multi-Akteur-Partnerschaften zur Mobilisierung und zum Austausch von Wissen, Fachkenntnissen, Technologie und finanziellen Ressourcen, um die Erreichung der Ziele für nachhaltige Entwicklung in allen Ländern und insbesondere in den Entwicklungsländern zu unterstützen</t>
+        </is>
+      </c>
+      <c r="E63" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="26" t="n">
+        <v>17</v>
+      </c>
+      <c r="B64" s="26" t="inlineStr">
+        <is>
+          <t>Partnerschaften zur Erreichung der Ziele</t>
+        </is>
+      </c>
+      <c r="C64" s="26" t="inlineStr">
+        <is>
+          <t>17.17</t>
+        </is>
+      </c>
+      <c r="D64" s="26" t="inlineStr">
+        <is>
+          <t>Die Bildung wirksamer öffentlicher, öffentlich-privater und zivilgesellschaftlicher Partnerschaften aufbauend auf den Erfahrungen und Mittelbeschaffungsstrategien bestehender Partnerschaften unterstützen und fördern</t>
+        </is>
+      </c>
+      <c r="E64" s="26" t="inlineStr">
+        <is>
+          <t>Agenda 2030, deutsche Fassung; Statistisches Bundesamt, sdg-indikatoren.de (abgerufen 27.10.2026)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B15"/>
+  <autoFilter ref="A1:E64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>